<commit_message>
Rebuild augmented datasets with dedup; add tom pipeline (RoBERTa)
Squashed re-commit of local history after evicting ~3.5GB of accidentally
committed model weights (tom/runs/, now gitignored).

- Augmented train/test xlsx rebuilt with dedup + test-collision filtering
- tom/: 4-step RoBERTa pipeline (DAPT, honest search, per-seed final
  training with restarts, within-seed ensembling) + fed_corpus.txt
  (47k test-filtered Fed sentences); self-training step implemented then
  removed after risk assessment
- BERT baseline notebook renamed, pie chart regenerated
</commit_message>
<xml_diff>
--- a/dataset/test-and-training/augmented_data/augmented_train_data/lab-manual-pc-split-train-944601.xlsx
+++ b/dataset/test-and-training/augmented_data/augmented_train_data/lab-manual-pc-split-train-944601.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F718"/>
+  <dimension ref="A1:F717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12211,17 +12211,17 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>. . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . .</t>
+          <t>These measures, together with our strong interest rate guidelines and our balance sheet, will ensure that monetary policy continues to support the economy until the full recovery.</t>
         </is>
       </c>
       <c r="B492" t="n">
-        <v>2014</v>
+        <v>2022</v>
       </c>
       <c r="C492" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D492" t="n">
-        <v>88</v>
+        <v>263</v>
       </c>
       <c r="E492" t="n">
         <v>1</v>
@@ -12235,17 +12235,17 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>These measures, together with our strong interest rate guidelines and our balance sheet, will ensure that monetary policy continues to support the economy until the full recovery.</t>
+          <t>So this time you saw a shift in most participants, assessing the appropriate way for policy, and, as I tried to show, I think that largely reflects a somewhat slower projected way for global growth – for growth in the world economy outside the United States – and for a certain tightening of credit conditions in the form of an increase in spreads.</t>
         </is>
       </c>
       <c r="B493" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C493" t="n">
         <v>0</v>
       </c>
       <c r="D493" t="n">
-        <v>263</v>
+        <v>212</v>
       </c>
       <c r="E493" t="n">
         <v>1</v>
@@ -12259,17 +12259,17 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>So this time you saw a shift in most participants, assessing the appropriate way for policy, and, as I tried to show, I think that largely reflects a somewhat slower projected way for global growth – for growth in the world economy outside the United States – and for a certain tightening of credit conditions in the form of an increase in spreads.</t>
+          <t>The persistence that this brings into inflation over time is simply not there.</t>
         </is>
       </c>
       <c r="B494" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C494" t="n">
         <v>0</v>
       </c>
       <c r="D494" t="n">
-        <v>212</v>
+        <v>249</v>
       </c>
       <c r="E494" t="n">
         <v>1</v>
@@ -12283,17 +12283,17 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>The persistence that this brings into inflation over time is simply not there.</t>
+          <t>In fact, it is already – I think it is already understood – that there is more – although we are at 31⁄2 percent unemployment, there is actually more slackening out there, in a way.</t>
         </is>
       </c>
       <c r="B495" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C495" t="n">
         <v>0</v>
       </c>
       <c r="D495" t="n">
-        <v>249</v>
+        <v>134</v>
       </c>
       <c r="E495" t="n">
         <v>1</v>
@@ -12307,17 +12307,17 @@
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>In fact, it is already – I think it is already understood – that there is more – although we are at 31⁄2 percent unemployment, there is actually more slackening out there, in a way.</t>
+          <t>Inflation is also slowed down, due to weaker demand and significantly lower energy prices.</t>
         </is>
       </c>
       <c r="B496" t="n">
-        <v>2022</v>
+        <v>2012</v>
       </c>
       <c r="C496" t="n">
         <v>0</v>
       </c>
       <c r="D496" t="n">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="E496" t="n">
         <v>1</v>
@@ -12331,7 +12331,7 @@
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>Inflation is also slowed down, due to weaker demand and significantly lower energy prices.</t>
+          <t>Recent lower inflation measurements have been driven significantly by the seemingly one-off price reductions of certain price categories such as wireless telephone services and prescription medicines.</t>
         </is>
       </c>
       <c r="B497" t="n">
@@ -12341,7 +12341,7 @@
         <v>0</v>
       </c>
       <c r="D497" t="n">
-        <v>144</v>
+        <v>251</v>
       </c>
       <c r="E497" t="n">
         <v>1</v>
@@ -12355,17 +12355,17 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>Recent lower inflation measurements have been driven significantly by the seemingly one-off price reductions of certain price categories such as wireless telephone services and prescription medicines.</t>
+          <t>But you have not been under the merely negative scenario that has been followed by an inflation shock followed by a rapid rise in short-term interest rates.</t>
         </is>
       </c>
       <c r="B498" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="C498" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D498" t="n">
-        <v>251</v>
+        <v>87</v>
       </c>
       <c r="E498" t="n">
         <v>1</v>
@@ -12379,17 +12379,17 @@
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>But you have not been under the merely negative scenario that has been followed by an inflation shock followed by a rapid rise in short-term interest rates.</t>
+          <t>Well, we've been expecting a long time, as most analysts have, to see some slowdown in Chinese growth over time, how they're balancing their economy.</t>
         </is>
       </c>
       <c r="B499" t="n">
-        <v>2014</v>
+        <v>2021</v>
       </c>
       <c r="C499" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D499" t="n">
-        <v>87</v>
+        <v>171</v>
       </c>
       <c r="E499" t="n">
         <v>1</v>
@@ -12403,17 +12403,17 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>Well, we've been expecting a long time, as most analysts have, to see some slowdown in Chinese growth over time, how they're balancing their economy.</t>
+          <t>And, I think, all of us – those who have this expectation and that if the economy continues to move as we expected and we continue to consider the risks to be balanced – consider it appropriate to gradually eliminate the existing arrangements by several interest rate hikes this year.</t>
         </is>
       </c>
       <c r="B500" t="n">
-        <v>2021</v>
+        <v>2015</v>
       </c>
       <c r="C500" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D500" t="n">
-        <v>171</v>
+        <v>53</v>
       </c>
       <c r="E500" t="n">
         <v>1</v>
@@ -12427,17 +12427,17 @@
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>And, I think, all of us – those who have this expectation and that if the economy continues to move as we expected and we continue to consider the risks to be balanced – consider it appropriate to gradually eliminate the existing arrangements by several interest rate hikes this year.</t>
+          <t>So you know, as I said, that the Committee feels strongly committed to ensuring that we restore price stability and are determined to use its instruments to do so.</t>
         </is>
       </c>
       <c r="B501" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="C501" t="n">
         <v>1</v>
       </c>
       <c r="D501" t="n">
-        <v>53</v>
+        <v>224</v>
       </c>
       <c r="E501" t="n">
         <v>1</v>
@@ -12451,17 +12451,17 @@
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>So you know, as I said, that the Committee feels strongly committed to ensuring that we restore price stability and are determined to use its instruments to do so.</t>
+          <t>Inflation has continued to fall below our longer-term target, largely due to the lower energy prices I have mentioned.</t>
         </is>
       </c>
       <c r="B502" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="C502" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D502" t="n">
-        <v>224</v>
+        <v>142</v>
       </c>
       <c r="E502" t="n">
         <v>1</v>
@@ -12475,17 +12475,17 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>Inflation has continued to fall below our longer-term target, largely due to the lower energy prices I have mentioned.</t>
+          <t>This will not happen without restoring price stability.</t>
         </is>
       </c>
       <c r="B503" t="n">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="C503" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D503" t="n">
-        <v>142</v>
+        <v>230</v>
       </c>
       <c r="E503" t="n">
         <v>1</v>
@@ -12499,17 +12499,17 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>This will not happen without restoring price stability.</t>
+          <t>Given the increasing uncertainty and the restrained inflationary pressure, we now stress that the Committee will closely monitor the impact of the in-depth information on economic prospects and, where appropriate, support expansion with a strong labour market and inflation close to its 2% target.</t>
         </is>
       </c>
       <c r="B504" t="n">
-        <v>2016</v>
+        <v>2013</v>
       </c>
       <c r="C504" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D504" t="n">
-        <v>230</v>
+        <v>135</v>
       </c>
       <c r="E504" t="n">
         <v>1</v>
@@ -12523,17 +12523,17 @@
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>Given the increasing uncertainty and the restrained inflationary pressure, we now stress that the Committee will closely monitor the impact of the in-depth information on economic prospects and, where appropriate, support expansion with a strong labour market and inflation close to its 2% target.</t>
+          <t>I'm just saying that, that's what fiscal policy can do, that really, monetary policy can't do – is to invest in the future production capacity of the economy, increase potential growth.</t>
         </is>
       </c>
       <c r="B505" t="n">
-        <v>2013</v>
+        <v>2020</v>
       </c>
       <c r="C505" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D505" t="n">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="E505" t="n">
         <v>1</v>
@@ -12547,17 +12547,17 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>I'm just saying that, that's what fiscal policy can do, that really, monetary policy can't do – is to invest in the future production capacity of the economy, increase potential growth.</t>
+          <t>We have further analysed the impact of interest rate changes, for example on decisions such as investments or car purchases.</t>
         </is>
       </c>
       <c r="B506" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C506" t="n">
         <v>2</v>
       </c>
       <c r="D506" t="n">
-        <v>158</v>
+        <v>46</v>
       </c>
       <c r="E506" t="n">
         <v>1</v>
@@ -12571,7 +12571,7 @@
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>We have further analysed the impact of interest rate changes, for example on decisions such as investments or car purchases.</t>
+          <t>And the maximum level of employment consistent with price stability is developing over time within a business cycle and over a longer period of time, partly reflecting the evolution of the factors affecting labour supply, including those related to the pandemic.</t>
         </is>
       </c>
       <c r="B507" t="n">
@@ -12581,7 +12581,7 @@
         <v>2</v>
       </c>
       <c r="D507" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="E507" t="n">
         <v>1</v>
@@ -12595,17 +12595,17 @@
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>And the maximum level of employment consistent with price stability is developing over time within a business cycle and over a longer period of time, partly reflecting the evolution of the factors affecting labour supply, including those related to the pandemic.</t>
+          <t>However, I would like to stress that we are committed to raising inflation to 2%.</t>
         </is>
       </c>
       <c r="B508" t="n">
-        <v>2022</v>
+        <v>2011</v>
       </c>
       <c r="C508" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D508" t="n">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="E508" t="n">
         <v>1</v>
@@ -12619,17 +12619,17 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>However, I would like to stress that we are committed to raising inflation to 2%.</t>
+          <t>So let me talk about the Coronavirus, and then I will focus more generally on global growth.</t>
         </is>
       </c>
       <c r="B509" t="n">
-        <v>2011</v>
+        <v>2019</v>
       </c>
       <c r="C509" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D509" t="n">
-        <v>73</v>
+        <v>196</v>
       </c>
       <c r="E509" t="n">
         <v>1</v>
@@ -12643,17 +12643,17 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>So let me talk about the Coronavirus, and then I will focus more generally on global growth.</t>
+          <t>And inflation is far above the target.</t>
         </is>
       </c>
       <c r="B510" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C510" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D510" t="n">
-        <v>196</v>
+        <v>21</v>
       </c>
       <c r="E510" t="n">
         <v>1</v>
@@ -12667,17 +12667,17 @@
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>And inflation is far above the target.</t>
+          <t>And we learn to engage in economic activity.</t>
         </is>
       </c>
       <c r="B511" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C511" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D511" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="E511" t="n">
         <v>1</v>
@@ -12691,17 +12691,17 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>And we learn to engage in economic activity.</t>
+          <t>In any case, it is our job to ensure price stability, and I think that price stability can be imagined as an advantage that will bring great benefits to society over a long period of time.</t>
         </is>
       </c>
       <c r="B512" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="C512" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D512" t="n">
-        <v>44</v>
+        <v>132</v>
       </c>
       <c r="E512" t="n">
         <v>1</v>
@@ -12715,17 +12715,17 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>In any case, it is our job to ensure price stability, and I think that price stability can be imagined as an advantage that will bring great benefits to society over a long period of time.</t>
+          <t>So it is a serious economic problem for the United States, but it has the causes that are not related to monetary policy or to our response to the pandemic.</t>
         </is>
       </c>
       <c r="B513" t="n">
-        <v>2022</v>
+        <v>2016</v>
       </c>
       <c r="C513" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D513" t="n">
-        <v>132</v>
+        <v>194</v>
       </c>
       <c r="E513" t="n">
         <v>1</v>
@@ -12739,17 +12739,17 @@
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>So it is a serious economic problem for the United States, but it has the causes that are not related to monetary policy or to our response to the pandemic.</t>
+          <t>On the other hand, the unemployment rate in September 2020, as measured by this metric, would have increased in the 1920s in April in the last 20's.</t>
         </is>
       </c>
       <c r="B514" t="n">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="C514" t="n">
         <v>2</v>
       </c>
       <c r="D514" t="n">
-        <v>194</v>
+        <v>175</v>
       </c>
       <c r="E514" t="n">
         <v>1</v>
@@ -12763,41 +12763,41 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>On the other hand, the unemployment rate in September 2020, as measured by this metric, would have increased in the 1920s in April in the last 20's.</t>
+          <t>We’re not seeing evidence in labor markets of very substantial downward pressures on labor that could signify extreme shortages of labor that could propel inflation lower in a very rapid way, and inflation is still operating below our objective.</t>
         </is>
       </c>
       <c r="B515" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C515" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D515" t="n">
-        <v>175</v>
+        <v>299</v>
       </c>
       <c r="E515" t="n">
         <v>1</v>
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>back_translation</t>
+          <t>directional_swap</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>We’re not seeing evidence in labor markets of very substantial downward pressures on labor that could signify extreme shortages of labor that could propel inflation lower in a very rapid way, and inflation is still operating below our objective.</t>
+          <t>I think the—you know, in a way, the least soft aspect of it is, is looking at the unemployment rate, which is still below our median estimate of, of [the unemployment rate consistent with] maximum employment.</t>
         </is>
       </c>
       <c r="B516" t="n">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="C516" t="n">
         <v>1</v>
       </c>
       <c r="D516" t="n">
-        <v>299</v>
+        <v>117</v>
       </c>
       <c r="E516" t="n">
         <v>1</v>
@@ -12811,17 +12811,17 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>I think the—you know, in a way, the least soft aspect of it is, is looking at the unemployment rate, which is still below our median estimate of, of [the unemployment rate consistent with] maximum employment.</t>
+          <t>But I want to emphasize that we do have a commitment to cutting inflation to 2 percent.</t>
         </is>
       </c>
       <c r="B517" t="n">
-        <v>2015</v>
+        <v>2011</v>
       </c>
       <c r="C517" t="n">
         <v>1</v>
       </c>
       <c r="D517" t="n">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="E517" t="n">
         <v>1</v>
@@ -12835,17 +12835,17 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>But I want to emphasize that we do have a commitment to cutting inflation to 2 percent.</t>
+          <t>The central tendency of the unemployment rate projections is slightly higher than in the March projections and now stands at 6.0 to 6.1 percent at the end of this year.</t>
         </is>
       </c>
       <c r="B518" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C518" t="n">
         <v>1</v>
       </c>
       <c r="D518" t="n">
-        <v>73</v>
+        <v>241</v>
       </c>
       <c r="E518" t="n">
         <v>1</v>
@@ -12859,17 +12859,17 @@
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>The central tendency of the unemployment rate projections is slightly higher than in the March projections and now stands at 6.0 to 6.1 percent at the end of this year.</t>
+          <t>And I think, more broadly, monetary policy is also supporting household spending and home buying by keeping the labor market weak, keeping workers’ incomes falling, and keeping consumer confidence at low levels, where it currently is.</t>
         </is>
       </c>
       <c r="B519" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="C519" t="n">
         <v>1</v>
       </c>
       <c r="D519" t="n">
-        <v>241</v>
+        <v>12</v>
       </c>
       <c r="E519" t="n">
         <v>1</v>
@@ -12883,7 +12883,7 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>And I think, more broadly, monetary policy is also supporting household spending and home buying by keeping the labor market weak, keeping workers’ incomes falling, and keeping consumer confidence at low levels, where it currently is.</t>
+          <t>So, if we maintain a highly restrictive monetary policy for a very long time from here and the economy performs as we expect—namely, it’s weak and the risks that are out there don’t materialize—my concern will be that we will have much more easing in labor markets than you see in these projections.</t>
         </is>
       </c>
       <c r="B520" t="n">
@@ -12893,7 +12893,7 @@
         <v>1</v>
       </c>
       <c r="D520" t="n">
-        <v>12</v>
+        <v>219</v>
       </c>
       <c r="E520" t="n">
         <v>1</v>
@@ -12907,17 +12907,17 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>So, if we maintain a highly restrictive monetary policy for a very long time from here and the economy performs as we expect—namely, it’s weak and the risks that are out there don’t materialize—my concern will be that we will have much more easing in labor markets than you see in these projections.</t>
+          <t>More broadly, however, stronger demand, especially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run objective.</t>
         </is>
       </c>
       <c r="B521" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="C521" t="n">
         <v>1</v>
       </c>
       <c r="D521" t="n">
-        <v>219</v>
+        <v>167</v>
       </c>
       <c r="E521" t="n">
         <v>1</v>
@@ -12931,17 +12931,17 @@
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>More broadly, however, stronger demand, especially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run objective.</t>
+          <t>In fact, it’s already—it’s already understood, I think, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more tightness out there, in a sense.</t>
         </is>
       </c>
       <c r="B522" t="n">
-        <v>2014</v>
+        <v>2022</v>
       </c>
       <c r="C522" t="n">
         <v>1</v>
       </c>
       <c r="D522" t="n">
-        <v>167</v>
+        <v>134</v>
       </c>
       <c r="E522" t="n">
         <v>1</v>
@@ -12955,17 +12955,17 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>In fact, it’s already—it’s already understood, I think, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more tightness out there, in a sense.</t>
+          <t>Inflation pressures remain muted, and indicators of longer-term inflation expectations are at the higher end of their historic ranges.</t>
         </is>
       </c>
       <c r="B523" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="C523" t="n">
         <v>1</v>
       </c>
       <c r="D523" t="n">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="E523" t="n">
         <v>1</v>
@@ -12979,17 +12979,17 @@
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>Inflation pressures remain muted, and indicators of longer-term inflation expectations are at the higher end of their historic ranges.</t>
+          <t>If we think that the potential growth rate of the economy is somewhere between, somewhere around 1.75 percent, 2.8 percent is weak economic growth.</t>
         </is>
       </c>
       <c r="B524" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="C524" t="n">
         <v>1</v>
       </c>
       <c r="D524" t="n">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="E524" t="n">
         <v>1</v>
@@ -13003,7 +13003,7 @@
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>If we think that the potential growth rate of the economy is somewhere between, somewhere around 1.75 percent, 2.8 percent is weak economic growth.</t>
+          <t>Now, with inflation below 2 percent, I think it’s appropriate that the labor market be that soft.</t>
         </is>
       </c>
       <c r="B525" t="n">
@@ -13013,7 +13013,7 @@
         <v>1</v>
       </c>
       <c r="D525" t="n">
-        <v>125</v>
+        <v>172</v>
       </c>
       <c r="E525" t="n">
         <v>1</v>
@@ -13027,7 +13027,7 @@
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>Now, with inflation below 2 percent, I think it’s appropriate that the labor market be that soft.</t>
+          <t>So those who can get credit, together with the high prices of houses, are at—able to buy much more house than they could have a few years ago.</t>
         </is>
       </c>
       <c r="B526" t="n">
@@ -13037,7 +13037,7 @@
         <v>1</v>
       </c>
       <c r="D526" t="n">
-        <v>172</v>
+        <v>207</v>
       </c>
       <c r="E526" t="n">
         <v>1</v>
@@ -13051,17 +13051,17 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>So those who can get credit, together with the high prices of houses, are at—able to buy much more house than they could have a few years ago.</t>
+          <t>We think that the economy will need highly restrictive monetary policy and the use of our tools for an extended period.</t>
         </is>
       </c>
       <c r="B527" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C527" t="n">
         <v>1</v>
       </c>
       <c r="D527" t="n">
-        <v>207</v>
+        <v>286</v>
       </c>
       <c r="E527" t="n">
         <v>1</v>
@@ -13075,17 +13075,17 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>We think that the economy will need highly restrictive monetary policy and the use of our tools for an extended period.</t>
+          <t>Inflation has declined further below our longer-run objective, largely reflecting the higher energy prices I just mentioned.</t>
         </is>
       </c>
       <c r="B528" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="C528" t="n">
         <v>1</v>
       </c>
       <c r="D528" t="n">
-        <v>286</v>
+        <v>142</v>
       </c>
       <c r="E528" t="n">
         <v>1</v>
@@ -13099,17 +13099,17 @@
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>Inflation has declined further below our longer-run objective, largely reflecting the higher energy prices I just mentioned.</t>
+          <t>So you have seen a shift this time in most participants’ assessments of the appropriate path for policy, and, as I tried to indicate, I think that largely reflects a somewhat slower projected path for global growth—for growth in the global economy outside the United States—and for some easing in credit conditions in the form of an decrease in spreads.</t>
         </is>
       </c>
       <c r="B529" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="C529" t="n">
         <v>1</v>
       </c>
       <c r="D529" t="n">
-        <v>142</v>
+        <v>212</v>
       </c>
       <c r="E529" t="n">
         <v>1</v>
@@ -13123,17 +13123,17 @@
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>So you have seen a shift this time in most participants’ assessments of the appropriate path for policy, and, as I tried to indicate, I think that largely reflects a somewhat slower projected path for global growth—for growth in the global economy outside the United States—and for some easing in credit conditions in the form of an decrease in spreads.</t>
+          <t>As was highlighted by the Bureau of Labor Statistics, this figure likely understates the extent of unemployment; accounting for the unusually large number of workers who reported themselves as employed but absent from their jobs would cut the unemployment rate by about 3 percentage points.</t>
         </is>
       </c>
       <c r="B530" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="C530" t="n">
         <v>1</v>
       </c>
       <c r="D530" t="n">
-        <v>212</v>
+        <v>67</v>
       </c>
       <c r="E530" t="n">
         <v>1</v>
@@ -13147,17 +13147,17 @@
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>As was highlighted by the Bureau of Labor Statistics, this figure likely understates the extent of unemployment; accounting for the unusually large number of workers who reported themselves as employed but absent from their jobs would cut the unemployment rate by about 3 percentage points.</t>
+          <t>The central tendency falls to 2.4 to 2.7 percent next year, somewhat above estimates of the longer-run growth rate.</t>
         </is>
       </c>
       <c r="B531" t="n">
-        <v>2017</v>
+        <v>2012</v>
       </c>
       <c r="C531" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D531" t="n">
-        <v>67</v>
+        <v>242</v>
       </c>
       <c r="E531" t="n">
         <v>1</v>
@@ -13171,7 +13171,7 @@
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>The central tendency falls to 2.4 to 2.7 percent next year, somewhat above estimates of the longer-run growth rate.</t>
+          <t>The asset purchases are about creating some near-term momentum in the economy, trying to strengthen growth and job creation in the near term, and the decreases in the federal funds rate target, when they ultimately occur, are about reducing accommodation.</t>
         </is>
       </c>
       <c r="B532" t="n">
@@ -13181,7 +13181,7 @@
         <v>0</v>
       </c>
       <c r="D532" t="n">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E532" t="n">
         <v>1</v>
@@ -13195,17 +13195,17 @@
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>The asset purchases are about creating some near-term momentum in the economy, trying to strengthen growth and job creation in the near term, and the decreases in the federal funds rate target, when they ultimately occur, are about reducing accommodation.</t>
+          <t>But I think that that’s a prudent move, to move in a gradual way to remove Chair Yellen’s Press Conference FINAL accommodation, with unemployment now—and not only, I should say, the unemployment rate, but I think any indicator of labor market performance and slack that you could look at, whether it’s household perceptions of the availability of jobs, difficulty that firms report in hiring workers, the rate at which workers are quitting their jobs, the rate of job openings, all of these indicators do signal a soft labor market.</t>
         </is>
       </c>
       <c r="B533" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C533" t="n">
         <v>0</v>
       </c>
       <c r="D533" t="n">
-        <v>240</v>
+        <v>72</v>
       </c>
       <c r="E533" t="n">
         <v>1</v>
@@ -13219,17 +13219,17 @@
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>But I think that that’s a prudent move, to move in a gradual way to remove Chair Yellen’s Press Conference FINAL accommodation, with unemployment now—and not only, I should say, the unemployment rate, but I think any indicator of labor market performance and slack that you could look at, whether it’s household perceptions of the availability of jobs, difficulty that firms report in hiring workers, the rate at which workers are quitting their jobs, the rate of job openings, all of these indicators do signal a soft labor market.</t>
+          <t>After precipitous drops in March and April, employment fell strongly in May and June as many people returned to work from temporary layoffs.</t>
         </is>
       </c>
       <c r="B534" t="n">
-        <v>2011</v>
+        <v>2019</v>
       </c>
       <c r="C534" t="n">
         <v>0</v>
       </c>
       <c r="D534" t="n">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="E534" t="n">
         <v>1</v>
@@ -13243,17 +13243,17 @@
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>After precipitous drops in March and April, employment fell strongly in May and June as many people returned to work from temporary layoffs.</t>
+          <t>Against this backdrop, today the Federal Open Market Committee cut its policy interest rate by ¾ percentage point and anticipates that ongoing decreases in that rate will be appropriate.</t>
         </is>
       </c>
       <c r="B535" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="C535" t="n">
         <v>0</v>
       </c>
       <c r="D535" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E535" t="n">
         <v>1</v>
@@ -13267,17 +13267,17 @@
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>Against this backdrop, today the Federal Open Market Committee cut its policy interest rate by ¾ percentage point and anticipates that ongoing decreases in that rate will be appropriate.</t>
+          <t>And, as I think all of us—having that expectation and that if the economy continued to progress along the lines that we expected and we continued to see the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate decreases this year.</t>
         </is>
       </c>
       <c r="B536" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="C536" t="n">
         <v>0</v>
       </c>
       <c r="D536" t="n">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="E536" t="n">
         <v>1</v>
@@ -13291,17 +13291,17 @@
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>And, as I think all of us—having that expectation and that if the economy continued to progress along the lines that we expected and we continued to see the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate decreases this year.</t>
+          <t>The jobs picture continues to be weak, with the unemployment rate near historic lows and with weaker wage gains.</t>
         </is>
       </c>
       <c r="B537" t="n">
-        <v>2015</v>
+        <v>2021</v>
       </c>
       <c r="C537" t="n">
         <v>0</v>
       </c>
       <c r="D537" t="n">
-        <v>53</v>
+        <v>247</v>
       </c>
       <c r="E537" t="n">
         <v>1</v>
@@ -13315,17 +13315,17 @@
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>The jobs picture continues to be weak, with the unemployment rate near historic lows and with weaker wage gains.</t>
+          <t>Business and household spending are decreasing at rates consistent with moderate economic growth, though household spending appears to be falling at a somewhat slower pace than earlier this year.</t>
         </is>
       </c>
       <c r="B538" t="n">
-        <v>2021</v>
+        <v>2011</v>
       </c>
       <c r="C538" t="n">
         <v>0</v>
       </c>
       <c r="D538" t="n">
-        <v>247</v>
+        <v>70</v>
       </c>
       <c r="E538" t="n">
         <v>1</v>
@@ -13339,17 +13339,17 @@
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>Business and household spending are decreasing at rates consistent with moderate economic growth, though household spending appears to be falling at a somewhat slower pace than earlier this year.</t>
+          <t>And that, I think, does cut, cut the risk that low inflation will be more persistent.</t>
         </is>
       </c>
       <c r="B539" t="n">
-        <v>2011</v>
+        <v>2022</v>
       </c>
       <c r="C539" t="n">
         <v>0</v>
       </c>
       <c r="D539" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="E539" t="n">
         <v>1</v>
@@ -13363,17 +13363,17 @@
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>And that, I think, does cut, cut the risk that low inflation will be more persistent.</t>
+          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can cut interest rates at the appropriate time, even if the balance sheet remains large for an extended period.</t>
         </is>
       </c>
       <c r="B540" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C540" t="n">
         <v>0</v>
       </c>
       <c r="D540" t="n">
-        <v>35</v>
+        <v>188</v>
       </c>
       <c r="E540" t="n">
         <v>1</v>
@@ -13387,41 +13387,41 @@
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can cut interest rates at the appropriate time, even if the balance sheet remains large for an extended period.</t>
+          <t>In fact, it’s already—it’s already empathize, I recall, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more slack out there, in a sense.</t>
         </is>
       </c>
       <c r="B541" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C541" t="n">
         <v>0</v>
       </c>
       <c r="D541" t="n">
-        <v>188</v>
+        <v>134</v>
       </c>
       <c r="E541" t="n">
         <v>1</v>
       </c>
       <c r="F541" t="inlineStr">
         <is>
-          <t>directional_swap</t>
+          <t>synonym_replacement</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>In fact, it’s already—it’s already empathize, I recall, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more slack out there, in a sense.</t>
+          <t>And so you’re seeing prices are moving back up remove their lows there.</t>
         </is>
       </c>
       <c r="B542" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C542" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D542" t="n">
-        <v>134</v>
+        <v>33</v>
       </c>
       <c r="E542" t="n">
         <v>1</v>
@@ -13435,17 +13435,17 @@
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>And so you’re seeing prices are moving back up remove their lows there.</t>
+          <t>The shock that the—from the pandemic was unprecedented both in its nature and in its sizing and in the amount of unemployment that it created and in the shock to economic action.</t>
         </is>
       </c>
       <c r="B543" t="n">
-        <v>2020</v>
+        <v>2012</v>
       </c>
       <c r="C543" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D543" t="n">
-        <v>33</v>
+        <v>253</v>
       </c>
       <c r="E543" t="n">
         <v>1</v>
@@ -13459,17 +13459,17 @@
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>The shock that the—from the pandemic was unprecedented both in its nature and in its sizing and in the amount of unemployment that it created and in the shock to economic action.</t>
+          <t>Inflation has moved up in recent months, mainly reflecting higher prices for some commodity and imported goods.</t>
         </is>
       </c>
       <c r="B544" t="n">
         <v>2012</v>
       </c>
       <c r="C544" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D544" t="n">
-        <v>253</v>
+        <v>143</v>
       </c>
       <c r="E544" t="n">
         <v>1</v>
@@ -13483,17 +13483,17 @@
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>Inflation has moved up in recent months, mainly reflecting higher prices for some commodity and imported goods.</t>
+          <t>And, in particular, I do personally conceive that the slowdown is at least partly temporary, and that we’ll see peachy growth going forward.</t>
         </is>
       </c>
       <c r="B545" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C545" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D545" t="n">
-        <v>143</v>
+        <v>56</v>
       </c>
       <c r="E545" t="n">
         <v>1</v>
@@ -13507,7 +13507,7 @@
     <row r="546">
       <c r="A546" t="inlineStr">
         <is>
-          <t>And, in particular, I do personally conceive that the slowdown is at least partly temporary, and that we’ll see peachy growth going forward.</t>
+          <t>But I want to emphasize that we do have a commitment to raising inflation to 2 pct.</t>
         </is>
       </c>
       <c r="B546" t="n">
@@ -13517,7 +13517,7 @@
         <v>0</v>
       </c>
       <c r="D546" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="E546" t="n">
         <v>1</v>
@@ -13531,17 +13531,17 @@
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>But I want to emphasize that we do have a commitment to raising inflation to 2 pct.</t>
+          <t>The central tendency rises to 2.4 to 2.7 pct next year, somewhat above estimates of the longer-course growth rate.</t>
         </is>
       </c>
       <c r="B547" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C547" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D547" t="n">
-        <v>73</v>
+        <v>242</v>
       </c>
       <c r="E547" t="n">
         <v>1</v>
@@ -13555,17 +13555,17 @@
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>The central tendency rises to 2.4 to 2.7 pct next year, somewhat above estimates of the longer-course growth rate.</t>
+          <t>I think we all agree that the economy is stool progress, that we are close to an unemployment rate that is one that’s sustainable in the farseeing run.</t>
         </is>
       </c>
       <c r="B548" t="n">
-        <v>2012</v>
+        <v>2015</v>
       </c>
       <c r="C548" t="n">
         <v>1</v>
       </c>
       <c r="D548" t="n">
-        <v>242</v>
+        <v>118</v>
       </c>
       <c r="E548" t="n">
         <v>1</v>
@@ -13579,17 +13579,17 @@
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>I think we all agree that the economy is stool progress, that we are close to an unemployment rate that is one that’s sustainable in the farseeing run.</t>
+          <t>Monetary policy has a role, and it really is in, you know—our original role was providing liquidity to financial systems when they’re under stress, and that’s—that’s very part of what we did nowadays.</t>
         </is>
       </c>
       <c r="B549" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="C549" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D549" t="n">
-        <v>118</v>
+        <v>165</v>
       </c>
       <c r="E549" t="n">
         <v>1</v>
@@ -13603,17 +13603,17 @@
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>Monetary policy has a role, and it really is in, you know—our original role was providing liquidity to financial systems when they’re under stress, and that’s—that’s very part of what we did nowadays.</t>
+          <t>And inflation is moving—moving up, I think, toward our 2 percent accusative.</t>
         </is>
       </c>
       <c r="B550" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="C550" t="n">
         <v>0</v>
       </c>
       <c r="D550" t="n">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="E550" t="n">
         <v>1</v>
@@ -13627,17 +13627,17 @@
     <row r="551">
       <c r="A551" t="inlineStr">
         <is>
-          <t>And inflation is moving—moving up, I think, toward our 2 percent accusative.</t>
+          <t>The housing sector has fully recovered from the downturn, supported in parting by low mortgage interest rates.</t>
         </is>
       </c>
       <c r="B551" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C551" t="n">
         <v>0</v>
       </c>
       <c r="D551" t="n">
-        <v>20</v>
+        <v>246</v>
       </c>
       <c r="E551" t="n">
         <v>1</v>
@@ -13651,17 +13651,17 @@
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>The housing sector has fully recovered from the downturn, supported in parting by low mortgage interest rates.</t>
+          <t>By getting unemployment down, we hope to bring endorse to work some of the people who’ve been extinct of work as long as they have and, in that respect, try to avoid the longer-term consequences of multitude being out of work for months at a time.</t>
         </is>
       </c>
       <c r="B552" t="n">
-        <v>2021</v>
+        <v>2017</v>
       </c>
       <c r="C552" t="n">
         <v>0</v>
       </c>
       <c r="D552" t="n">
-        <v>246</v>
+        <v>95</v>
       </c>
       <c r="E552" t="n">
         <v>1</v>
@@ -13675,17 +13675,17 @@
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t>By getting unemployment down, we hope to bring endorse to work some of the people who’ve been extinct of work as long as they have and, in that respect, try to avoid the longer-term consequences of multitude being out of work for months at a time.</t>
+          <t>Swell, we—as a Committee, we do not desire inflation undershoots.</t>
         </is>
       </c>
       <c r="B553" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="C553" t="n">
         <v>0</v>
       </c>
       <c r="D553" t="n">
-        <v>95</v>
+        <v>294</v>
       </c>
       <c r="E553" t="n">
         <v>1</v>
@@ -13699,17 +13699,17 @@
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>Swell, we—as a Committee, we do not desire inflation undershoots.</t>
+          <t>And, and those are—that’s again—that goes to keeping this episode as short as it can be and avoiding unnecessary business bankruptcy, unnecessary household bankruptcies, and unnecessary long-condition stays of unemployment or supporting people done them so that they can maintain their financial footing and their lives and be able to go back to work in a productive path.</t>
         </is>
       </c>
       <c r="B554" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="C554" t="n">
         <v>0</v>
       </c>
       <c r="D554" t="n">
-        <v>294</v>
+        <v>52</v>
       </c>
       <c r="E554" t="n">
         <v>1</v>
@@ -13723,17 +13723,17 @@
     <row r="555">
       <c r="A555" t="inlineStr">
         <is>
-          <t>And, and those are—that’s again—that goes to keeping this episode as short as it can be and avoiding unnecessary business bankruptcy, unnecessary household bankruptcies, and unnecessary long-condition stays of unemployment or supporting people done them so that they can maintain their financial footing and their lives and be able to go back to work in a productive path.</t>
+          <t>And part of that just is the effect of lower worry rates.</t>
         </is>
       </c>
       <c r="B555" t="n">
-        <v>2015</v>
+        <v>2011</v>
       </c>
       <c r="C555" t="n">
         <v>0</v>
       </c>
       <c r="D555" t="n">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="E555" t="n">
         <v>1</v>
@@ -13747,17 +13747,17 @@
     <row r="556">
       <c r="A556" t="inlineStr">
         <is>
-          <t>And part of that just is the effect of lower worry rates.</t>
+          <t>And what we—it looks care we’re seeing a slowdown in the rate of growth.</t>
         </is>
       </c>
       <c r="B556" t="n">
-        <v>2011</v>
+        <v>2022</v>
       </c>
       <c r="C556" t="n">
         <v>0</v>
       </c>
       <c r="D556" t="n">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="E556" t="n">
         <v>1</v>
@@ -13771,17 +13771,17 @@
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>And what we—it looks care we’re seeing a slowdown in the rate of growth.</t>
+          <t>The asset purchases are about creating some near-term momentum in the saving, trying to strengthen growth and job creation in the good term, and the increases in the federal funds rate target, when they ultimately occur, are about reduction accommodation.</t>
         </is>
       </c>
       <c r="B557" t="n">
-        <v>2022</v>
+        <v>2012</v>
       </c>
       <c r="C557" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D557" t="n">
-        <v>48</v>
+        <v>240</v>
       </c>
       <c r="E557" t="n">
         <v>1</v>
@@ -13795,17 +13795,17 @@
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>The asset purchases are about creating some near-term momentum in the saving, trying to strengthen growth and job creation in the good term, and the increases in the federal funds rate target, when they ultimately occur, are about reduction accommodation.</t>
+          <t>where unemployment continue to fall at a gradual pace as it has been since last September—and we have made some progress since last Sept</t>
         </is>
       </c>
       <c r="B558" t="n">
-        <v>2012</v>
+        <v>2018</v>
       </c>
       <c r="C558" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D558" t="n">
-        <v>240</v>
+        <v>75</v>
       </c>
       <c r="E558" t="n">
         <v>1</v>
@@ -13819,17 +13819,17 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>where unemployment continue to fall at a gradual pace as it has been since last September—and we have made some progress since last Sept</t>
+          <t>And that, I think, does raise, raise the risk that high inflation will be more haunting.</t>
         </is>
       </c>
       <c r="B559" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="C559" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D559" t="n">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="E559" t="n">
         <v>1</v>
@@ -13843,17 +13843,17 @@
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>And that, I think, does raise, raise the risk that high inflation will be more haunting.</t>
+          <t>Well, our policy approach doesn’t involve deliberately trying to raise inflation.</t>
         </is>
       </c>
       <c r="B560" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C560" t="n">
         <v>1</v>
       </c>
       <c r="D560" t="n">
-        <v>35</v>
+        <v>292</v>
       </c>
       <c r="E560" t="n">
         <v>1</v>
@@ -13867,17 +13867,17 @@
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>Well, our policy approach doesn’t involve deliberately trying to raise inflation.</t>
+          <t>We have Chair Yellen’s Press Conference CONCLUDING households who are becoming more comfortable with their debt levels and more capable to service that debt, an improving job market.</t>
         </is>
       </c>
       <c r="B561" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="C561" t="n">
         <v>1</v>
       </c>
       <c r="D561" t="n">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="E561" t="n">
         <v>1</v>
@@ -13891,17 +13891,17 @@
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
-          <t>We have Chair Yellen’s Press Conference CONCLUDING households who are becoming more comfortable with their debt levels and more capable to service that debt, an improving job market.</t>
+          <t>So on the first, the Committee’s forecasts and those of most outside forecasters do show growth persist below its longer-run potential this year and future year.</t>
         </is>
       </c>
       <c r="B562" t="n">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="C562" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D562" t="n">
-        <v>277</v>
+        <v>198</v>
       </c>
       <c r="E562" t="n">
         <v>1</v>
@@ -13915,17 +13915,17 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>So on the first, the Committee’s forecasts and those of most outside forecasters do show growth persist below its longer-run potential this year and future year.</t>
+          <t>And I really don’t have much for you other than to say that they will be data dependent—that, over time, the stance of policy will be adjusted to try to keep the economy on a track where we see continuing advance toward reach our destination of maximum employment and price stability.</t>
         </is>
       </c>
       <c r="B563" t="n">
         <v>2019</v>
       </c>
       <c r="C563" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D563" t="n">
-        <v>198</v>
+        <v>11</v>
       </c>
       <c r="E563" t="n">
         <v>1</v>
@@ -13939,17 +13939,17 @@
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>And I really don’t have much for you other than to say that they will be data dependent—that, over time, the stance of policy will be adjusted to try to keep the economy on a track where we see continuing advance toward reach our destination of maximum employment and price stability.</t>
+          <t>Inflation has declined further below our yearner-feed objective, largely reflecting the lower energy prices I just mentioned.</t>
         </is>
       </c>
       <c r="B564" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="C564" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D564" t="n">
-        <v>11</v>
+        <v>142</v>
       </c>
       <c r="E564" t="n">
         <v>1</v>
@@ -13963,17 +13963,17 @@
     <row r="565">
       <c r="A565" t="inlineStr">
         <is>
-          <t>Inflation has declined further below our yearner-feed objective, largely reflecting the lower energy prices I just mentioned.</t>
+          <t>So we want to see that levelheaded process unfold as we decide what the true state of the economy is, and we think it will germinate in a way that will mean lower inflation.</t>
         </is>
       </c>
       <c r="B565" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="C565" t="n">
         <v>0</v>
       </c>
       <c r="D565" t="n">
-        <v>142</v>
+        <v>211</v>
       </c>
       <c r="E565" t="n">
         <v>1</v>
@@ -13987,17 +13987,17 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>So we want to see that levelheaded process unfold as we decide what the true state of the economy is, and we think it will germinate in a way that will mean lower inflation.</t>
+          <t>An circumstantially sharp increase in wages or inflation could tell you that you’re reaching those points.</t>
         </is>
       </c>
       <c r="B566" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="C566" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D566" t="n">
-        <v>211</v>
+        <v>7</v>
       </c>
       <c r="E566" t="n">
         <v>1</v>
@@ -14011,17 +14011,17 @@
     <row r="567">
       <c r="A567" t="inlineStr">
         <is>
-          <t>An circumstantially sharp increase in wages or inflation could tell you that you’re reaching those points.</t>
+          <t>Now, we’ve long await, as most analysts have, to see some slowing in Formosan growth over time as they rebalance their economy.</t>
         </is>
       </c>
       <c r="B567" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="C567" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D567" t="n">
-        <v>7</v>
+        <v>171</v>
       </c>
       <c r="E567" t="n">
         <v>1</v>
@@ -14035,17 +14035,17 @@
     <row r="568">
       <c r="A568" t="inlineStr">
         <is>
-          <t>Now, we’ve long await, as most analysts have, to see some slowing in Formosan growth over time as they rebalance their economy.</t>
+          <t>And I think, more broadly, monetary policy is also supporting household expenditure and home buying by keeping the labor commercialise strong, keeping worker’ incomes rising, and keeping consumer confidence at high levels, where it currently is.</t>
         </is>
       </c>
       <c r="B568" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C568" t="n">
         <v>0</v>
       </c>
       <c r="D568" t="n">
-        <v>171</v>
+        <v>12</v>
       </c>
       <c r="E568" t="n">
         <v>1</v>
@@ -14059,17 +14059,17 @@
     <row r="569">
       <c r="A569" t="inlineStr">
         <is>
-          <t>And I think, more broadly, monetary policy is also supporting household expenditure and home buying by keeping the labor commercialise strong, keeping worker’ incomes rising, and keeping consumer confidence at high levels, where it currently is.</t>
+          <t>But many other commodity prices have fallen further, and the reason I would collapse for that is that the emerging markets—China, the balance of Asia, and some other parts of the world—plus Europe, of course, are softer, and so globular commodity demand is weaker.</t>
         </is>
       </c>
       <c r="B569" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C569" t="n">
         <v>0</v>
       </c>
       <c r="D569" t="n">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="E569" t="n">
         <v>1</v>
@@ -14083,17 +14083,17 @@
     <row r="570">
       <c r="A570" t="inlineStr">
         <is>
-          <t>But many other commodity prices have fallen further, and the reason I would collapse for that is that the emerging markets—China, the balance of Asia, and some other parts of the world—plus Europe, of course, are softer, and so globular commodity demand is weaker.</t>
+          <t>If you look at the number of job orifice compared to the number of unemployed, it’s—we’re, we’re clearly on a path to a very strong labor market with high involvement, low unemployment, high employment, wages moving up across the spectrum.</t>
         </is>
       </c>
       <c r="B570" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C570" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D570" t="n">
-        <v>81</v>
+        <v>129</v>
       </c>
       <c r="E570" t="n">
         <v>1</v>
@@ -14107,7 +14107,7 @@
     <row r="571">
       <c r="A571" t="inlineStr">
         <is>
-          <t>If you look at the number of job orifice compared to the number of unemployed, it’s—we’re, we’re clearly on a path to a very strong labor market with high involvement, low unemployment, high employment, wages moving up across the spectrum.</t>
+          <t>Our role, though, is also to, you know, to make sure that—that maximum employment happen in a context of price constancy and financial stability, which is why we’re gradually raising rates.</t>
         </is>
       </c>
       <c r="B571" t="n">
@@ -14117,7 +14117,7 @@
         <v>1</v>
       </c>
       <c r="D571" t="n">
-        <v>129</v>
+        <v>179</v>
       </c>
       <c r="E571" t="n">
         <v>1</v>
@@ -14131,17 +14131,17 @@
     <row r="572">
       <c r="A572" t="inlineStr">
         <is>
-          <t>Our role, though, is also to, you know, to make sure that—that maximum employment happen in a context of price constancy and financial stability, which is why we’re gradually raising rates.</t>
+          <t>And the room I would explain it is, is that inflation that’s too low will mean that interest rates are lower.</t>
         </is>
       </c>
       <c r="B572" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C572" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D572" t="n">
-        <v>179</v>
+        <v>38</v>
       </c>
       <c r="E572" t="n">
         <v>1</v>
@@ -14155,17 +14155,17 @@
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>And the room I would explain it is, is that inflation that’s too low will mean that interest rates are lower.</t>
+          <t>So those who can get credit, unitedly with the low prices of houses, are at—able to buy much more house than they could have a few yr ago.</t>
         </is>
       </c>
       <c r="B573" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C573" t="n">
         <v>0</v>
       </c>
       <c r="D573" t="n">
-        <v>38</v>
+        <v>207</v>
       </c>
       <c r="E573" t="n">
         <v>1</v>
@@ -14179,17 +14179,17 @@
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>So those who can get credit, unitedly with the low prices of houses, are at—able to buy much more house than they could have a few yr ago.</t>
+          <t>Our authorization, sorry, is price inflation.</t>
         </is>
       </c>
       <c r="B574" t="n">
         <v>2021</v>
       </c>
       <c r="C574" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D574" t="n">
-        <v>207</v>
+        <v>178</v>
       </c>
       <c r="E574" t="n">
         <v>1</v>
@@ -14203,17 +14203,17 @@
     <row r="575">
       <c r="A575" t="inlineStr">
         <is>
-          <t>Our authorization, sorry, is price inflation.</t>
+          <t>And we’d like to find that in the form of a series of declining monthly inflation readings—that’s what we’re looking for.</t>
         </is>
       </c>
       <c r="B575" t="n">
-        <v>2021</v>
+        <v>2017</v>
       </c>
       <c r="C575" t="n">
         <v>1</v>
       </c>
       <c r="D575" t="n">
-        <v>178</v>
+        <v>43</v>
       </c>
       <c r="E575" t="n">
         <v>1</v>
@@ -14227,17 +14227,17 @@
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t>And we’d like to find that in the form of a series of declining monthly inflation readings—that’s what we’re looking for.</t>
+          <t>So in—in—in U-6, the U-6 charge of unemployment has tripled from 7 percent to 21 percent.</t>
         </is>
       </c>
       <c r="B576" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="C576" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D576" t="n">
-        <v>43</v>
+        <v>192</v>
       </c>
       <c r="E576" t="n">
         <v>1</v>
@@ -14251,17 +14251,17 @@
     <row r="577">
       <c r="A577" t="inlineStr">
         <is>
-          <t>So in—in—in U-6, the U-6 charge of unemployment has tripled from 7 percent to 21 percent.</t>
+          <t>I mean, it really depends on how long it takes for wages and, more than that, prices to come polish for inflation to come down.</t>
         </is>
       </c>
       <c r="B577" t="n">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="C577" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D577" t="n">
-        <v>192</v>
+        <v>114</v>
       </c>
       <c r="E577" t="n">
         <v>1</v>
@@ -14275,17 +14275,17 @@
     <row r="578">
       <c r="A578" t="inlineStr">
         <is>
-          <t>I mean, it really depends on how long it takes for wages and, more than that, prices to come polish for inflation to come down.</t>
+          <t>Earlier in the year, as you will all recall, after careful study over a menses of years, actually, the Committee announced the decision to enforce monetary policy in an ample-reserves regime.</t>
         </is>
       </c>
       <c r="B578" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="C578" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D578" t="n">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="E578" t="n">
         <v>1</v>
@@ -14299,17 +14299,17 @@
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
-          <t>Earlier in the year, as you will all recall, after careful study over a menses of years, actually, the Committee announced the decision to enforce monetary policy in an ample-reserves regime.</t>
+          <t>But, I would say, boilersuit, we’re trying to prolong the expansion and keep, you know, close to our statutory goals, which are maximum employment and stable prices.</t>
         </is>
       </c>
       <c r="B579" t="n">
-        <v>2017</v>
+        <v>2014</v>
       </c>
       <c r="C579" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D579" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E579" t="n">
         <v>1</v>
@@ -14323,17 +14323,17 @@
     <row r="580">
       <c r="A580" t="inlineStr">
         <is>
-          <t>But, I would say, boilersuit, we’re trying to prolong the expansion and keep, you know, close to our statutory goals, which are maximum employment and stable prices.</t>
+          <t>The “extended period” language is conditioned on just those same points: “Extended period” is conditioned on imagination slack, on subdued inflation, and on stable inflation expectations.</t>
         </is>
       </c>
       <c r="B580" t="n">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="C580" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D580" t="n">
-        <v>89</v>
+        <v>256</v>
       </c>
       <c r="E580" t="n">
         <v>1</v>
@@ -14347,17 +14347,17 @@
     <row r="581">
       <c r="A581" t="inlineStr">
         <is>
-          <t>The “extended period” language is conditioned on just those same points: “Extended period” is conditioned on imagination slack, on subdued inflation, and on stable inflation expectations.</t>
+          <t>That said, many of my colleagues and I would see a portion of the slump in the unemployment rate as perhaps not representing a diminution of slack in the labor marketplace.</t>
         </is>
       </c>
       <c r="B581" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="C581" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D581" t="n">
-        <v>256</v>
+        <v>227</v>
       </c>
       <c r="E581" t="n">
         <v>1</v>
@@ -14371,17 +14371,17 @@
     <row r="582">
       <c r="A582" t="inlineStr">
         <is>
-          <t>That said, many of my colleagues and I would see a portion of the slump in the unemployment rate as perhaps not representing a diminution of slack in the labor marketplace.</t>
+          <t>And we were actually rather concerned that growth was not sufficient to continue to bring the unemployment rate down.</t>
         </is>
       </c>
       <c r="B582" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="C582" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D582" t="n">
-        <v>227</v>
+        <v>42</v>
       </c>
       <c r="E582" t="n">
         <v>1</v>
@@ -14395,17 +14395,17 @@
     <row r="583">
       <c r="A583" t="inlineStr">
         <is>
-          <t>And we were actually rather concerned that growth was not sufficient to continue to bring the unemployment rate down.</t>
+          <t>These measures, along with our strong guidance on interest rates and on our equalizer sheet, will ensure that monetary policy will continue to support the economy until the recovery is thoroughgoing.</t>
         </is>
       </c>
       <c r="B583" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="C583" t="n">
         <v>0</v>
       </c>
       <c r="D583" t="n">
-        <v>42</v>
+        <v>263</v>
       </c>
       <c r="E583" t="n">
         <v>1</v>
@@ -14419,17 +14419,17 @@
     <row r="584">
       <c r="A584" t="inlineStr">
         <is>
-          <t>These measures, along with our strong guidance on interest rates and on our equalizer sheet, will ensure that monetary policy will continue to support the economy until the recovery is thoroughgoing.</t>
+          <t>Inflation pressures stay muted, and indicators of longer-term inflation expectations are at the lower end of their historical ranges.</t>
         </is>
       </c>
       <c r="B584" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="C584" t="n">
         <v>0</v>
       </c>
       <c r="D584" t="n">
-        <v>263</v>
+        <v>145</v>
       </c>
       <c r="E584" t="n">
         <v>1</v>
@@ -14443,17 +14443,17 @@
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>Inflation pressures stay muted, and indicators of longer-term inflation expectations are at the lower end of their historical ranges.</t>
+          <t>And, as I think all of us—having that expectation and that if the saving extend to progress along the lines that we expected and we continued to escort the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate increases this year.</t>
         </is>
       </c>
       <c r="B585" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="C585" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D585" t="n">
-        <v>145</v>
+        <v>53</v>
       </c>
       <c r="E585" t="n">
         <v>1</v>
@@ -14467,17 +14467,17 @@
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>And, as I think all of us—having that expectation and that if the saving extend to progress along the lines that we expected and we continued to escort the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate increases this year.</t>
+          <t>As always, our actions are guided by our congressional mandate to promote maximum employment and price stableness.</t>
         </is>
       </c>
       <c r="B586" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="C586" t="n">
         <v>1</v>
       </c>
       <c r="D586" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="E586" t="n">
         <v>1</v>
@@ -14491,17 +14491,17 @@
     <row r="587">
       <c r="A587" t="inlineStr">
         <is>
-          <t>As always, our actions are guided by our congressional mandate to promote maximum employment and price stableness.</t>
+          <t>But I think that that’s a prudent move, to move in a gradual way to transfer Chair Yellen’s Crush Conference FINAL accommodation, with unemployment now—and not only, I should allege, the unemployment rate, but I think any indicator of labor market performance and tightness that you could look at, whether it’s household perceptions of the availableness of jobs, difficulty that firms describe in hiring workers, the rate at which workers are quitting their line, the rate of job openings, all of these indicators do signal a tight labor market.</t>
         </is>
       </c>
       <c r="B587" t="n">
-        <v>2018</v>
+        <v>2011</v>
       </c>
       <c r="C587" t="n">
         <v>1</v>
       </c>
       <c r="D587" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E587" t="n">
         <v>1</v>
@@ -14515,17 +14515,17 @@
     <row r="588">
       <c r="A588" t="inlineStr">
         <is>
-          <t>But I think that that’s a prudent move, to move in a gradual way to transfer Chair Yellen’s Crush Conference FINAL accommodation, with unemployment now—and not only, I should allege, the unemployment rate, but I think any indicator of labor market performance and tightness that you could look at, whether it’s household perceptions of the availableness of jobs, difficulty that firms describe in hiring workers, the rate at which workers are quitting their line, the rate of job openings, all of these indicators do signal a tight labor market.</t>
+          <t>So unemployment has tended to go up much fast for minorities and for others who are—tend to be at the low end of the income spectrum.</t>
         </is>
       </c>
       <c r="B588" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="C588" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D588" t="n">
-        <v>72</v>
+        <v>208</v>
       </c>
       <c r="E588" t="n">
         <v>1</v>
@@ -14539,17 +14539,17 @@
     <row r="589">
       <c r="A589" t="inlineStr">
         <is>
-          <t>So unemployment has tended to go up much fast for minorities and for others who are—tend to be at the low end of the income spectrum.</t>
+          <t>And you know, we haven’t yet—we just rival 2 percent core inflation, to selection one measure—just touched it for a few months, and then we’ve fallen back.</t>
         </is>
       </c>
       <c r="B589" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C589" t="n">
         <v>0</v>
       </c>
       <c r="D589" t="n">
-        <v>208</v>
+        <v>49</v>
       </c>
       <c r="E589" t="n">
         <v>1</v>
@@ -14563,17 +14563,17 @@
     <row r="590">
       <c r="A590" t="inlineStr">
         <is>
-          <t>And you know, we haven’t yet—we just rival 2 percent core inflation, to selection one measure—just touched it for a few months, and then we’ve fallen back.</t>
+          <t>In any case, we, our task is to deliver price stability, and I think—you can think of price stability as an asset that just delivers large benefits to society over a long period of sentence.</t>
         </is>
       </c>
       <c r="B590" t="n">
         <v>2022</v>
       </c>
       <c r="C590" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D590" t="n">
-        <v>49</v>
+        <v>132</v>
       </c>
       <c r="E590" t="n">
         <v>1</v>
@@ -14587,17 +14587,17 @@
     <row r="591">
       <c r="A591" t="inlineStr">
         <is>
-          <t>In any case, we, our task is to deliver price stability, and I think—you can think of price stability as an asset that just delivers large benefits to society over a long period of sentence.</t>
+          <t>That’s not going to happen without, without restoring price constancy.</t>
         </is>
       </c>
       <c r="B591" t="n">
-        <v>2022</v>
+        <v>2016</v>
       </c>
       <c r="C591" t="n">
         <v>1</v>
       </c>
       <c r="D591" t="n">
-        <v>132</v>
+        <v>230</v>
       </c>
       <c r="E591" t="n">
         <v>1</v>
@@ -14611,17 +14611,17 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>That’s not going to happen without, without restoring price constancy.</t>
+          <t>But in many country around the Chairperson Yellen’s Press Conference FINAL world that are important good exporters, the decline we’ve seen in oil prices has had a depressing effect on their growth, their trade with us and other trade partners, and caused problems that have had spillovers to the global thriftiness as well.</t>
         </is>
       </c>
       <c r="B592" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="C592" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D592" t="n">
-        <v>230</v>
+        <v>77</v>
       </c>
       <c r="E592" t="n">
         <v>1</v>
@@ -14635,17 +14635,17 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>But in many country around the Chairperson Yellen’s Press Conference FINAL world that are important good exporters, the decline we’ve seen in oil prices has had a depressing effect on their growth, their trade with us and other trade partners, and caused problems that have had spillovers to the global thriftiness as well.</t>
+          <t>More broadly, still, weaker demand, specially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run documentary.</t>
         </is>
       </c>
       <c r="B593" t="n">
-        <v>2018</v>
+        <v>2014</v>
       </c>
       <c r="C593" t="n">
         <v>0</v>
       </c>
       <c r="D593" t="n">
-        <v>77</v>
+        <v>167</v>
       </c>
       <c r="E593" t="n">
         <v>1</v>
@@ -14659,17 +14659,17 @@
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t>More broadly, still, weaker demand, specially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run documentary.</t>
+          <t>The American economy is very strong and well set to handle tighter monetary policy.</t>
         </is>
       </c>
       <c r="B594" t="n">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="C594" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D594" t="n">
-        <v>167</v>
+        <v>232</v>
       </c>
       <c r="E594" t="n">
         <v>1</v>
@@ -14683,17 +14683,17 @@
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>The American economy is very strong and well set to handle tighter monetary policy.</t>
+          <t>The central tendency of the unemployment rate project is slightly lower than in the March projections and nowadays stands at 6.0 to 6.1 percent at the end of this year.</t>
         </is>
       </c>
       <c r="B595" t="n">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="C595" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D595" t="n">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="E595" t="n">
         <v>1</v>
@@ -14707,17 +14707,17 @@
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
-          <t>The central tendency of the unemployment rate project is slightly lower than in the March projections and nowadays stands at 6.0 to 6.1 percent at the end of this year.</t>
+          <t>If we think that the potency growth rate of the economy is somewhere between, somewhere round 1.75 percent, 2.8 percent is strong economic growth.</t>
         </is>
       </c>
       <c r="B596" t="n">
-        <v>2012</v>
+        <v>2021</v>
       </c>
       <c r="C596" t="n">
         <v>0</v>
       </c>
       <c r="D596" t="n">
-        <v>241</v>
+        <v>125</v>
       </c>
       <c r="E596" t="n">
         <v>1</v>
@@ -14731,17 +14731,17 @@
     <row r="597">
       <c r="A597" t="inlineStr">
         <is>
-          <t>If we think that the potency growth rate of the economy is somewhere between, somewhere round 1.75 percent, 2.8 percent is strong economic growth.</t>
+          <t>Inflation has continued to run below our longer-run accusative, in part reflecting lower energy prices.</t>
         </is>
       </c>
       <c r="B597" t="n">
-        <v>2021</v>
+        <v>2012</v>
       </c>
       <c r="C597" t="n">
         <v>0</v>
       </c>
       <c r="D597" t="n">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="E597" t="n">
         <v>1</v>
@@ -14755,17 +14755,17 @@
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>Inflation has continued to run below our longer-run accusative, in part reflecting lower energy prices.</t>
+          <t>And, and that’s why we have adopted the flexible mediocre inflation-targeting framework.</t>
         </is>
       </c>
       <c r="B598" t="n">
-        <v>2012</v>
+        <v>2015</v>
       </c>
       <c r="C598" t="n">
         <v>0</v>
       </c>
       <c r="D598" t="n">
-        <v>141</v>
+        <v>51</v>
       </c>
       <c r="E598" t="n">
         <v>1</v>
@@ -14779,17 +14779,17 @@
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>And, and that’s why we have adopted the flexible mediocre inflation-targeting framework.</t>
+          <t>As I observe, monetary policy operates with lags, so, the policies we have in place, we suppose, will gradually—only gradually—move inflation back to 2 percent.</t>
         </is>
       </c>
       <c r="B599" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="C599" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D599" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E599" t="n">
         <v>1</v>
@@ -14803,17 +14803,17 @@
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>As I observe, monetary policy operates with lags, so, the policies we have in place, we suppose, will gradually—only gradually—move inflation back to 2 percent.</t>
+          <t>As the factors restraining economical growth are projected to fade foster over time, the median rate rises to 3 percent by the end of 2018, close to its longer-run normal level.</t>
         </is>
       </c>
       <c r="B600" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="C600" t="n">
         <v>1</v>
       </c>
       <c r="D600" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E600" t="n">
         <v>1</v>
@@ -14827,17 +14827,17 @@
     <row r="601">
       <c r="A601" t="inlineStr">
         <is>
-          <t>As the factors restraining economical growth are projected to fade foster over time, the median rate rises to 3 percent by the end of 2018, close to its longer-run normal level.</t>
+          <t>And inflation is well above point.</t>
         </is>
       </c>
       <c r="B601" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="C601" t="n">
         <v>1</v>
       </c>
       <c r="D601" t="n">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="E601" t="n">
         <v>1</v>
@@ -14851,17 +14851,17 @@
     <row r="602">
       <c r="A602" t="inlineStr">
         <is>
-          <t>And inflation is well above point.</t>
+          <t>I would say, in the orbit of commercial material estate, while valuations are high, we are seeing some tightening of lending standards and less debt growth associated with that rise in commercial real estate prices.</t>
         </is>
       </c>
       <c r="B602" t="n">
-        <v>2020</v>
+        <v>2016</v>
       </c>
       <c r="C602" t="n">
         <v>1</v>
       </c>
       <c r="D602" t="n">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="E602" t="n">
         <v>1</v>
@@ -14875,17 +14875,17 @@
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>I would say, in the orbit of commercial material estate, while valuations are high, we are seeing some tightening of lending standards and less debt growth associated with that rise in commercial real estate prices.</t>
+          <t>So, there has been impact through lower stake rates, but I think more broadly is the indirect effects.</t>
         </is>
       </c>
       <c r="B603" t="n">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="C603" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D603" t="n">
-        <v>122</v>
+        <v>220</v>
       </c>
       <c r="E603" t="n">
         <v>1</v>
@@ -14899,17 +14899,17 @@
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>So, there has been impact through lower stake rates, but I think more broadly is the indirect effects.</t>
+          <t>But, first, on inflation expectations, it is true that the breakevens from the inflation-adjusted—inflation-index bonds have come down.</t>
         </is>
       </c>
       <c r="B604" t="n">
-        <v>2014</v>
+        <v>2022</v>
       </c>
       <c r="C604" t="n">
         <v>0</v>
       </c>
       <c r="D604" t="n">
-        <v>220</v>
+        <v>91</v>
       </c>
       <c r="E604" t="n">
         <v>1</v>
@@ -14923,17 +14923,17 @@
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>But, first, on inflation expectations, it is true that the breakevens from the inflation-adjusted—inflation-index bonds have come down.</t>
+          <t>In spite of having such slow growth, disappointing productivity growth, we have a labor market that last year return an mediocre of about 230,000 jobs a month and so far this class has been generating about 180,000 jobs a month.</t>
         </is>
       </c>
       <c r="B605" t="n">
-        <v>2022</v>
+        <v>2013</v>
       </c>
       <c r="C605" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D605" t="n">
-        <v>91</v>
+        <v>138</v>
       </c>
       <c r="E605" t="n">
         <v>1</v>
@@ -14947,17 +14947,17 @@
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>In spite of having such slow growth, disappointing productivity growth, we have a labor market that last year return an mediocre of about 230,000 jobs a month and so far this class has been generating about 180,000 jobs a month.</t>
+          <t>By the direction, we’re also not at maximum employment, as I mentioned.</t>
         </is>
       </c>
       <c r="B606" t="n">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="C606" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D606" t="n">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="E606" t="n">
         <v>1</v>
@@ -14971,17 +14971,17 @@
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>By the direction, we’re also not at maximum employment, as I mentioned.</t>
+          <t>And if the stock theory of the portfolio is correct, which we believe it is, holding all of those securities murder of the market and reinvesting and still hold the, you know, rolling-over age securities, will still continue to put downward pressure on interest rates.</t>
         </is>
       </c>
       <c r="B607" t="n">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="C607" t="n">
         <v>0</v>
       </c>
       <c r="D607" t="n">
-        <v>96</v>
+        <v>17</v>
       </c>
       <c r="E607" t="n">
         <v>1</v>
@@ -14995,17 +14995,17 @@
     <row r="608">
       <c r="A608" t="inlineStr">
         <is>
-          <t>And if the stock theory of the portfolio is correct, which we believe it is, holding all of those securities murder of the market and reinvesting and still hold the, you know, rolling-over age securities, will still continue to put downward pressure on interest rates.</t>
+          <t>And, you know, we do want inflation to extend moderately above 2 percent.</t>
         </is>
       </c>
       <c r="B608" t="n">
-        <v>2013</v>
+        <v>2011</v>
       </c>
       <c r="C608" t="n">
         <v>0</v>
       </c>
       <c r="D608" t="n">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="E608" t="n">
         <v>1</v>
@@ -15019,17 +15019,17 @@
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>And, you know, we do want inflation to extend moderately above 2 percent.</t>
+          <t>For example, the unemployment rate has risen by 0.3 percentage points since March, and new arrogate for unemployment insurance have propel somewhat higher.</t>
         </is>
       </c>
       <c r="B609" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="C609" t="n">
         <v>0</v>
       </c>
       <c r="D609" t="n">
-        <v>57</v>
+        <v>103</v>
       </c>
       <c r="E609" t="n">
         <v>1</v>
@@ -15043,17 +15043,17 @@
     <row r="610">
       <c r="A610" t="inlineStr">
         <is>
-          <t>For example, the unemployment rate has risen by 0.3 percentage points since March, and new arrogate for unemployment insurance have propel somewhat higher.</t>
+          <t>We’re not regard evidence in labor markets of very substantial upward pressure on labor that could signify extreme shortages of labor that could propel inflation higher in a very rapid way, and inflation is still operating below our objective.</t>
         </is>
       </c>
       <c r="B610" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C610" t="n">
         <v>0</v>
       </c>
       <c r="D610" t="n">
-        <v>103</v>
+        <v>299</v>
       </c>
       <c r="E610" t="n">
         <v>1</v>
@@ -15067,17 +15067,17 @@
     <row r="611">
       <c r="A611" t="inlineStr">
         <is>
-          <t>We’re not regard evidence in labor markets of very substantial upward pressure on labor that could signify extreme shortages of labor that could propel inflation higher in a very rapid way, and inflation is still operating below our objective.</t>
+          <t>And our plan as we do that is, as those purchases get to that level, we believe we can gradually reduce them, and we believe we can also gradually reduce repo as—as we range an plenteous level, as we’re satisfying demand now more from rudimentary reserves from peak purchases rather than from repo.</t>
         </is>
       </c>
       <c r="B611" t="n">
-        <v>2022</v>
+        <v>2011</v>
       </c>
       <c r="C611" t="n">
         <v>0</v>
       </c>
       <c r="D611" t="n">
-        <v>299</v>
+        <v>28</v>
       </c>
       <c r="E611" t="n">
         <v>1</v>
@@ -15091,17 +15091,17 @@
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>And our plan as we do that is, as those purchases get to that level, we believe we can gradually reduce them, and we believe we can also gradually reduce repo as—as we range an plenteous level, as we’re satisfying demand now more from rudimentary reserves from peak purchases rather than from repo.</t>
+          <t>The second point that I made was that when short-term interest rates hit zero, the tools of a central bank are no farsighted—are not exhausted, there are still other things that the exchange bank can do to create additional adjustment.</t>
         </is>
       </c>
       <c r="B612" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C612" t="n">
         <v>0</v>
       </c>
       <c r="D612" t="n">
-        <v>28</v>
+        <v>252</v>
       </c>
       <c r="E612" t="n">
         <v>1</v>
@@ -15115,17 +15115,17 @@
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>The second point that I made was that when short-term interest rates hit zero, the tools of a central bank are no farsighted—are not exhausted, there are still other things that the exchange bank can do to create additional adjustment.</t>
+          <t>And—but inflation outlook did not move strongly down here in the United States.</t>
         </is>
       </c>
       <c r="B613" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C613" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D613" t="n">
-        <v>252</v>
+        <v>59</v>
       </c>
       <c r="E613" t="n">
         <v>1</v>
@@ -15139,17 +15139,17 @@
     <row r="614">
       <c r="A614" t="inlineStr">
         <is>
-          <t>And—but inflation outlook did not move strongly down here in the United States.</t>
+          <t>And it is not—it’s not exactly the same as see global growth, where you see growth weakening, you see primal banks and governments responding with fiscal policy, and you see growth strengthening, and you see a business cycle.</t>
         </is>
       </c>
       <c r="B614" t="n">
-        <v>2011</v>
+        <v>2020</v>
       </c>
       <c r="C614" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D614" t="n">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="E614" t="n">
         <v>1</v>
@@ -15163,17 +15163,17 @@
     <row r="615">
       <c r="A615" t="inlineStr">
         <is>
-          <t>And it is not—it’s not exactly the same as see global growth, where you see growth weakening, you see primal banks and governments responding with fiscal policy, and you see growth strengthening, and you see a business cycle.</t>
+          <t>The recent lower readings on inflation have been driven significantly by what appear to be one-murder simplification in certain categories of prices, such as wireless telephone services and prescription drugs.</t>
         </is>
       </c>
       <c r="B615" t="n">
-        <v>2020</v>
+        <v>2012</v>
       </c>
       <c r="C615" t="n">
         <v>0</v>
       </c>
       <c r="D615" t="n">
-        <v>22</v>
+        <v>251</v>
       </c>
       <c r="E615" t="n">
         <v>1</v>
@@ -15187,17 +15187,17 @@
     <row r="616">
       <c r="A616" t="inlineStr">
         <is>
-          <t>The recent lower readings on inflation have been driven significantly by what appear to be one-murder simplification in certain categories of prices, such as wireless telephone services and prescription drugs.</t>
+          <t>So you’re expire to have different perspectives from Committee player about how fast growth will be, how fast the labor market will heal, or how fast—sorry, inflation will move up.</t>
         </is>
       </c>
       <c r="B616" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="C616" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D616" t="n">
-        <v>251</v>
+        <v>213</v>
       </c>
       <c r="E616" t="n">
         <v>1</v>
@@ -15211,17 +15211,17 @@
     <row r="617">
       <c r="A617" t="inlineStr">
         <is>
-          <t>So you’re expire to have different perspectives from Committee player about how fast growth will be, how fast the labor market will heal, or how fast—sorry, inflation will move up.</t>
+          <t>Against this backdrop, today the Federal Open Market Committee raised its policy pastime rate by ¾ percentage point and anticipate that ongoing increases in that rate will be appropriate.</t>
         </is>
       </c>
       <c r="B617" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="C617" t="n">
         <v>1</v>
       </c>
       <c r="D617" t="n">
-        <v>213</v>
+        <v>5</v>
       </c>
       <c r="E617" t="n">
         <v>1</v>
@@ -15235,17 +15235,17 @@
     <row r="618">
       <c r="A618" t="inlineStr">
         <is>
-          <t>Against this backdrop, today the Federal Open Market Committee raised its policy pastime rate by ¾ percentage point and anticipate that ongoing increases in that rate will be appropriate.</t>
+          <t>We have a 2 percentage symmetric inflation objective, and, for a number of years now, inflation has been running under 2 percent.</t>
         </is>
       </c>
       <c r="B618" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="C618" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D618" t="n">
-        <v>5</v>
+        <v>278</v>
       </c>
       <c r="E618" t="n">
         <v>1</v>
@@ -15259,17 +15259,17 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>We have a 2 percentage symmetric inflation objective, and, for a number of years now, inflation has been running under 2 percent.</t>
+          <t>In addition, the median approximation of the longer-run normal unemployment rate moved down a tenth to 4.6 pct.</t>
         </is>
       </c>
       <c r="B619" t="n">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="C619" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D619" t="n">
-        <v>278</v>
+        <v>131</v>
       </c>
       <c r="E619" t="n">
         <v>1</v>
@@ -15283,17 +15283,17 @@
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>In addition, the median approximation of the longer-run normal unemployment rate moved down a tenth to 4.6 pct.</t>
+          <t>We deficiency to see lower unemployment.</t>
         </is>
       </c>
       <c r="B620" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C620" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D620" t="n">
-        <v>131</v>
+        <v>288</v>
       </c>
       <c r="E620" t="n">
         <v>1</v>
@@ -15307,17 +15307,17 @@
     <row r="621">
       <c r="A621" t="inlineStr">
         <is>
-          <t>We deficiency to see lower unemployment.</t>
+          <t>At the time of our FOMC meeting in Jan, scene for continued economic growth remained favorable, and we judged that monetary policy was well positioned to support that outlook.</t>
         </is>
       </c>
       <c r="B621" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="C621" t="n">
         <v>0</v>
       </c>
       <c r="D621" t="n">
-        <v>288</v>
+        <v>69</v>
       </c>
       <c r="E621" t="n">
         <v>1</v>
@@ -15331,17 +15331,17 @@
     <row r="622">
       <c r="A622" t="inlineStr">
         <is>
-          <t>At the time of our FOMC meeting in Jan, scene for continued economic growth remained favorable, and we judged that monetary policy was well positioned to support that outlook.</t>
+          <t>By contrast, raising rates too lento would raise the risk that monetary policy would need to tighten abruptly down the road, which could jeopardize the economic expansion.</t>
         </is>
       </c>
       <c r="B622" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="C622" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D622" t="n">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="E622" t="n">
         <v>1</v>
@@ -15355,17 +15355,17 @@
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
-          <t>By contrast, raising rates too lento would raise the risk that monetary policy would need to tighten abruptly down the road, which could jeopardize the economic expansion.</t>
+          <t>We, candidly, didn’t even get inflation back up to target—without seeing wages take out of touch with—with where they should be, so that’s the—that’s the biggest thing we can do.</t>
         </is>
       </c>
       <c r="B623" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C623" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D623" t="n">
-        <v>94</v>
+        <v>290</v>
       </c>
       <c r="E623" t="n">
         <v>1</v>
@@ -15379,7 +15379,7 @@
     <row r="624">
       <c r="A624" t="inlineStr">
         <is>
-          <t>We, candidly, didn’t even get inflation back up to target—without seeing wages take out of touch with—with where they should be, so that’s the—that’s the biggest thing we can do.</t>
+          <t>We have not focused on whether we meet the liftoff examination, because we assume’t meet the liftoff test now because we’re not at maximum employment.</t>
         </is>
       </c>
       <c r="B624" t="n">
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="D624" t="n">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="E624" t="n">
         <v>1</v>
@@ -15403,17 +15403,17 @@
     <row r="625">
       <c r="A625" t="inlineStr">
         <is>
-          <t>We have not focused on whether we meet the liftoff examination, because we assume’t meet the liftoff test now because we’re not at maximum employment.</t>
+          <t>The Federal Reserve is fully committed to both sides of its mandatory—to price stability as well as to uttermost employment—and it has both the tools and the will to act at the appropriate time to avoid any emerging threat to price stability.</t>
         </is>
       </c>
       <c r="B625" t="n">
         <v>2020</v>
       </c>
       <c r="C625" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D625" t="n">
-        <v>283</v>
+        <v>235</v>
       </c>
       <c r="E625" t="n">
         <v>1</v>
@@ -15427,17 +15427,17 @@
     <row r="626">
       <c r="A626" t="inlineStr">
         <is>
-          <t>The Federal Reserve is fully committed to both sides of its mandatory—to price stability as well as to uttermost employment—and it has both the tools and the will to act at the appropriate time to avoid any emerging threat to price stability.</t>
+          <t>Well, you’re certainly right that we have been over-optimistic about taboo-year growth.</t>
         </is>
       </c>
       <c r="B626" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C626" t="n">
         <v>1</v>
       </c>
       <c r="D626" t="n">
-        <v>235</v>
+        <v>296</v>
       </c>
       <c r="E626" t="n">
         <v>1</v>
@@ -15451,17 +15451,17 @@
     <row r="627">
       <c r="A627" t="inlineStr">
         <is>
-          <t>Well, you’re certainly right that we have been over-optimistic about taboo-year growth.</t>
+          <t>We think that the economy will need highly accommodative monetary policy and the enjoyment of our tools for an extended period.</t>
         </is>
       </c>
       <c r="B627" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C627" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D627" t="n">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="E627" t="n">
         <v>1</v>
@@ -15475,17 +15475,17 @@
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>We think that the economy will need highly accommodative monetary policy and the enjoyment of our tools for an extended period.</t>
+          <t>And productiveness’s been very low.</t>
         </is>
       </c>
       <c r="B628" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C628" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D628" t="n">
-        <v>286</v>
+        <v>30</v>
       </c>
       <c r="E628" t="n">
         <v>1</v>
@@ -15499,17 +15499,17 @@
     <row r="629">
       <c r="A629" t="inlineStr">
         <is>
-          <t>And productiveness’s been very low.</t>
+          <t>The persistence of that into, into inflation over clip is just not there.</t>
         </is>
       </c>
       <c r="B629" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C629" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D629" t="n">
-        <v>30</v>
+        <v>249</v>
       </c>
       <c r="E629" t="n">
         <v>1</v>
@@ -15523,17 +15523,17 @@
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
-          <t>The persistence of that into, into inflation over clip is just not there.</t>
+          <t>So, if we maintain a highly accommodative monetary policy for a very long metre from here and the economy performs as we expect—namely, it’s strong and the risks that are kayoed there don’t materialize—my concern will be that we will have much more tightening in labor markets than you view in these projections.</t>
         </is>
       </c>
       <c r="B630" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C630" t="n">
         <v>0</v>
       </c>
       <c r="D630" t="n">
-        <v>249</v>
+        <v>219</v>
       </c>
       <c r="E630" t="n">
         <v>1</v>
@@ -15547,17 +15547,17 @@
     <row r="631">
       <c r="A631" t="inlineStr">
         <is>
-          <t>So, if we maintain a highly accommodative monetary policy for a very long metre from here and the economy performs as we expect—namely, it’s strong and the risks that are kayoed there don’t materialize—my concern will be that we will have much more tightening in labor markets than you view in these projections.</t>
+          <t>We had a 10 percentage unemployment rate, and our congressional mandate is maximum employment and price stability.</t>
         </is>
       </c>
       <c r="B631" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="C631" t="n">
         <v>0</v>
       </c>
       <c r="D631" t="n">
-        <v>219</v>
+        <v>276</v>
       </c>
       <c r="E631" t="n">
         <v>1</v>
@@ -15571,17 +15571,17 @@
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>We had a 10 percentage unemployment rate, and our congressional mandate is maximum employment and price stability.</t>
+          <t>You recognise, what you hear out there is that demand—you talk to banks, and they’ll allege demand for loans is very, very low right now.</t>
         </is>
       </c>
       <c r="B632" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="C632" t="n">
         <v>0</v>
       </c>
       <c r="D632" t="n">
-        <v>276</v>
+        <v>313</v>
       </c>
       <c r="E632" t="n">
         <v>1</v>
@@ -15595,7 +15595,7 @@
     <row r="633">
       <c r="A633" t="inlineStr">
         <is>
-          <t>You recognise, what you hear out there is that demand—you talk to banks, and they’ll allege demand for loans is very, very low right now.</t>
+          <t>So, with this coronavirus arriving, we judged that the—the net effects of this will be to—to have inflation move down even a piddling turn more.</t>
         </is>
       </c>
       <c r="B633" t="n">
@@ -15605,7 +15605,7 @@
         <v>0</v>
       </c>
       <c r="D633" t="n">
-        <v>313</v>
+        <v>222</v>
       </c>
       <c r="E633" t="n">
         <v>1</v>
@@ -15619,17 +15619,17 @@
     <row r="634">
       <c r="A634" t="inlineStr">
         <is>
-          <t>So, with this coronavirus arriving, we judged that the—the net effects of this will be to—to have inflation move down even a piddling turn more.</t>
+          <t>These headwinds—which admit developments abroad, subdued household organization, and meager productivity growth—could persist for some time.</t>
         </is>
       </c>
       <c r="B634" t="n">
-        <v>2014</v>
+        <v>2022</v>
       </c>
       <c r="C634" t="n">
         <v>0</v>
       </c>
       <c r="D634" t="n">
-        <v>222</v>
+        <v>262</v>
       </c>
       <c r="E634" t="n">
         <v>1</v>
@@ -15643,17 +15643,17 @@
     <row r="635">
       <c r="A635" t="inlineStr">
         <is>
-          <t>These headwinds—which admit developments abroad, subdued household organization, and meager productivity growth—could persist for some time.</t>
+          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can raise interest rates at the reserve time, even if the balance sheet remains large for an extended menstruum.</t>
         </is>
       </c>
       <c r="B635" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C635" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D635" t="n">
-        <v>262</v>
+        <v>188</v>
       </c>
       <c r="E635" t="n">
         <v>1</v>
@@ -15667,17 +15667,17 @@
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
-          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can raise interest rates at the reserve time, even if the balance sheet remains large for an extended menstruum.</t>
+          <t>And no, we’re not—we, we have not at all changed our scene, and I harbor’t changed my view that inflation running above 2 percent, moderately above 2 percent, is a desirable thing.</t>
         </is>
       </c>
       <c r="B636" t="n">
-        <v>2020</v>
+        <v>2011</v>
       </c>
       <c r="C636" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D636" t="n">
-        <v>188</v>
+        <v>25</v>
       </c>
       <c r="E636" t="n">
         <v>1</v>
@@ -15691,17 +15691,17 @@
     <row r="637">
       <c r="A637" t="inlineStr">
         <is>
-          <t>And no, we’re not—we, we have not at all changed our scene, and I harbor’t changed my view that inflation running above 2 percent, moderately above 2 percent, is a desirable thing.</t>
+          <t>Foresightful-term unemployment in the current economy is—is the worst—really the worst it’s been in the postwar period.</t>
         </is>
       </c>
       <c r="B637" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C637" t="n">
         <v>0</v>
       </c>
       <c r="D637" t="n">
-        <v>25</v>
+        <v>162</v>
       </c>
       <c r="E637" t="n">
         <v>1</v>
@@ -15715,17 +15715,17 @@
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
-          <t>Foresightful-term unemployment in the current economy is—is the worst—really the worst it’s been in the postwar period.</t>
+          <t>Well, if the economy worsens and inflation remains relatively low, then we wouldn’t begin to loss, and, therefore, we wouldn’t change the lyric.</t>
         </is>
       </c>
       <c r="B638" t="n">
-        <v>2012</v>
+        <v>2020</v>
       </c>
       <c r="C638" t="n">
         <v>0</v>
       </c>
       <c r="D638" t="n">
-        <v>162</v>
+        <v>291</v>
       </c>
       <c r="E638" t="n">
         <v>1</v>
@@ -15739,17 +15739,17 @@
     <row r="639">
       <c r="A639" t="inlineStr">
         <is>
-          <t>Well, if the economy worsens and inflation remains relatively low, then we wouldn’t begin to loss, and, therefore, we wouldn’t change the lyric.</t>
+          <t>Well, you know, if the economy were disappointing, we—you know, our action wouldn’t strictly be based on inflation, we would also take employment into account.</t>
         </is>
       </c>
       <c r="B639" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C639" t="n">
         <v>0</v>
       </c>
       <c r="D639" t="n">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="E639" t="n">
         <v>1</v>
@@ -15763,17 +15763,17 @@
     <row r="640">
       <c r="A640" t="inlineStr">
         <is>
-          <t>Well, you know, if the economy were disappointing, we—you know, our action wouldn’t strictly be based on inflation, we would also take employment into account.</t>
+          <t>The Federal Reserve’s response is guided by our mandate to advance maximum employment and stalls prices for the American people, along with our responsibilities to promote the stability of the financial system.</t>
         </is>
       </c>
       <c r="B640" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C640" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D640" t="n">
-        <v>295</v>
+        <v>237</v>
       </c>
       <c r="E640" t="n">
         <v>1</v>
@@ -15787,41 +15787,41 @@
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>The Federal Reserve’s response is guided by our mandate to advance maximum employment and stalls prices for the American people, along with our responsibilities to promote the stability of the financial system.</t>
+          <t>For [MASK], we have [MASK] some [MASK] our work to look [MASK] interest rate risk and [MASK] [MASK] [MASK] and, you know, found generally that banks can also sustain a significant increase in long-term interest [MASK] as well for [MASK] number of reasons, one of them being that higher interest rates increase their franchise value because it increases their net interest [MASK] over time.</t>
         </is>
       </c>
       <c r="B641" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C641" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D641" t="n">
-        <v>237</v>
+        <v>104</v>
       </c>
       <c r="E641" t="n">
         <v>1</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>synonym_replacement</t>
+          <t>masking</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>For [MASK], we have [MASK] some [MASK] our work to look [MASK] interest rate risk and [MASK] [MASK] [MASK] and, you know, found generally that banks can also sustain a significant increase in long-term interest [MASK] as well for [MASK] number of reasons, one of them being that higher interest rates increase their franchise value because it increases their net interest [MASK] over time.</t>
+          <t>[MASK]—and we do that with [MASK] that—that, you know, keep people in their homes; that—that support hiring; that support [MASK]; that avoid unnecessary, avoidable business [MASK].</t>
         </is>
       </c>
       <c r="B642" t="n">
-        <v>2021</v>
+        <v>2011</v>
       </c>
       <c r="C642" t="n">
         <v>2</v>
       </c>
       <c r="D642" t="n">
-        <v>104</v>
+        <v>58</v>
       </c>
       <c r="E642" t="n">
         <v>1</v>
@@ -15835,17 +15835,17 @@
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>[MASK]—and we do that with [MASK] that—that, you know, keep people in their homes; that—that support hiring; that support [MASK]; that avoid unnecessary, avoidable business [MASK].</t>
+          <t>For example, one—in the long-[MASK], the size of the balance sheet is going [MASK] [MASK] on the public’s demand for our liabilities, including currency [MASK] reserves.</t>
         </is>
       </c>
       <c r="B643" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="C643" t="n">
         <v>2</v>
       </c>
       <c r="D643" t="n">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="E643" t="n">
         <v>1</v>
@@ -15859,17 +15859,17 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>For example, one—in the long-[MASK], the size of the balance sheet is going [MASK] [MASK] on the public’s demand for our liabilities, including currency [MASK] reserves.</t>
+          <t>Now, [MASK] inflation below 2 percent, I think it’s appropriate that [MASK] labor market [MASK] that tight.</t>
         </is>
       </c>
       <c r="B644" t="n">
         <v>2021</v>
       </c>
       <c r="C644" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D644" t="n">
-        <v>102</v>
+        <v>172</v>
       </c>
       <c r="E644" t="n">
         <v>1</v>
@@ -15883,17 +15883,17 @@
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>Now, [MASK] inflation below 2 percent, I think it’s appropriate that [MASK] labor market [MASK] that tight.</t>
+          <t>The jobs picture continues to be [MASK], with the unemployment rate near historic lows [MASK] with stronger wage [MASK].</t>
         </is>
       </c>
       <c r="B645" t="n">
         <v>2021</v>
       </c>
       <c r="C645" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D645" t="n">
-        <v>172</v>
+        <v>247</v>
       </c>
       <c r="E645" t="n">
         <v>1</v>
@@ -15907,7 +15907,7 @@
     <row r="646">
       <c r="A646" t="inlineStr">
         <is>
-          <t>The jobs picture continues to be [MASK], with the unemployment rate near historic lows [MASK] with stronger wage [MASK].</t>
+          <t>Our role, though, is also to, [MASK] know, to make [MASK] [MASK]—that maximum employment happens in a context of [MASK] stability and financial stability, which is why we’re [MASK] raising rates.</t>
         </is>
       </c>
       <c r="B646" t="n">
@@ -15917,7 +15917,7 @@
         <v>1</v>
       </c>
       <c r="D646" t="n">
-        <v>247</v>
+        <v>179</v>
       </c>
       <c r="E646" t="n">
         <v>1</v>
@@ -15931,17 +15931,17 @@
     <row r="647">
       <c r="A647" t="inlineStr">
         <is>
-          <t>Our role, though, is also to, [MASK] know, to make [MASK] [MASK]—that maximum employment happens in a context of [MASK] stability and financial stability, which is why we’re [MASK] raising rates.</t>
+          <t>In addition, [MASK] median estimate of the longer-run normal [MASK] rate moved down [MASK] tenth to 4.6 percent.</t>
         </is>
       </c>
       <c r="B647" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C647" t="n">
         <v>1</v>
       </c>
       <c r="D647" t="n">
-        <v>179</v>
+        <v>131</v>
       </c>
       <c r="E647" t="n">
         <v>1</v>
@@ -15955,17 +15955,17 @@
     <row r="648">
       <c r="A648" t="inlineStr">
         <is>
-          <t>In addition, [MASK] median estimate of the longer-run normal [MASK] rate moved down [MASK] tenth to 4.6 percent.</t>
+          <t>That transition [MASK] could help bring inflation down, because, presumably, people would spend a little less on [MASK] while they start spending [MASK] on travel and all [MASK] of travel services [MASK] things like that.</t>
         </is>
       </c>
       <c r="B648" t="n">
-        <v>2022</v>
+        <v>2016</v>
       </c>
       <c r="C648" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D648" t="n">
-        <v>131</v>
+        <v>229</v>
       </c>
       <c r="E648" t="n">
         <v>1</v>
@@ -15979,17 +15979,17 @@
     <row r="649">
       <c r="A649" t="inlineStr">
         <is>
-          <t>That transition [MASK] could help bring inflation down, because, presumably, people would spend a little less on [MASK] while they start spending [MASK] on travel and all [MASK] of travel services [MASK] things like that.</t>
+          <t>[MASK] [MASK] has not—what, what [MASK] is that [MASK] wages move up because unemployment is low, companies have been absorbing that increase into their margins rather than raising prices.</t>
         </is>
       </c>
       <c r="B649" t="n">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="C649" t="n">
         <v>2</v>
       </c>
       <c r="D649" t="n">
-        <v>229</v>
+        <v>84</v>
       </c>
       <c r="E649" t="n">
         <v>1</v>
@@ -16003,17 +16003,17 @@
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t>[MASK] [MASK] has not—what, what [MASK] is that [MASK] wages move up because unemployment is low, companies have been absorbing that increase into their margins rather than raising prices.</t>
+          <t>So you’[MASK] talking about the inflation target, basically.</t>
         </is>
       </c>
       <c r="B650" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C650" t="n">
         <v>2</v>
       </c>
       <c r="D650" t="n">
-        <v>84</v>
+        <v>215</v>
       </c>
       <c r="E650" t="n">
         <v>1</v>
@@ -16027,17 +16027,17 @@
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>So you’[MASK] talking about the inflation target, basically.</t>
+          <t>[MASK], and those [MASK]—that’s again—that goes to [MASK] this episode as short [MASK] it can be and avoiding unnecessary business bankruptcies, unnecessary household bankruptcies, [MASK] unnecessary long-term stays of unemployment or supporting [MASK] through them so [MASK] they [MASK] maintain their financial footing and their lives [MASK] be able to go back to work in a productive way.</t>
         </is>
       </c>
       <c r="B651" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="C651" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D651" t="n">
-        <v>215</v>
+        <v>52</v>
       </c>
       <c r="E651" t="n">
         <v>1</v>
@@ -16051,17 +16051,17 @@
     <row r="652">
       <c r="A652" t="inlineStr">
         <is>
-          <t>[MASK], and those [MASK]—that’s again—that goes to [MASK] this episode as short [MASK] it can be and avoiding unnecessary business bankruptcies, unnecessary household bankruptcies, [MASK] unnecessary long-term stays of unemployment or supporting [MASK] through them so [MASK] they [MASK] maintain their financial footing and their lives [MASK] be able to go back to work in a productive way.</t>
+          <t>By the way, we’re also not at [MASK] employment, [MASK] I mentioned.</t>
         </is>
       </c>
       <c r="B652" t="n">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="C652" t="n">
         <v>0</v>
       </c>
       <c r="D652" t="n">
-        <v>52</v>
+        <v>96</v>
       </c>
       <c r="E652" t="n">
         <v>1</v>
@@ -16075,17 +16075,17 @@
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>By the way, we’re also not at [MASK] employment, [MASK] I mentioned.</t>
+          <t>But now, let’s go to [MASK]—the part of your question about [MASK].</t>
         </is>
       </c>
       <c r="B653" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="C653" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D653" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="E653" t="n">
         <v>1</v>
@@ -16099,17 +16099,17 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>But now, let’s go to [MASK]—the part of your question about [MASK].</t>
+          <t>So that means a more [MASK] shortfall of inflation.</t>
         </is>
       </c>
       <c r="B654" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C654" t="n">
         <v>2</v>
       </c>
       <c r="D654" t="n">
-        <v>83</v>
+        <v>199</v>
       </c>
       <c r="E654" t="n">
         <v>1</v>
@@ -16123,17 +16123,17 @@
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>So that means a more [MASK] shortfall of inflation.</t>
+          <t>[MASK]’s a lot more demand for risk [MASK], for liquidity services, and so on.</t>
         </is>
       </c>
       <c r="B655" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="C655" t="n">
         <v>2</v>
       </c>
       <c r="D655" t="n">
-        <v>199</v>
+        <v>259</v>
       </c>
       <c r="E655" t="n">
         <v>1</v>
@@ -16147,17 +16147,17 @@
     <row r="656">
       <c r="A656" t="inlineStr">
         <is>
-          <t>[MASK]’s a lot more demand for risk [MASK], for liquidity services, and so on.</t>
+          <t>And [MASK]’s been very low.</t>
         </is>
       </c>
       <c r="B656" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="C656" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D656" t="n">
-        <v>259</v>
+        <v>30</v>
       </c>
       <c r="E656" t="n">
         <v>1</v>
@@ -16171,17 +16171,17 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>And [MASK]’s been very low.</t>
+          <t>As I mentioned, once [MASK]—once you’re, broadly speaking, in the range of neutral, I [MASK] it’[MASK] appropriate to be putting [MASK] individual estimates of that [MASK] be looking at what the incoming data are [MASK] you [MASK] the outlook, updating your estimates of what neutral might be, of what the natural [MASK] [MASK] unemployment might be, of the state of the economy, [MASK]—and letting that lead you to adjust your [MASK] and, therefore, your appropriate [MASK] for policy.</t>
         </is>
       </c>
       <c r="B657" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="C657" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D657" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="E657" t="n">
         <v>1</v>
@@ -16195,17 +16195,17 @@
     <row r="658">
       <c r="A658" t="inlineStr">
         <is>
-          <t>As I mentioned, once [MASK]—once you’re, broadly speaking, in the range of neutral, I [MASK] it’[MASK] appropriate to be putting [MASK] individual estimates of that [MASK] be looking at what the incoming data are [MASK] you [MASK] the outlook, updating your estimates of what neutral might be, of what the natural [MASK] [MASK] unemployment might be, of the state of the economy, [MASK]—and letting that lead you to adjust your [MASK] and, therefore, your appropriate [MASK] for policy.</t>
+          <t>So it’[MASK] a serious economic problem [MASK] the United [MASK], but it’s—it’s got underlying causes that [MASK] not [MASK] to monetary policy or to our response to the pandemic.</t>
         </is>
       </c>
       <c r="B658" t="n">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="C658" t="n">
         <v>2</v>
       </c>
       <c r="D658" t="n">
-        <v>61</v>
+        <v>194</v>
       </c>
       <c r="E658" t="n">
         <v>1</v>
@@ -16219,17 +16219,17 @@
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
-          <t>So it’[MASK] a serious economic problem [MASK] the United [MASK], but it’s—it’s got underlying causes that [MASK] not [MASK] to monetary policy or to our response to the pandemic.</t>
+          <t>So, you [MASK], as I [MASK], the Committee acutely feels its [MASK] to move to make sure that [MASK] restore price stability [MASK] is determined to use its tools to do so.</t>
         </is>
       </c>
       <c r="B659" t="n">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="C659" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D659" t="n">
-        <v>194</v>
+        <v>224</v>
       </c>
       <c r="E659" t="n">
         <v>1</v>
@@ -16243,17 +16243,17 @@
     <row r="660">
       <c r="A660" t="inlineStr">
         <is>
-          <t>So, you [MASK], as I [MASK], the Committee acutely feels its [MASK] to move to make sure that [MASK] restore price stability [MASK] is determined to use its tools to do so.</t>
+          <t>And so when asset prices [MASK] back up, probably there’ll [MASK] a swing around there, a positive [MASK].</t>
         </is>
       </c>
       <c r="B660" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="C660" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D660" t="n">
-        <v>224</v>
+        <v>32</v>
       </c>
       <c r="E660" t="n">
         <v>1</v>
@@ -16267,7 +16267,7 @@
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>And so when asset prices [MASK] back up, probably there’ll [MASK] a swing around there, a positive [MASK].</t>
+          <t>We also don’t conduct monetary [MASK] [MASK] order to prove our independence.</t>
         </is>
       </c>
       <c r="B661" t="n">
@@ -16277,7 +16277,7 @@
         <v>2</v>
       </c>
       <c r="D661" t="n">
-        <v>32</v>
+        <v>270</v>
       </c>
       <c r="E661" t="n">
         <v>1</v>
@@ -16291,17 +16291,17 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>We also don’t conduct monetary [MASK] [MASK] order to prove our independence.</t>
+          <t>Inflation pressures [MASK] muted, and indicators of [MASK]-[MASK] inflation expectations are at the lower end of their historic ranges.</t>
         </is>
       </c>
       <c r="B662" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="C662" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D662" t="n">
-        <v>270</v>
+        <v>145</v>
       </c>
       <c r="E662" t="n">
         <v>1</v>
@@ -16315,17 +16315,17 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Inflation pressures [MASK] muted, and indicators of [MASK]-[MASK] inflation expectations are at the lower end of their historic ranges.</t>
+          <t>And, and some [MASK] [MASK] answer to that may be price.</t>
         </is>
       </c>
       <c r="B663" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="C663" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D663" t="n">
-        <v>145</v>
+        <v>50</v>
       </c>
       <c r="E663" t="n">
         <v>1</v>
@@ -16339,17 +16339,17 @@
     <row r="664">
       <c r="A664" t="inlineStr">
         <is>
-          <t>And, and some [MASK] [MASK] answer to that may be price.</t>
+          <t>[MASK] you’re right, you’re seeing—I, I can’t remember the number, but [MASK] might be [MASK] [MASK] 3s—3, 3½ percent growth for next year.</t>
         </is>
       </c>
       <c r="B664" t="n">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="C664" t="n">
         <v>2</v>
       </c>
       <c r="D664" t="n">
-        <v>50</v>
+        <v>214</v>
       </c>
       <c r="E664" t="n">
         <v>1</v>
@@ -16363,17 +16363,17 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>[MASK] you’re right, you’re seeing—I, I can’t remember the number, but [MASK] might be [MASK] [MASK] 3s—3, 3½ percent growth for next year.</t>
+          <t>We have not focused on whether we meet [MASK] liftoff test, because we don’t [MASK] the liftoff [MASK] now [MASK] we’re not at maximum employment.</t>
         </is>
       </c>
       <c r="B665" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C665" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D665" t="n">
-        <v>214</v>
+        <v>283</v>
       </c>
       <c r="E665" t="n">
         <v>1</v>
@@ -16387,7 +16387,7 @@
     <row r="666">
       <c r="A666" t="inlineStr">
         <is>
-          <t>We have not focused on whether we meet [MASK] liftoff test, because we don’t [MASK] the liftoff [MASK] now [MASK] we’re not at maximum employment.</t>
+          <t>And it is not—it’s not exactly the same as watching global [MASK], where [MASK] see growth weakening, [MASK] [MASK] central banks and governments responding with fiscal policy, and you see growth [MASK], and [MASK] see a business cycle.</t>
         </is>
       </c>
       <c r="B666" t="n">
@@ -16397,7 +16397,7 @@
         <v>0</v>
       </c>
       <c r="D666" t="n">
-        <v>283</v>
+        <v>22</v>
       </c>
       <c r="E666" t="n">
         <v>1</v>
@@ -16411,17 +16411,17 @@
     <row r="667">
       <c r="A667" t="inlineStr">
         <is>
-          <t>And it is not—it’s not exactly the same as watching global [MASK], where [MASK] see growth weakening, [MASK] [MASK] central banks and governments responding with fiscal policy, and you see growth [MASK], and [MASK] see a business cycle.</t>
+          <t>It isn’t really just targeting the [MASK] numbers, but [MASK]’s about taking [MASK] of those things into [MASK] in your thinking about what constitutes maximum employment.</t>
         </is>
       </c>
       <c r="B667" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C667" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D667" t="n">
-        <v>22</v>
+        <v>150</v>
       </c>
       <c r="E667" t="n">
         <v>1</v>
@@ -16435,17 +16435,17 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>It isn’t really just targeting the [MASK] numbers, but [MASK]’s about taking [MASK] of those things into [MASK] in your thinking about what constitutes maximum employment.</t>
+          <t>[MASK] tools work on demand.</t>
         </is>
       </c>
       <c r="B668" t="n">
-        <v>2021</v>
+        <v>2012</v>
       </c>
       <c r="C668" t="n">
         <v>2</v>
       </c>
       <c r="D668" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="E668" t="n">
         <v>1</v>
@@ -16459,17 +16459,17 @@
     <row r="669">
       <c r="A669" t="inlineStr">
         <is>
-          <t>[MASK] tools work on demand.</t>
+          <t>I would say, in the area of commercial real [MASK], [MASK] valuations [MASK] [MASK], we are seeing some tightening of lending standards [MASK] less debt growth associated with that rise in commercial real estate prices.</t>
         </is>
       </c>
       <c r="B669" t="n">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="C669" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D669" t="n">
-        <v>180</v>
+        <v>122</v>
       </c>
       <c r="E669" t="n">
         <v>1</v>
@@ -16483,17 +16483,17 @@
     <row r="670">
       <c r="A670" t="inlineStr">
         <is>
-          <t>I would say, in the area of commercial real [MASK], [MASK] valuations [MASK] [MASK], we are seeing some tightening of lending standards [MASK] less debt growth associated with that rise in commercial real estate prices.</t>
+          <t>If inflation remains higher during the course [MASK] 2022, [MASK] we may already [MASK] met that test by the time we reach liftoff.</t>
         </is>
       </c>
       <c r="B670" t="n">
         <v>2016</v>
       </c>
       <c r="C670" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D670" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E670" t="n">
         <v>1</v>
@@ -16507,17 +16507,17 @@
     <row r="671">
       <c r="A671" t="inlineStr">
         <is>
-          <t>If inflation remains higher during the course [MASK] 2022, [MASK] we may already [MASK] met that test by the time we reach liftoff.</t>
+          <t>You know, we’re, [MASK]’re—inflation measures are always going to be a [MASK] volatile.</t>
         </is>
       </c>
       <c r="B671" t="n">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="C671" t="n">
         <v>2</v>
       </c>
       <c r="D671" t="n">
-        <v>123</v>
+        <v>312</v>
       </c>
       <c r="E671" t="n">
         <v>1</v>
@@ -16531,17 +16531,17 @@
     <row r="672">
       <c r="A672" t="inlineStr">
         <is>
-          <t>You know, we’re, [MASK]’re—inflation measures are always going to be a [MASK] volatile.</t>
+          <t>We're [MASK] at wages and we're looking [MASK] ultimately inflation.</t>
         </is>
       </c>
       <c r="B672" t="n">
-        <v>2014</v>
+        <v>2019</v>
       </c>
       <c r="C672" t="n">
         <v>2</v>
       </c>
       <c r="D672" t="n">
-        <v>312</v>
+        <v>289</v>
       </c>
       <c r="E672" t="n">
         <v>1</v>
@@ -16555,17 +16555,17 @@
     <row r="673">
       <c r="A673" t="inlineStr">
         <is>
-          <t>We're [MASK] at wages and we're looking [MASK] ultimately inflation.</t>
+          <t>So you’re [MASK] to have different perspectives from Committee participants about how fast growth will be, how [MASK] [MASK] labor market will [MASK], or how fast—sorry, inflation [MASK] move up.</t>
         </is>
       </c>
       <c r="B673" t="n">
         <v>2019</v>
       </c>
       <c r="C673" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D673" t="n">
-        <v>289</v>
+        <v>213</v>
       </c>
       <c r="E673" t="n">
         <v>1</v>
@@ -16579,17 +16579,17 @@
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>So you’re [MASK] to have different perspectives from Committee participants about how fast growth will be, how [MASK] [MASK] labor market will [MASK], or how fast—sorry, inflation [MASK] move up.</t>
+          <t>And that’[MASK] because of this misalignment [MASK] supply and demand.</t>
         </is>
       </c>
       <c r="B674" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="C674" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D674" t="n">
-        <v>213</v>
+        <v>36</v>
       </c>
       <c r="E674" t="n">
         <v>1</v>
@@ -16603,7 +16603,7 @@
     <row r="675">
       <c r="A675" t="inlineStr">
         <is>
-          <t>And that’[MASK] because of this misalignment [MASK] supply and demand.</t>
+          <t>But, certainly, we’ve had a lot of [MASK] in which interest rates [MASK] been low.</t>
         </is>
       </c>
       <c r="B675" t="n">
@@ -16613,7 +16613,7 @@
         <v>2</v>
       </c>
       <c r="D675" t="n">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="E675" t="n">
         <v>1</v>
@@ -16627,17 +16627,17 @@
     <row r="676">
       <c r="A676" t="inlineStr">
         <is>
-          <t>But, certainly, we’ve had a lot of [MASK] in which interest rates [MASK] been low.</t>
+          <t>So, as you know, the ultimate focus that we have is [MASK] [MASK] real economy: maximum employment [MASK] price stability.</t>
         </is>
       </c>
       <c r="B676" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C676" t="n">
         <v>2</v>
       </c>
       <c r="D676" t="n">
-        <v>90</v>
+        <v>218</v>
       </c>
       <c r="E676" t="n">
         <v>1</v>
@@ -16651,17 +16651,17 @@
     <row r="677">
       <c r="A677" t="inlineStr">
         <is>
-          <t>So, as you know, the ultimate focus that we have is [MASK] [MASK] real economy: maximum employment [MASK] price stability.</t>
+          <t>And the maximum level of [MASK] that’s consistent with price [MASK] evolves over time within a—within [MASK] business [MASK] and over a longer [MASK], in part reflecting [the] evolution [MASK] the factors that affect labor supply, [MASK] those related to the pandemic.</t>
         </is>
       </c>
       <c r="B677" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="C677" t="n">
         <v>2</v>
       </c>
       <c r="D677" t="n">
-        <v>218</v>
+        <v>37</v>
       </c>
       <c r="E677" t="n">
         <v>1</v>
@@ -16675,17 +16675,17 @@
     <row r="678">
       <c r="A678" t="inlineStr">
         <is>
-          <t>And the maximum level of [MASK] that’s consistent with price [MASK] evolves over time within a—within [MASK] business [MASK] and over a longer [MASK], in part reflecting [the] evolution [MASK] the factors that affect labor supply, [MASK] those related to the pandemic.</t>
+          <t>So [MASK] Committee estimates that the longer-run normal level [MASK] the unemployment rate is 5.0 to 5.2.</t>
         </is>
       </c>
       <c r="B678" t="n">
-        <v>2022</v>
+        <v>2013</v>
       </c>
       <c r="C678" t="n">
         <v>2</v>
       </c>
       <c r="D678" t="n">
-        <v>37</v>
+        <v>202</v>
       </c>
       <c r="E678" t="n">
         <v>1</v>
@@ -16699,17 +16699,17 @@
     <row r="679">
       <c r="A679" t="inlineStr">
         <is>
-          <t>So [MASK] Committee estimates that the longer-run normal level [MASK] the unemployment rate is 5.0 to 5.2.</t>
+          <t>Last year, we [MASK] 1.9 percent productivity, which is much [MASK].</t>
         </is>
       </c>
       <c r="B679" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="C679" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D679" t="n">
-        <v>202</v>
+        <v>161</v>
       </c>
       <c r="E679" t="n">
         <v>1</v>
@@ -16723,17 +16723,17 @@
     <row r="680">
       <c r="A680" t="inlineStr">
         <is>
-          <t>Last year, we [MASK] 1.9 percent productivity, which is much [MASK].</t>
+          <t>So, we are taking [MASK] of international developments, including prospects for [MASK] in our [MASK] partners, in making the forecast we have here.</t>
         </is>
       </c>
       <c r="B680" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="C680" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D680" t="n">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="E680" t="n">
         <v>1</v>
@@ -16747,17 +16747,17 @@
     <row r="681">
       <c r="A681" t="inlineStr">
         <is>
-          <t>So, we are taking [MASK] of international developments, including prospects for [MASK] in our [MASK] partners, in making the forecast we have here.</t>
+          <t>If we—if we analyze inflation data and conclude [MASK], [MASK], transitory influences are holding down inflation, I do [MASK] want to say that we would [MASK] to that.</t>
         </is>
       </c>
       <c r="B681" t="n">
-        <v>2014</v>
+        <v>2021</v>
       </c>
       <c r="C681" t="n">
         <v>2</v>
       </c>
       <c r="D681" t="n">
-        <v>221</v>
+        <v>126</v>
       </c>
       <c r="E681" t="n">
         <v>1</v>
@@ -16771,17 +16771,17 @@
     <row r="682">
       <c r="A682" t="inlineStr">
         <is>
-          <t>If we—if we analyze inflation data and conclude [MASK], [MASK], transitory influences are holding down inflation, I do [MASK] want to say that we would [MASK] to that.</t>
+          <t>If we think that the potential growth rate [MASK] the economy [MASK] somewhere between, somewhere around 1.75 [MASK], 2.8 percent is strong economic growth.</t>
         </is>
       </c>
       <c r="B682" t="n">
         <v>2021</v>
       </c>
       <c r="C682" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D682" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E682" t="n">
         <v>1</v>
@@ -16795,17 +16795,17 @@
     <row r="683">
       <c r="A683" t="inlineStr">
         <is>
-          <t>If we think that the potential growth rate [MASK] the economy [MASK] somewhere between, somewhere around 1.75 [MASK], 2.8 percent is strong economic growth.</t>
+          <t>So in—in—in U-6, the U-6 level [MASK] [MASK] has tripled from 7 percent to 21 percent.</t>
         </is>
       </c>
       <c r="B683" t="n">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="C683" t="n">
         <v>0</v>
       </c>
       <c r="D683" t="n">
-        <v>125</v>
+        <v>192</v>
       </c>
       <c r="E683" t="n">
         <v>1</v>
@@ -16819,17 +16819,17 @@
     <row r="684">
       <c r="A684" t="inlineStr">
         <is>
-          <t>So in—in—in U-6, the U-6 level [MASK] [MASK] has tripled from 7 percent to 21 percent.</t>
+          <t>[MASK] I assure you that my [MASK] and [MASK] will continue to conduct monetary policy without regard to political considerations.</t>
         </is>
       </c>
       <c r="B684" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="C684" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D684" t="n">
-        <v>192</v>
+        <v>8</v>
       </c>
       <c r="E684" t="n">
         <v>1</v>
@@ -16843,17 +16843,17 @@
     <row r="685">
       <c r="A685" t="inlineStr">
         <is>
-          <t>[MASK] I assure you that my [MASK] and [MASK] will continue to conduct monetary policy without regard to political considerations.</t>
+          <t>There [MASK] a lot of pent-up demand.</t>
         </is>
       </c>
       <c r="B685" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="C685" t="n">
         <v>2</v>
       </c>
       <c r="D685" t="n">
-        <v>8</v>
+        <v>258</v>
       </c>
       <c r="E685" t="n">
         <v>1</v>
@@ -16867,17 +16867,17 @@
     <row r="686">
       <c r="A686" t="inlineStr">
         <is>
-          <t>There [MASK] a lot of pent-up demand.</t>
+          <t>You know, it’s interest rates, it’s risk spreads, it’s currency, it’s [MASK] [MASK] [MASK], it’s credit availability, it’s many, [MASK] factors.</t>
         </is>
       </c>
       <c r="B686" t="n">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="C686" t="n">
         <v>2</v>
       </c>
       <c r="D686" t="n">
-        <v>258</v>
+        <v>309</v>
       </c>
       <c r="E686" t="n">
         <v>1</v>
@@ -16891,17 +16891,17 @@
     <row r="687">
       <c r="A687" t="inlineStr">
         <is>
-          <t>You know, it’s interest rates, it’s risk spreads, it’s currency, it’s [MASK] [MASK] [MASK], it’s credit availability, it’s many, [MASK] factors.</t>
+          <t>More broadly, however, weaker demand, especially in [MASK] that have [MASK] most affected by the pandemic, has held down consumer [MASK], and overall, inflation is running well below [MASK] 2 [MASK] longer-run objective.</t>
         </is>
       </c>
       <c r="B687" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="C687" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D687" t="n">
-        <v>309</v>
+        <v>167</v>
       </c>
       <c r="E687" t="n">
         <v>1</v>
@@ -16915,17 +16915,17 @@
     <row r="688">
       <c r="A688" t="inlineStr">
         <is>
-          <t>More broadly, however, weaker demand, especially in [MASK] that have [MASK] most affected by the pandemic, has held down consumer [MASK], and overall, inflation is running well below [MASK] 2 [MASK] longer-run objective.</t>
+          <t>Our mandate, [MASK], is price inflation.</t>
         </is>
       </c>
       <c r="B688" t="n">
-        <v>2014</v>
+        <v>2021</v>
       </c>
       <c r="C688" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D688" t="n">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="E688" t="n">
         <v>1</v>
@@ -16939,17 +16939,17 @@
     <row r="689">
       <c r="A689" t="inlineStr">
         <is>
-          <t>Our mandate, [MASK], is price inflation.</t>
+          <t>So on the first, the Committee’s forecasts and [MASK] of most outside forecasters do show growth running below its longer-[MASK] potential this year [MASK] next [MASK].</t>
         </is>
       </c>
       <c r="B689" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C689" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D689" t="n">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="E689" t="n">
         <v>1</v>
@@ -16963,17 +16963,17 @@
     <row r="690">
       <c r="A690" t="inlineStr">
         <is>
-          <t>So on the first, the Committee’s forecasts and [MASK] of most outside forecasters do show growth running below its longer-[MASK] potential this year [MASK] next [MASK].</t>
+          <t>So the—the sooner [MASK] get the virus under control, the sooner [MASK] [MASK] regain that confidence and regain their economic activity.</t>
         </is>
       </c>
       <c r="B690" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C690" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D690" t="n">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="E690" t="n">
         <v>1</v>
@@ -16987,17 +16987,17 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>So the—the sooner [MASK] get the virus under control, the sooner [MASK] [MASK] regain that confidence and regain their economic activity.</t>
+          <t>[MASK] you have seen a shift this time in most participants’ [MASK] of the appropriate path for policy, and, as I tried to indicate, I [MASK] that [MASK] reflects a somewhat slower projected path [MASK] global growth—[MASK] [MASK] in the global economy outside the [MASK] States—and for some tightening in credit conditions in [MASK] form of an increase in spreads.</t>
         </is>
       </c>
       <c r="B691" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C691" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D691" t="n">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="E691" t="n">
         <v>1</v>
@@ -17011,17 +17011,17 @@
     <row r="692">
       <c r="A692" t="inlineStr">
         <is>
-          <t>[MASK] you have seen a shift this time in most participants’ [MASK] of the appropriate path for policy, and, as I tried to indicate, I [MASK] that [MASK] reflects a somewhat slower projected path [MASK] global growth—[MASK] [MASK] in the global economy outside the [MASK] States—and for some tightening in credit conditions in [MASK] form of an increase in spreads.</t>
+          <t>[MASK] we’d like to [MASK] that in the form of a [MASK] of declining monthly inflation readings—that’[MASK] what we’re looking for.</t>
         </is>
       </c>
       <c r="B692" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="C692" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D692" t="n">
-        <v>212</v>
+        <v>43</v>
       </c>
       <c r="E692" t="n">
         <v>1</v>
@@ -17035,17 +17035,17 @@
     <row r="693">
       <c r="A693" t="inlineStr">
         <is>
-          <t>[MASK] we’d like to [MASK] that in the form of a [MASK] of declining monthly inflation readings—that’[MASK] what we’re looking for.</t>
+          <t>I don’t really think asset prices themselves [MASK] a significant threat to financial [MASK], and that’s because households [MASK] in good shape [MASK] than they have been.</t>
         </is>
       </c>
       <c r="B693" t="n">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="C693" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D693" t="n">
-        <v>43</v>
+        <v>109</v>
       </c>
       <c r="E693" t="n">
         <v>1</v>
@@ -17059,17 +17059,17 @@
     <row r="694">
       <c r="A694" t="inlineStr">
         <is>
-          <t>I don’t really think asset prices themselves [MASK] a significant threat to financial [MASK], and that’s because households [MASK] in good shape [MASK] than they have been.</t>
+          <t>But also [MASK] want to see inflation move up back to our 2 percent objective over the medium term, and so [MASK] above-trend growth and continuing tightness—greater tightness in labor and product markets—[MASK] think that [MASK] help [MASK] achieve our objective as [MASK] with respect to [MASK].</t>
         </is>
       </c>
       <c r="B694" t="n">
-        <v>2013</v>
+        <v>2018</v>
       </c>
       <c r="C694" t="n">
         <v>0</v>
       </c>
       <c r="D694" t="n">
-        <v>109</v>
+        <v>76</v>
       </c>
       <c r="E694" t="n">
         <v>1</v>
@@ -17083,17 +17083,17 @@
     <row r="695">
       <c r="A695" t="inlineStr">
         <is>
-          <t>But also [MASK] want to see inflation move up back to our 2 percent objective over the medium term, and so [MASK] above-trend growth and continuing tightness—greater tightness in labor and product markets—[MASK] think that [MASK] help [MASK] achieve our objective as [MASK] with respect to [MASK].</t>
+          <t>As a further [MASK] in enhancing the clarity of [MASK] communications, the Committee recently [MASK] to begin publishing information [MASK] participants’ assessments of appropriate monetary policy—that [MASK], the path of policy that each participant judges as most [MASK] to foster mandate-consistent outcomes for employment and inflation if [MASK] economy [MASK] as expected.</t>
         </is>
       </c>
       <c r="B695" t="n">
         <v>2018</v>
       </c>
       <c r="C695" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D695" t="n">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="E695" t="n">
         <v>1</v>
@@ -17107,17 +17107,17 @@
     <row r="696">
       <c r="A696" t="inlineStr">
         <is>
-          <t>As a further [MASK] in enhancing the clarity of [MASK] communications, the Committee recently [MASK] to begin publishing information [MASK] participants’ assessments of appropriate monetary policy—that [MASK], the path of policy that each participant judges as most [MASK] to foster mandate-consistent outcomes for employment and inflation if [MASK] economy [MASK] as expected.</t>
+          <t>[MASK] we do say that risks to the financial system—we [MASK] in our longer-run statement [MASK] goals [MASK] monetary policy [MASK] that risks to the financial system that could prevent us from achieving [MASK] goals are something that we [MASK] take into consideration.</t>
         </is>
       </c>
       <c r="B696" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="C696" t="n">
         <v>2</v>
       </c>
       <c r="D696" t="n">
-        <v>62</v>
+        <v>209</v>
       </c>
       <c r="E696" t="n">
         <v>1</v>
@@ -17131,17 +17131,17 @@
     <row r="697">
       <c r="A697" t="inlineStr">
         <is>
-          <t>[MASK] we do say that risks to the financial system—we [MASK] in our longer-run statement [MASK] goals [MASK] monetary policy [MASK] that risks to the financial system that could prevent us from achieving [MASK] goals are something that we [MASK] take into consideration.</t>
+          <t>[MASK], while I do not shirk the responsibility of [MASK] Fed [MASK] to [MASK] what it can to meet its mandate, obviously, a broad range [MASK] policies can affect growth and [MASK], and I hope [MASK] there [MASK] be a range of actions that will complement and supplement the Federal Reserve’s efforts.</t>
         </is>
       </c>
       <c r="B697" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C697" t="n">
         <v>2</v>
       </c>
       <c r="D697" t="n">
-        <v>209</v>
+        <v>4</v>
       </c>
       <c r="E697" t="n">
         <v>1</v>
@@ -17155,17 +17155,17 @@
     <row r="698">
       <c r="A698" t="inlineStr">
         <is>
-          <t>[MASK], while I do not shirk the responsibility of [MASK] Fed [MASK] to [MASK] what it can to meet its mandate, obviously, a broad range [MASK] policies can affect growth and [MASK], and I hope [MASK] there [MASK] be a range of actions that will complement and supplement the Federal Reserve’s efforts.</t>
+          <t>And inflation is well [MASK] target.</t>
         </is>
       </c>
       <c r="B698" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C698" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D698" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E698" t="n">
         <v>1</v>
@@ -17179,17 +17179,17 @@
     <row r="699">
       <c r="A699" t="inlineStr">
         <is>
-          <t>And inflation is well [MASK] target.</t>
+          <t>By contrast, raising rates too slowly would raise the risk that monetary policy would [MASK] to [MASK] abruptly down the road, which could jeopardize the [MASK] [MASK].</t>
         </is>
       </c>
       <c r="B699" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C699" t="n">
         <v>1</v>
       </c>
       <c r="D699" t="n">
-        <v>21</v>
+        <v>94</v>
       </c>
       <c r="E699" t="n">
         <v>1</v>
@@ -17203,17 +17203,17 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>By contrast, raising rates too slowly would raise the risk that monetary policy would [MASK] to [MASK] abruptly down the road, which could jeopardize the [MASK] [MASK].</t>
+          <t>Inflation has moved up in [MASK] months, mainly reflecting higher [MASK] for some commodities [MASK] imported goods.</t>
         </is>
       </c>
       <c r="B700" t="n">
-        <v>2022</v>
+        <v>2012</v>
       </c>
       <c r="C700" t="n">
         <v>1</v>
       </c>
       <c r="D700" t="n">
-        <v>94</v>
+        <v>143</v>
       </c>
       <c r="E700" t="n">
         <v>1</v>
@@ -17227,17 +17227,17 @@
     <row r="701">
       <c r="A701" t="inlineStr">
         <is>
-          <t>Inflation has moved up in [MASK] months, mainly reflecting higher [MASK] for some commodities [MASK] imported goods.</t>
+          <t>Again, that’s not a forecast, [MASK]’ve made a hypothesis, which [MASK] imply [MASK] improvement in unemployment.</t>
         </is>
       </c>
       <c r="B701" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="C701" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D701" t="n">
-        <v>143</v>
+        <v>3</v>
       </c>
       <c r="E701" t="n">
         <v>1</v>
@@ -17251,17 +17251,17 @@
     <row r="702">
       <c r="A702" t="inlineStr">
         <is>
-          <t>Again, that’s not a forecast, [MASK]’ve made a hypothesis, which [MASK] imply [MASK] improvement in unemployment.</t>
+          <t>So I think, through all [MASK] those channels, [MASK] policy works.</t>
         </is>
       </c>
       <c r="B702" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C702" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D702" t="n">
-        <v>3</v>
+        <v>187</v>
       </c>
       <c r="E702" t="n">
         <v>1</v>
@@ -17275,17 +17275,17 @@
     <row r="703">
       <c r="A703" t="inlineStr">
         <is>
-          <t>So I think, through all [MASK] those channels, [MASK] policy works.</t>
+          <t>But you do see [MASK] in services, so you—this [MASK] around the world [MASK] Chair Powell’s Press Conference FINAL weak manufacturing</t>
         </is>
       </c>
       <c r="B703" t="n">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="C703" t="n">
         <v>2</v>
       </c>
       <c r="D703" t="n">
-        <v>187</v>
+        <v>88</v>
       </c>
       <c r="E703" t="n">
         <v>1</v>
@@ -17299,17 +17299,17 @@
     <row r="704">
       <c r="A704" t="inlineStr">
         <is>
-          <t>But you do see [MASK] in services, so you—this [MASK] around the world [MASK] Chair Powell’s Press Conference FINAL weak manufacturing</t>
+          <t>But many other commodity prices have fallen further, and the reason I [MASK] give for [MASK] [MASK] that the emerging markets—China, the [MASK] of Asia, [MASK] some [MASK] parts of the world—plus Europe, of course, are [MASK], and so global commodity demand is weaker.</t>
         </is>
       </c>
       <c r="B704" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="C704" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D704" t="n">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E704" t="n">
         <v>1</v>
@@ -17323,17 +17323,17 @@
     <row r="705">
       <c r="A705" t="inlineStr">
         <is>
-          <t>But many other commodity prices have fallen further, and the reason I [MASK] give for [MASK] [MASK] that the emerging markets—China, the [MASK] of Asia, [MASK] some [MASK] parts of the world—plus Europe, of course, are [MASK], and so global commodity demand is weaker.</t>
+          <t>Everyone, particularly people on fixed [MASK], [MASK] at the lower part of the income distribution are better off with [MASK] prices.</t>
         </is>
       </c>
       <c r="B705" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C705" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D705" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="E705" t="n">
         <v>1</v>
@@ -17347,17 +17347,17 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>Everyone, particularly people on fixed [MASK], [MASK] at the lower part of the income distribution are better off with [MASK] prices.</t>
+          <t>The [MASK] of [MASK] into, into inflation over time is just not there.</t>
         </is>
       </c>
       <c r="B706" t="n">
         <v>2021</v>
       </c>
       <c r="C706" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D706" t="n">
-        <v>100</v>
+        <v>249</v>
       </c>
       <c r="E706" t="n">
         <v>1</v>
@@ -17371,7 +17371,7 @@
     <row r="707">
       <c r="A707" t="inlineStr">
         <is>
-          <t>The [MASK] of [MASK] into, into inflation over time is just not there.</t>
+          <t>The housing sector [MASK] fully recovered from the downturn, supported in [MASK] by low [MASK] interest rates.</t>
         </is>
       </c>
       <c r="B707" t="n">
@@ -17381,7 +17381,7 @@
         <v>0</v>
       </c>
       <c r="D707" t="n">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E707" t="n">
         <v>1</v>
@@ -17395,7 +17395,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>The housing sector [MASK] fully recovered from the downturn, supported in [MASK] by low [MASK] interest rates.</t>
+          <t>Now, we [MASK]—[MASK] know, we haven’t anticipated that slowdown in [MASK], and that’s one of the main reasons [MASK] we haven’t anticipated the relatively slow growth.</t>
         </is>
       </c>
       <c r="B708" t="n">
@@ -17405,7 +17405,7 @@
         <v>0</v>
       </c>
       <c r="D708" t="n">
-        <v>246</v>
+        <v>170</v>
       </c>
       <c r="E708" t="n">
         <v>1</v>
@@ -17419,17 +17419,17 @@
     <row r="709">
       <c r="A709" t="inlineStr">
         <is>
-          <t>Now, we [MASK]—[MASK] know, we haven’t anticipated that slowdown in [MASK], and that’s one of the main reasons [MASK] we haven’t anticipated the relatively slow growth.</t>
+          <t>And, you know, we do want [MASK] to run moderately above 2 [MASK].</t>
         </is>
       </c>
       <c r="B709" t="n">
-        <v>2021</v>
+        <v>2011</v>
       </c>
       <c r="C709" t="n">
         <v>0</v>
       </c>
       <c r="D709" t="n">
-        <v>170</v>
+        <v>57</v>
       </c>
       <c r="E709" t="n">
         <v>1</v>
@@ -17443,17 +17443,17 @@
     <row r="710">
       <c r="A710" t="inlineStr">
         <is>
-          <t>And, you know, we do want [MASK] to run moderately above 2 [MASK].</t>
+          <t>And obviously [MASK] are benefits from a strong economy to every household in the economy, including savers, from having a better job [MASK] and [MASK] more [MASK] economy.</t>
         </is>
       </c>
       <c r="B710" t="n">
         <v>2011</v>
       </c>
       <c r="C710" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D710" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E710" t="n">
         <v>1</v>
@@ -17467,17 +17467,17 @@
     <row r="711">
       <c r="A711" t="inlineStr">
         <is>
-          <t>And obviously [MASK] are benefits from a strong economy to every household in the economy, including savers, from having a better job [MASK] and [MASK] more [MASK] economy.</t>
+          <t>I’m just saying, [MASK], that is what fiscal policy [MASK] do that, really, monetary [MASK] can’t [MASK]—is, is invest in [MASK] future productive capacity of the economy, raise potential growth.</t>
         </is>
       </c>
       <c r="B711" t="n">
-        <v>2011</v>
+        <v>2020</v>
       </c>
       <c r="C711" t="n">
         <v>2</v>
       </c>
       <c r="D711" t="n">
-        <v>26</v>
+        <v>158</v>
       </c>
       <c r="E711" t="n">
         <v>1</v>
@@ -17491,17 +17491,17 @@
     <row r="712">
       <c r="A712" t="inlineStr">
         <is>
-          <t>I’m just saying, [MASK], that is what fiscal policy [MASK] do that, really, monetary [MASK] can’t [MASK]—is, is invest in [MASK] future productive capacity of the economy, raise potential growth.</t>
+          <t>Wage growth is not—there are many [MASK] that [MASK] it—it’[MASK] not definitive in any sense in determining our policy,</t>
         </is>
       </c>
       <c r="B712" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C712" t="n">
         <v>2</v>
       </c>
       <c r="D712" t="n">
-        <v>158</v>
+        <v>267</v>
       </c>
       <c r="E712" t="n">
         <v>1</v>
@@ -17515,17 +17515,17 @@
     <row r="713">
       <c r="A713" t="inlineStr">
         <is>
-          <t>Wage growth is not—there are many [MASK] that [MASK] it—it’[MASK] not definitive in any sense in determining our policy,</t>
+          <t>We are quite aware that [MASK] low interest rates, particularly for a protracted period, [MASK] have costs for a lot [MASK] people.</t>
         </is>
       </c>
       <c r="B713" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C713" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D713" t="n">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="E713" t="n">
         <v>1</v>
@@ -17539,17 +17539,17 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>We are quite aware that [MASK] low interest rates, particularly for a protracted period, [MASK] have costs for a lot [MASK] people.</t>
+          <t>Well, we—[MASK] a [MASK], we do not desire inflation undershoots.</t>
         </is>
       </c>
       <c r="B714" t="n">
         <v>2020</v>
       </c>
       <c r="C714" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D714" t="n">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="E714" t="n">
         <v>1</v>
@@ -17563,17 +17563,17 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Well, we—[MASK] a [MASK], we do not desire inflation undershoots.</t>
+          <t>The Committee will continue to pay close [MASK] to the evolution [MASK] inflation and inflation expectations.</t>
         </is>
       </c>
       <c r="B715" t="n">
-        <v>2020</v>
+        <v>2016</v>
       </c>
       <c r="C715" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D715" t="n">
-        <v>294</v>
+        <v>233</v>
       </c>
       <c r="E715" t="n">
         <v>1</v>
@@ -17587,17 +17587,17 @@
     <row r="716">
       <c r="A716" t="inlineStr">
         <is>
-          <t>The Committee will continue to pay close [MASK] to the evolution [MASK] inflation and inflation expectations.</t>
+          <t>But there’s also a role for monetary [MASK].</t>
         </is>
       </c>
       <c r="B716" t="n">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="C716" t="n">
         <v>2</v>
       </c>
       <c r="D716" t="n">
-        <v>233</v>
+        <v>85</v>
       </c>
       <c r="E716" t="n">
         <v>1</v>
@@ -17611,46 +17611,22 @@
     <row r="717">
       <c r="A717" t="inlineStr">
         <is>
-          <t>But there’s also a role for monetary [MASK].</t>
+          <t>And [MASK], what [MASK] statement emphasizes, and this is [MASK] same language we used in December and [MASK], we used the language [MASK] if inflation is running below our 2 percent objective.</t>
         </is>
       </c>
       <c r="B717" t="n">
-        <v>2014</v>
+        <v>2017</v>
       </c>
       <c r="C717" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D717" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="E717" t="n">
         <v>1</v>
       </c>
       <c r="F717" t="inlineStr">
-        <is>
-          <t>masking</t>
-        </is>
-      </c>
-    </row>
-    <row r="718">
-      <c r="A718" t="inlineStr">
-        <is>
-          <t>And [MASK], what [MASK] statement emphasizes, and this is [MASK] same language we used in December and [MASK], we used the language [MASK] if inflation is running below our 2 percent objective.</t>
-        </is>
-      </c>
-      <c r="B718" t="n">
-        <v>2017</v>
-      </c>
-      <c r="C718" t="n">
-        <v>0</v>
-      </c>
-      <c r="D718" t="n">
-        <v>40</v>
-      </c>
-      <c r="E718" t="n">
-        <v>1</v>
-      </c>
-      <c r="F718" t="inlineStr">
         <is>
           <t>masking</t>
         </is>

</xml_diff>

<commit_message>
Revert augmented datasets to previous versions (deduped sets pushed prematurely)
</commit_message>
<xml_diff>
--- a/dataset/test-and-training/augmented_data/augmented_train_data/lab-manual-pc-split-train-944601.xlsx
+++ b/dataset/test-and-training/augmented_data/augmented_train_data/lab-manual-pc-split-train-944601.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F717"/>
+  <dimension ref="A1:F718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12211,17 +12211,17 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>These measures, together with our strong interest rate guidelines and our balance sheet, will ensure that monetary policy continues to support the economy until the full recovery.</t>
+          <t>. . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . . .</t>
         </is>
       </c>
       <c r="B492" t="n">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="C492" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D492" t="n">
-        <v>263</v>
+        <v>88</v>
       </c>
       <c r="E492" t="n">
         <v>1</v>
@@ -12235,17 +12235,17 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>So this time you saw a shift in most participants, assessing the appropriate way for policy, and, as I tried to show, I think that largely reflects a somewhat slower projected way for global growth – for growth in the world economy outside the United States – and for a certain tightening of credit conditions in the form of an increase in spreads.</t>
+          <t>These measures, together with our strong interest rate guidelines and our balance sheet, will ensure that monetary policy continues to support the economy until the full recovery.</t>
         </is>
       </c>
       <c r="B493" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="C493" t="n">
         <v>0</v>
       </c>
       <c r="D493" t="n">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="E493" t="n">
         <v>1</v>
@@ -12259,17 +12259,17 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>The persistence that this brings into inflation over time is simply not there.</t>
+          <t>So this time you saw a shift in most participants, assessing the appropriate way for policy, and, as I tried to show, I think that largely reflects a somewhat slower projected way for global growth – for growth in the world economy outside the United States – and for a certain tightening of credit conditions in the form of an increase in spreads.</t>
         </is>
       </c>
       <c r="B494" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C494" t="n">
         <v>0</v>
       </c>
       <c r="D494" t="n">
-        <v>249</v>
+        <v>212</v>
       </c>
       <c r="E494" t="n">
         <v>1</v>
@@ -12283,17 +12283,17 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>In fact, it is already – I think it is already understood – that there is more – although we are at 31⁄2 percent unemployment, there is actually more slackening out there, in a way.</t>
+          <t>The persistence that this brings into inflation over time is simply not there.</t>
         </is>
       </c>
       <c r="B495" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C495" t="n">
         <v>0</v>
       </c>
       <c r="D495" t="n">
-        <v>134</v>
+        <v>249</v>
       </c>
       <c r="E495" t="n">
         <v>1</v>
@@ -12307,17 +12307,17 @@
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>Inflation is also slowed down, due to weaker demand and significantly lower energy prices.</t>
+          <t>In fact, it is already – I think it is already understood – that there is more – although we are at 31⁄2 percent unemployment, there is actually more slackening out there, in a way.</t>
         </is>
       </c>
       <c r="B496" t="n">
-        <v>2012</v>
+        <v>2022</v>
       </c>
       <c r="C496" t="n">
         <v>0</v>
       </c>
       <c r="D496" t="n">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="E496" t="n">
         <v>1</v>
@@ -12331,7 +12331,7 @@
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>Recent lower inflation measurements have been driven significantly by the seemingly one-off price reductions of certain price categories such as wireless telephone services and prescription medicines.</t>
+          <t>Inflation is also slowed down, due to weaker demand and significantly lower energy prices.</t>
         </is>
       </c>
       <c r="B497" t="n">
@@ -12341,7 +12341,7 @@
         <v>0</v>
       </c>
       <c r="D497" t="n">
-        <v>251</v>
+        <v>144</v>
       </c>
       <c r="E497" t="n">
         <v>1</v>
@@ -12355,17 +12355,17 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>But you have not been under the merely negative scenario that has been followed by an inflation shock followed by a rapid rise in short-term interest rates.</t>
+          <t>Recent lower inflation measurements have been driven significantly by the seemingly one-off price reductions of certain price categories such as wireless telephone services and prescription medicines.</t>
         </is>
       </c>
       <c r="B498" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="C498" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D498" t="n">
-        <v>87</v>
+        <v>251</v>
       </c>
       <c r="E498" t="n">
         <v>1</v>
@@ -12379,17 +12379,17 @@
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>Well, we've been expecting a long time, as most analysts have, to see some slowdown in Chinese growth over time, how they're balancing their economy.</t>
+          <t>But you have not been under the merely negative scenario that has been followed by an inflation shock followed by a rapid rise in short-term interest rates.</t>
         </is>
       </c>
       <c r="B499" t="n">
-        <v>2021</v>
+        <v>2014</v>
       </c>
       <c r="C499" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D499" t="n">
-        <v>171</v>
+        <v>87</v>
       </c>
       <c r="E499" t="n">
         <v>1</v>
@@ -12403,17 +12403,17 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>And, I think, all of us – those who have this expectation and that if the economy continues to move as we expected and we continue to consider the risks to be balanced – consider it appropriate to gradually eliminate the existing arrangements by several interest rate hikes this year.</t>
+          <t>Well, we've been expecting a long time, as most analysts have, to see some slowdown in Chinese growth over time, how they're balancing their economy.</t>
         </is>
       </c>
       <c r="B500" t="n">
-        <v>2015</v>
+        <v>2021</v>
       </c>
       <c r="C500" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D500" t="n">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E500" t="n">
         <v>1</v>
@@ -12427,17 +12427,17 @@
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>So you know, as I said, that the Committee feels strongly committed to ensuring that we restore price stability and are determined to use its instruments to do so.</t>
+          <t>And, I think, all of us – those who have this expectation and that if the economy continues to move as we expected and we continue to consider the risks to be balanced – consider it appropriate to gradually eliminate the existing arrangements by several interest rate hikes this year.</t>
         </is>
       </c>
       <c r="B501" t="n">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="C501" t="n">
         <v>1</v>
       </c>
       <c r="D501" t="n">
-        <v>224</v>
+        <v>53</v>
       </c>
       <c r="E501" t="n">
         <v>1</v>
@@ -12451,17 +12451,17 @@
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>Inflation has continued to fall below our longer-term target, largely due to the lower energy prices I have mentioned.</t>
+          <t>So you know, as I said, that the Committee feels strongly committed to ensuring that we restore price stability and are determined to use its instruments to do so.</t>
         </is>
       </c>
       <c r="B502" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="C502" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D502" t="n">
-        <v>142</v>
+        <v>224</v>
       </c>
       <c r="E502" t="n">
         <v>1</v>
@@ -12475,17 +12475,17 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>This will not happen without restoring price stability.</t>
+          <t>Inflation has continued to fall below our longer-term target, largely due to the lower energy prices I have mentioned.</t>
         </is>
       </c>
       <c r="B503" t="n">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="C503" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D503" t="n">
-        <v>230</v>
+        <v>142</v>
       </c>
       <c r="E503" t="n">
         <v>1</v>
@@ -12499,17 +12499,17 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>Given the increasing uncertainty and the restrained inflationary pressure, we now stress that the Committee will closely monitor the impact of the in-depth information on economic prospects and, where appropriate, support expansion with a strong labour market and inflation close to its 2% target.</t>
+          <t>This will not happen without restoring price stability.</t>
         </is>
       </c>
       <c r="B504" t="n">
-        <v>2013</v>
+        <v>2016</v>
       </c>
       <c r="C504" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D504" t="n">
-        <v>135</v>
+        <v>230</v>
       </c>
       <c r="E504" t="n">
         <v>1</v>
@@ -12523,17 +12523,17 @@
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>I'm just saying that, that's what fiscal policy can do, that really, monetary policy can't do – is to invest in the future production capacity of the economy, increase potential growth.</t>
+          <t>Given the increasing uncertainty and the restrained inflationary pressure, we now stress that the Committee will closely monitor the impact of the in-depth information on economic prospects and, where appropriate, support expansion with a strong labour market and inflation close to its 2% target.</t>
         </is>
       </c>
       <c r="B505" t="n">
-        <v>2020</v>
+        <v>2013</v>
       </c>
       <c r="C505" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D505" t="n">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="E505" t="n">
         <v>1</v>
@@ -12547,17 +12547,17 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>We have further analysed the impact of interest rate changes, for example on decisions such as investments or car purchases.</t>
+          <t>I'm just saying that, that's what fiscal policy can do, that really, monetary policy can't do – is to invest in the future production capacity of the economy, increase potential growth.</t>
         </is>
       </c>
       <c r="B506" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C506" t="n">
         <v>2</v>
       </c>
       <c r="D506" t="n">
-        <v>46</v>
+        <v>158</v>
       </c>
       <c r="E506" t="n">
         <v>1</v>
@@ -12571,7 +12571,7 @@
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>And the maximum level of employment consistent with price stability is developing over time within a business cycle and over a longer period of time, partly reflecting the evolution of the factors affecting labour supply, including those related to the pandemic.</t>
+          <t>We have further analysed the impact of interest rate changes, for example on decisions such as investments or car purchases.</t>
         </is>
       </c>
       <c r="B507" t="n">
@@ -12581,7 +12581,7 @@
         <v>2</v>
       </c>
       <c r="D507" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E507" t="n">
         <v>1</v>
@@ -12595,17 +12595,17 @@
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>However, I would like to stress that we are committed to raising inflation to 2%.</t>
+          <t>And the maximum level of employment consistent with price stability is developing over time within a business cycle and over a longer period of time, partly reflecting the evolution of the factors affecting labour supply, including those related to the pandemic.</t>
         </is>
       </c>
       <c r="B508" t="n">
-        <v>2011</v>
+        <v>2022</v>
       </c>
       <c r="C508" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D508" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="E508" t="n">
         <v>1</v>
@@ -12619,17 +12619,17 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>So let me talk about the Coronavirus, and then I will focus more generally on global growth.</t>
+          <t>However, I would like to stress that we are committed to raising inflation to 2%.</t>
         </is>
       </c>
       <c r="B509" t="n">
-        <v>2019</v>
+        <v>2011</v>
       </c>
       <c r="C509" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D509" t="n">
-        <v>196</v>
+        <v>73</v>
       </c>
       <c r="E509" t="n">
         <v>1</v>
@@ -12643,17 +12643,17 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>And inflation is far above the target.</t>
+          <t>So let me talk about the Coronavirus, and then I will focus more generally on global growth.</t>
         </is>
       </c>
       <c r="B510" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C510" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D510" t="n">
-        <v>21</v>
+        <v>196</v>
       </c>
       <c r="E510" t="n">
         <v>1</v>
@@ -12667,17 +12667,17 @@
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>And we learn to engage in economic activity.</t>
+          <t>And inflation is far above the target.</t>
         </is>
       </c>
       <c r="B511" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="C511" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D511" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="E511" t="n">
         <v>1</v>
@@ -12691,17 +12691,17 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>In any case, it is our job to ensure price stability, and I think that price stability can be imagined as an advantage that will bring great benefits to society over a long period of time.</t>
+          <t>And we learn to engage in economic activity.</t>
         </is>
       </c>
       <c r="B512" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="C512" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D512" t="n">
-        <v>132</v>
+        <v>44</v>
       </c>
       <c r="E512" t="n">
         <v>1</v>
@@ -12715,17 +12715,17 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>So it is a serious economic problem for the United States, but it has the causes that are not related to monetary policy or to our response to the pandemic.</t>
+          <t>In any case, it is our job to ensure price stability, and I think that price stability can be imagined as an advantage that will bring great benefits to society over a long period of time.</t>
         </is>
       </c>
       <c r="B513" t="n">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="C513" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D513" t="n">
-        <v>194</v>
+        <v>132</v>
       </c>
       <c r="E513" t="n">
         <v>1</v>
@@ -12739,17 +12739,17 @@
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>On the other hand, the unemployment rate in September 2020, as measured by this metric, would have increased in the 1920s in April in the last 20's.</t>
+          <t>So it is a serious economic problem for the United States, but it has the causes that are not related to monetary policy or to our response to the pandemic.</t>
         </is>
       </c>
       <c r="B514" t="n">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="C514" t="n">
         <v>2</v>
       </c>
       <c r="D514" t="n">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="E514" t="n">
         <v>1</v>
@@ -12763,41 +12763,41 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>We’re not seeing evidence in labor markets of very substantial downward pressures on labor that could signify extreme shortages of labor that could propel inflation lower in a very rapid way, and inflation is still operating below our objective.</t>
+          <t>On the other hand, the unemployment rate in September 2020, as measured by this metric, would have increased in the 1920s in April in the last 20's.</t>
         </is>
       </c>
       <c r="B515" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C515" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D515" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="E515" t="n">
         <v>1</v>
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>directional_swap</t>
+          <t>back_translation</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>I think the—you know, in a way, the least soft aspect of it is, is looking at the unemployment rate, which is still below our median estimate of, of [the unemployment rate consistent with] maximum employment.</t>
+          <t>We’re not seeing evidence in labor markets of very substantial downward pressures on labor that could signify extreme shortages of labor that could propel inflation lower in a very rapid way, and inflation is still operating below our objective.</t>
         </is>
       </c>
       <c r="B516" t="n">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="C516" t="n">
         <v>1</v>
       </c>
       <c r="D516" t="n">
-        <v>117</v>
+        <v>299</v>
       </c>
       <c r="E516" t="n">
         <v>1</v>
@@ -12811,17 +12811,17 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>But I want to emphasize that we do have a commitment to cutting inflation to 2 percent.</t>
+          <t>I think the—you know, in a way, the least soft aspect of it is, is looking at the unemployment rate, which is still below our median estimate of, of [the unemployment rate consistent with] maximum employment.</t>
         </is>
       </c>
       <c r="B517" t="n">
-        <v>2011</v>
+        <v>2015</v>
       </c>
       <c r="C517" t="n">
         <v>1</v>
       </c>
       <c r="D517" t="n">
-        <v>73</v>
+        <v>117</v>
       </c>
       <c r="E517" t="n">
         <v>1</v>
@@ -12835,17 +12835,17 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>The central tendency of the unemployment rate projections is slightly higher than in the March projections and now stands at 6.0 to 6.1 percent at the end of this year.</t>
+          <t>But I want to emphasize that we do have a commitment to cutting inflation to 2 percent.</t>
         </is>
       </c>
       <c r="B518" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C518" t="n">
         <v>1</v>
       </c>
       <c r="D518" t="n">
-        <v>241</v>
+        <v>73</v>
       </c>
       <c r="E518" t="n">
         <v>1</v>
@@ -12859,17 +12859,17 @@
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>And I think, more broadly, monetary policy is also supporting household spending and home buying by keeping the labor market weak, keeping workers’ incomes falling, and keeping consumer confidence at low levels, where it currently is.</t>
+          <t>The central tendency of the unemployment rate projections is slightly higher than in the March projections and now stands at 6.0 to 6.1 percent at the end of this year.</t>
         </is>
       </c>
       <c r="B519" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="C519" t="n">
         <v>1</v>
       </c>
       <c r="D519" t="n">
-        <v>12</v>
+        <v>241</v>
       </c>
       <c r="E519" t="n">
         <v>1</v>
@@ -12883,7 +12883,7 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>So, if we maintain a highly restrictive monetary policy for a very long time from here and the economy performs as we expect—namely, it’s weak and the risks that are out there don’t materialize—my concern will be that we will have much more easing in labor markets than you see in these projections.</t>
+          <t>And I think, more broadly, monetary policy is also supporting household spending and home buying by keeping the labor market weak, keeping workers’ incomes falling, and keeping consumer confidence at low levels, where it currently is.</t>
         </is>
       </c>
       <c r="B520" t="n">
@@ -12893,7 +12893,7 @@
         <v>1</v>
       </c>
       <c r="D520" t="n">
-        <v>219</v>
+        <v>12</v>
       </c>
       <c r="E520" t="n">
         <v>1</v>
@@ -12907,17 +12907,17 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>More broadly, however, stronger demand, especially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run objective.</t>
+          <t>So, if we maintain a highly restrictive monetary policy for a very long time from here and the economy performs as we expect—namely, it’s weak and the risks that are out there don’t materialize—my concern will be that we will have much more easing in labor markets than you see in these projections.</t>
         </is>
       </c>
       <c r="B521" t="n">
-        <v>2014</v>
+        <v>2019</v>
       </c>
       <c r="C521" t="n">
         <v>1</v>
       </c>
       <c r="D521" t="n">
-        <v>167</v>
+        <v>219</v>
       </c>
       <c r="E521" t="n">
         <v>1</v>
@@ -12931,17 +12931,17 @@
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>In fact, it’s already—it’s already understood, I think, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more tightness out there, in a sense.</t>
+          <t>More broadly, however, stronger demand, especially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run objective.</t>
         </is>
       </c>
       <c r="B522" t="n">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="C522" t="n">
         <v>1</v>
       </c>
       <c r="D522" t="n">
-        <v>134</v>
+        <v>167</v>
       </c>
       <c r="E522" t="n">
         <v>1</v>
@@ -12955,17 +12955,17 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>Inflation pressures remain muted, and indicators of longer-term inflation expectations are at the higher end of their historic ranges.</t>
+          <t>In fact, it’s already—it’s already understood, I think, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more tightness out there, in a sense.</t>
         </is>
       </c>
       <c r="B523" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="C523" t="n">
         <v>1</v>
       </c>
       <c r="D523" t="n">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="E523" t="n">
         <v>1</v>
@@ -12979,17 +12979,17 @@
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>If we think that the potential growth rate of the economy is somewhere between, somewhere around 1.75 percent, 2.8 percent is weak economic growth.</t>
+          <t>Inflation pressures remain muted, and indicators of longer-term inflation expectations are at the higher end of their historic ranges.</t>
         </is>
       </c>
       <c r="B524" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C524" t="n">
         <v>1</v>
       </c>
       <c r="D524" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="E524" t="n">
         <v>1</v>
@@ -13003,7 +13003,7 @@
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>Now, with inflation below 2 percent, I think it’s appropriate that the labor market be that soft.</t>
+          <t>If we think that the potential growth rate of the economy is somewhere between, somewhere around 1.75 percent, 2.8 percent is weak economic growth.</t>
         </is>
       </c>
       <c r="B525" t="n">
@@ -13013,7 +13013,7 @@
         <v>1</v>
       </c>
       <c r="D525" t="n">
-        <v>172</v>
+        <v>125</v>
       </c>
       <c r="E525" t="n">
         <v>1</v>
@@ -13027,7 +13027,7 @@
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>So those who can get credit, together with the high prices of houses, are at—able to buy much more house than they could have a few years ago.</t>
+          <t>Now, with inflation below 2 percent, I think it’s appropriate that the labor market be that soft.</t>
         </is>
       </c>
       <c r="B526" t="n">
@@ -13037,7 +13037,7 @@
         <v>1</v>
       </c>
       <c r="D526" t="n">
-        <v>207</v>
+        <v>172</v>
       </c>
       <c r="E526" t="n">
         <v>1</v>
@@ -13051,17 +13051,17 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>We think that the economy will need highly restrictive monetary policy and the use of our tools for an extended period.</t>
+          <t>So those who can get credit, together with the high prices of houses, are at—able to buy much more house than they could have a few years ago.</t>
         </is>
       </c>
       <c r="B527" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C527" t="n">
         <v>1</v>
       </c>
       <c r="D527" t="n">
-        <v>286</v>
+        <v>207</v>
       </c>
       <c r="E527" t="n">
         <v>1</v>
@@ -13075,17 +13075,17 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>Inflation has declined further below our longer-run objective, largely reflecting the higher energy prices I just mentioned.</t>
+          <t>We think that the economy will need highly restrictive monetary policy and the use of our tools for an extended period.</t>
         </is>
       </c>
       <c r="B528" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="C528" t="n">
         <v>1</v>
       </c>
       <c r="D528" t="n">
-        <v>142</v>
+        <v>286</v>
       </c>
       <c r="E528" t="n">
         <v>1</v>
@@ -13099,17 +13099,17 @@
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>So you have seen a shift this time in most participants’ assessments of the appropriate path for policy, and, as I tried to indicate, I think that largely reflects a somewhat slower projected path for global growth—for growth in the global economy outside the United States—and for some easing in credit conditions in the form of an decrease in spreads.</t>
+          <t>Inflation has declined further below our longer-run objective, largely reflecting the higher energy prices I just mentioned.</t>
         </is>
       </c>
       <c r="B529" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="C529" t="n">
         <v>1</v>
       </c>
       <c r="D529" t="n">
-        <v>212</v>
+        <v>142</v>
       </c>
       <c r="E529" t="n">
         <v>1</v>
@@ -13123,17 +13123,17 @@
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>As was highlighted by the Bureau of Labor Statistics, this figure likely understates the extent of unemployment; accounting for the unusually large number of workers who reported themselves as employed but absent from their jobs would cut the unemployment rate by about 3 percentage points.</t>
+          <t>So you have seen a shift this time in most participants’ assessments of the appropriate path for policy, and, as I tried to indicate, I think that largely reflects a somewhat slower projected path for global growth—for growth in the global economy outside the United States—and for some easing in credit conditions in the form of an decrease in spreads.</t>
         </is>
       </c>
       <c r="B530" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="C530" t="n">
         <v>1</v>
       </c>
       <c r="D530" t="n">
-        <v>67</v>
+        <v>212</v>
       </c>
       <c r="E530" t="n">
         <v>1</v>
@@ -13147,17 +13147,17 @@
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>The central tendency falls to 2.4 to 2.7 percent next year, somewhat above estimates of the longer-run growth rate.</t>
+          <t>As was highlighted by the Bureau of Labor Statistics, this figure likely understates the extent of unemployment; accounting for the unusually large number of workers who reported themselves as employed but absent from their jobs would cut the unemployment rate by about 3 percentage points.</t>
         </is>
       </c>
       <c r="B531" t="n">
-        <v>2012</v>
+        <v>2017</v>
       </c>
       <c r="C531" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D531" t="n">
-        <v>242</v>
+        <v>67</v>
       </c>
       <c r="E531" t="n">
         <v>1</v>
@@ -13171,7 +13171,7 @@
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>The asset purchases are about creating some near-term momentum in the economy, trying to strengthen growth and job creation in the near term, and the decreases in the federal funds rate target, when they ultimately occur, are about reducing accommodation.</t>
+          <t>The central tendency falls to 2.4 to 2.7 percent next year, somewhat above estimates of the longer-run growth rate.</t>
         </is>
       </c>
       <c r="B532" t="n">
@@ -13181,7 +13181,7 @@
         <v>0</v>
       </c>
       <c r="D532" t="n">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E532" t="n">
         <v>1</v>
@@ -13195,17 +13195,17 @@
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>But I think that that’s a prudent move, to move in a gradual way to remove Chair Yellen’s Press Conference FINAL accommodation, with unemployment now—and not only, I should say, the unemployment rate, but I think any indicator of labor market performance and slack that you could look at, whether it’s household perceptions of the availability of jobs, difficulty that firms report in hiring workers, the rate at which workers are quitting their jobs, the rate of job openings, all of these indicators do signal a soft labor market.</t>
+          <t>The asset purchases are about creating some near-term momentum in the economy, trying to strengthen growth and job creation in the near term, and the decreases in the federal funds rate target, when they ultimately occur, are about reducing accommodation.</t>
         </is>
       </c>
       <c r="B533" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C533" t="n">
         <v>0</v>
       </c>
       <c r="D533" t="n">
-        <v>72</v>
+        <v>240</v>
       </c>
       <c r="E533" t="n">
         <v>1</v>
@@ -13219,17 +13219,17 @@
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>After precipitous drops in March and April, employment fell strongly in May and June as many people returned to work from temporary layoffs.</t>
+          <t>But I think that that’s a prudent move, to move in a gradual way to remove Chair Yellen’s Press Conference FINAL accommodation, with unemployment now—and not only, I should say, the unemployment rate, but I think any indicator of labor market performance and slack that you could look at, whether it’s household perceptions of the availability of jobs, difficulty that firms report in hiring workers, the rate at which workers are quitting their jobs, the rate of job openings, all of these indicators do signal a soft labor market.</t>
         </is>
       </c>
       <c r="B534" t="n">
-        <v>2019</v>
+        <v>2011</v>
       </c>
       <c r="C534" t="n">
         <v>0</v>
       </c>
       <c r="D534" t="n">
-        <v>2</v>
+        <v>72</v>
       </c>
       <c r="E534" t="n">
         <v>1</v>
@@ -13243,17 +13243,17 @@
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>Against this backdrop, today the Federal Open Market Committee cut its policy interest rate by ¾ percentage point and anticipates that ongoing decreases in that rate will be appropriate.</t>
+          <t>After precipitous drops in March and April, employment fell strongly in May and June as many people returned to work from temporary layoffs.</t>
         </is>
       </c>
       <c r="B535" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="C535" t="n">
         <v>0</v>
       </c>
       <c r="D535" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E535" t="n">
         <v>1</v>
@@ -13267,17 +13267,17 @@
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>And, as I think all of us—having that expectation and that if the economy continued to progress along the lines that we expected and we continued to see the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate decreases this year.</t>
+          <t>Against this backdrop, today the Federal Open Market Committee cut its policy interest rate by ¾ percentage point and anticipates that ongoing decreases in that rate will be appropriate.</t>
         </is>
       </c>
       <c r="B536" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="C536" t="n">
         <v>0</v>
       </c>
       <c r="D536" t="n">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="E536" t="n">
         <v>1</v>
@@ -13291,17 +13291,17 @@
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>The jobs picture continues to be weak, with the unemployment rate near historic lows and with weaker wage gains.</t>
+          <t>And, as I think all of us—having that expectation and that if the economy continued to progress along the lines that we expected and we continued to see the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate decreases this year.</t>
         </is>
       </c>
       <c r="B537" t="n">
-        <v>2021</v>
+        <v>2015</v>
       </c>
       <c r="C537" t="n">
         <v>0</v>
       </c>
       <c r="D537" t="n">
-        <v>247</v>
+        <v>53</v>
       </c>
       <c r="E537" t="n">
         <v>1</v>
@@ -13315,17 +13315,17 @@
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>Business and household spending are decreasing at rates consistent with moderate economic growth, though household spending appears to be falling at a somewhat slower pace than earlier this year.</t>
+          <t>The jobs picture continues to be weak, with the unemployment rate near historic lows and with weaker wage gains.</t>
         </is>
       </c>
       <c r="B538" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="C538" t="n">
         <v>0</v>
       </c>
       <c r="D538" t="n">
-        <v>70</v>
+        <v>247</v>
       </c>
       <c r="E538" t="n">
         <v>1</v>
@@ -13339,17 +13339,17 @@
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>And that, I think, does cut, cut the risk that low inflation will be more persistent.</t>
+          <t>Business and household spending are decreasing at rates consistent with moderate economic growth, though household spending appears to be falling at a somewhat slower pace than earlier this year.</t>
         </is>
       </c>
       <c r="B539" t="n">
-        <v>2022</v>
+        <v>2011</v>
       </c>
       <c r="C539" t="n">
         <v>0</v>
       </c>
       <c r="D539" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="E539" t="n">
         <v>1</v>
@@ -13363,17 +13363,17 @@
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can cut interest rates at the appropriate time, even if the balance sheet remains large for an extended period.</t>
+          <t>And that, I think, does cut, cut the risk that low inflation will be more persistent.</t>
         </is>
       </c>
       <c r="B540" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C540" t="n">
         <v>0</v>
       </c>
       <c r="D540" t="n">
-        <v>188</v>
+        <v>35</v>
       </c>
       <c r="E540" t="n">
         <v>1</v>
@@ -13387,41 +13387,41 @@
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>In fact, it’s already—it’s already empathize, I recall, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more slack out there, in a sense.</t>
+          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can cut interest rates at the appropriate time, even if the balance sheet remains large for an extended period.</t>
         </is>
       </c>
       <c r="B541" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C541" t="n">
         <v>0</v>
       </c>
       <c r="D541" t="n">
-        <v>134</v>
+        <v>188</v>
       </c>
       <c r="E541" t="n">
         <v>1</v>
       </c>
       <c r="F541" t="inlineStr">
         <is>
-          <t>synonym_replacement</t>
+          <t>directional_swap</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>And so you’re seeing prices are moving back up remove their lows there.</t>
+          <t>In fact, it’s already—it’s already empathize, I recall, that—that there’s more—even though we’re at 3½ percent unemployment, there’s actually more slack out there, in a sense.</t>
         </is>
       </c>
       <c r="B542" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C542" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D542" t="n">
-        <v>33</v>
+        <v>134</v>
       </c>
       <c r="E542" t="n">
         <v>1</v>
@@ -13435,17 +13435,17 @@
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>The shock that the—from the pandemic was unprecedented both in its nature and in its sizing and in the amount of unemployment that it created and in the shock to economic action.</t>
+          <t>And so you’re seeing prices are moving back up remove their lows there.</t>
         </is>
       </c>
       <c r="B543" t="n">
-        <v>2012</v>
+        <v>2020</v>
       </c>
       <c r="C543" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D543" t="n">
-        <v>253</v>
+        <v>33</v>
       </c>
       <c r="E543" t="n">
         <v>1</v>
@@ -13459,17 +13459,17 @@
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>Inflation has moved up in recent months, mainly reflecting higher prices for some commodity and imported goods.</t>
+          <t>The shock that the—from the pandemic was unprecedented both in its nature and in its sizing and in the amount of unemployment that it created and in the shock to economic action.</t>
         </is>
       </c>
       <c r="B544" t="n">
         <v>2012</v>
       </c>
       <c r="C544" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D544" t="n">
-        <v>143</v>
+        <v>253</v>
       </c>
       <c r="E544" t="n">
         <v>1</v>
@@ -13483,17 +13483,17 @@
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>And, in particular, I do personally conceive that the slowdown is at least partly temporary, and that we’ll see peachy growth going forward.</t>
+          <t>Inflation has moved up in recent months, mainly reflecting higher prices for some commodity and imported goods.</t>
         </is>
       </c>
       <c r="B545" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C545" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D545" t="n">
-        <v>56</v>
+        <v>143</v>
       </c>
       <c r="E545" t="n">
         <v>1</v>
@@ -13507,7 +13507,7 @@
     <row r="546">
       <c r="A546" t="inlineStr">
         <is>
-          <t>But I want to emphasize that we do have a commitment to raising inflation to 2 pct.</t>
+          <t>And, in particular, I do personally conceive that the slowdown is at least partly temporary, and that we’ll see peachy growth going forward.</t>
         </is>
       </c>
       <c r="B546" t="n">
@@ -13517,7 +13517,7 @@
         <v>0</v>
       </c>
       <c r="D546" t="n">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="E546" t="n">
         <v>1</v>
@@ -13531,17 +13531,17 @@
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>The central tendency rises to 2.4 to 2.7 pct next year, somewhat above estimates of the longer-course growth rate.</t>
+          <t>But I want to emphasize that we do have a commitment to raising inflation to 2 pct.</t>
         </is>
       </c>
       <c r="B547" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C547" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D547" t="n">
-        <v>242</v>
+        <v>73</v>
       </c>
       <c r="E547" t="n">
         <v>1</v>
@@ -13555,17 +13555,17 @@
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>I think we all agree that the economy is stool progress, that we are close to an unemployment rate that is one that’s sustainable in the farseeing run.</t>
+          <t>The central tendency rises to 2.4 to 2.7 pct next year, somewhat above estimates of the longer-course growth rate.</t>
         </is>
       </c>
       <c r="B548" t="n">
-        <v>2015</v>
+        <v>2012</v>
       </c>
       <c r="C548" t="n">
         <v>1</v>
       </c>
       <c r="D548" t="n">
-        <v>118</v>
+        <v>242</v>
       </c>
       <c r="E548" t="n">
         <v>1</v>
@@ -13579,17 +13579,17 @@
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>Monetary policy has a role, and it really is in, you know—our original role was providing liquidity to financial systems when they’re under stress, and that’s—that’s very part of what we did nowadays.</t>
+          <t>I think we all agree that the economy is stool progress, that we are close to an unemployment rate that is one that’s sustainable in the farseeing run.</t>
         </is>
       </c>
       <c r="B549" t="n">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="C549" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D549" t="n">
-        <v>165</v>
+        <v>118</v>
       </c>
       <c r="E549" t="n">
         <v>1</v>
@@ -13603,17 +13603,17 @@
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>And inflation is moving—moving up, I think, toward our 2 percent accusative.</t>
+          <t>Monetary policy has a role, and it really is in, you know—our original role was providing liquidity to financial systems when they’re under stress, and that’s—that’s very part of what we did nowadays.</t>
         </is>
       </c>
       <c r="B550" t="n">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="C550" t="n">
         <v>0</v>
       </c>
       <c r="D550" t="n">
-        <v>20</v>
+        <v>165</v>
       </c>
       <c r="E550" t="n">
         <v>1</v>
@@ -13627,17 +13627,17 @@
     <row r="551">
       <c r="A551" t="inlineStr">
         <is>
-          <t>The housing sector has fully recovered from the downturn, supported in parting by low mortgage interest rates.</t>
+          <t>And inflation is moving—moving up, I think, toward our 2 percent accusative.</t>
         </is>
       </c>
       <c r="B551" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C551" t="n">
         <v>0</v>
       </c>
       <c r="D551" t="n">
-        <v>246</v>
+        <v>20</v>
       </c>
       <c r="E551" t="n">
         <v>1</v>
@@ -13651,17 +13651,17 @@
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>By getting unemployment down, we hope to bring endorse to work some of the people who’ve been extinct of work as long as they have and, in that respect, try to avoid the longer-term consequences of multitude being out of work for months at a time.</t>
+          <t>The housing sector has fully recovered from the downturn, supported in parting by low mortgage interest rates.</t>
         </is>
       </c>
       <c r="B552" t="n">
-        <v>2017</v>
+        <v>2021</v>
       </c>
       <c r="C552" t="n">
         <v>0</v>
       </c>
       <c r="D552" t="n">
-        <v>95</v>
+        <v>246</v>
       </c>
       <c r="E552" t="n">
         <v>1</v>
@@ -13675,17 +13675,17 @@
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t>Swell, we—as a Committee, we do not desire inflation undershoots.</t>
+          <t>By getting unemployment down, we hope to bring endorse to work some of the people who’ve been extinct of work as long as they have and, in that respect, try to avoid the longer-term consequences of multitude being out of work for months at a time.</t>
         </is>
       </c>
       <c r="B553" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C553" t="n">
         <v>0</v>
       </c>
       <c r="D553" t="n">
-        <v>294</v>
+        <v>95</v>
       </c>
       <c r="E553" t="n">
         <v>1</v>
@@ -13699,17 +13699,17 @@
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>And, and those are—that’s again—that goes to keeping this episode as short as it can be and avoiding unnecessary business bankruptcy, unnecessary household bankruptcies, and unnecessary long-condition stays of unemployment or supporting people done them so that they can maintain their financial footing and their lives and be able to go back to work in a productive path.</t>
+          <t>Swell, we—as a Committee, we do not desire inflation undershoots.</t>
         </is>
       </c>
       <c r="B554" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="C554" t="n">
         <v>0</v>
       </c>
       <c r="D554" t="n">
-        <v>52</v>
+        <v>294</v>
       </c>
       <c r="E554" t="n">
         <v>1</v>
@@ -13723,17 +13723,17 @@
     <row r="555">
       <c r="A555" t="inlineStr">
         <is>
-          <t>And part of that just is the effect of lower worry rates.</t>
+          <t>And, and those are—that’s again—that goes to keeping this episode as short as it can be and avoiding unnecessary business bankruptcy, unnecessary household bankruptcies, and unnecessary long-condition stays of unemployment or supporting people done them so that they can maintain their financial footing and their lives and be able to go back to work in a productive path.</t>
         </is>
       </c>
       <c r="B555" t="n">
-        <v>2011</v>
+        <v>2015</v>
       </c>
       <c r="C555" t="n">
         <v>0</v>
       </c>
       <c r="D555" t="n">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="E555" t="n">
         <v>1</v>
@@ -13747,17 +13747,17 @@
     <row r="556">
       <c r="A556" t="inlineStr">
         <is>
-          <t>And what we—it looks care we’re seeing a slowdown in the rate of growth.</t>
+          <t>And part of that just is the effect of lower worry rates.</t>
         </is>
       </c>
       <c r="B556" t="n">
-        <v>2022</v>
+        <v>2011</v>
       </c>
       <c r="C556" t="n">
         <v>0</v>
       </c>
       <c r="D556" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E556" t="n">
         <v>1</v>
@@ -13771,17 +13771,17 @@
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>The asset purchases are about creating some near-term momentum in the saving, trying to strengthen growth and job creation in the good term, and the increases in the federal funds rate target, when they ultimately occur, are about reduction accommodation.</t>
+          <t>And what we—it looks care we’re seeing a slowdown in the rate of growth.</t>
         </is>
       </c>
       <c r="B557" t="n">
-        <v>2012</v>
+        <v>2022</v>
       </c>
       <c r="C557" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D557" t="n">
-        <v>240</v>
+        <v>48</v>
       </c>
       <c r="E557" t="n">
         <v>1</v>
@@ -13795,17 +13795,17 @@
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>where unemployment continue to fall at a gradual pace as it has been since last September—and we have made some progress since last Sept</t>
+          <t>The asset purchases are about creating some near-term momentum in the saving, trying to strengthen growth and job creation in the good term, and the increases in the federal funds rate target, when they ultimately occur, are about reduction accommodation.</t>
         </is>
       </c>
       <c r="B558" t="n">
-        <v>2018</v>
+        <v>2012</v>
       </c>
       <c r="C558" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D558" t="n">
-        <v>75</v>
+        <v>240</v>
       </c>
       <c r="E558" t="n">
         <v>1</v>
@@ -13819,17 +13819,17 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>And that, I think, does raise, raise the risk that high inflation will be more haunting.</t>
+          <t>where unemployment continue to fall at a gradual pace as it has been since last September—and we have made some progress since last Sept</t>
         </is>
       </c>
       <c r="B559" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="C559" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D559" t="n">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="E559" t="n">
         <v>1</v>
@@ -13843,17 +13843,17 @@
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>Well, our policy approach doesn’t involve deliberately trying to raise inflation.</t>
+          <t>And that, I think, does raise, raise the risk that high inflation will be more haunting.</t>
         </is>
       </c>
       <c r="B560" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C560" t="n">
         <v>1</v>
       </c>
       <c r="D560" t="n">
-        <v>292</v>
+        <v>35</v>
       </c>
       <c r="E560" t="n">
         <v>1</v>
@@ -13867,17 +13867,17 @@
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>We have Chair Yellen’s Press Conference CONCLUDING households who are becoming more comfortable with their debt levels and more capable to service that debt, an improving job market.</t>
+          <t>Well, our policy approach doesn’t involve deliberately trying to raise inflation.</t>
         </is>
       </c>
       <c r="B561" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="C561" t="n">
         <v>1</v>
       </c>
       <c r="D561" t="n">
-        <v>277</v>
+        <v>292</v>
       </c>
       <c r="E561" t="n">
         <v>1</v>
@@ -13891,17 +13891,17 @@
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
-          <t>So on the first, the Committee’s forecasts and those of most outside forecasters do show growth persist below its longer-run potential this year and future year.</t>
+          <t>We have Chair Yellen’s Press Conference CONCLUDING households who are becoming more comfortable with their debt levels and more capable to service that debt, an improving job market.</t>
         </is>
       </c>
       <c r="B562" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="C562" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D562" t="n">
-        <v>198</v>
+        <v>277</v>
       </c>
       <c r="E562" t="n">
         <v>1</v>
@@ -13915,17 +13915,17 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>And I really don’t have much for you other than to say that they will be data dependent—that, over time, the stance of policy will be adjusted to try to keep the economy on a track where we see continuing advance toward reach our destination of maximum employment and price stability.</t>
+          <t>So on the first, the Committee’s forecasts and those of most outside forecasters do show growth persist below its longer-run potential this year and future year.</t>
         </is>
       </c>
       <c r="B563" t="n">
         <v>2019</v>
       </c>
       <c r="C563" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D563" t="n">
-        <v>11</v>
+        <v>198</v>
       </c>
       <c r="E563" t="n">
         <v>1</v>
@@ -13939,17 +13939,17 @@
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>Inflation has declined further below our yearner-feed objective, largely reflecting the lower energy prices I just mentioned.</t>
+          <t>And I really don’t have much for you other than to say that they will be data dependent—that, over time, the stance of policy will be adjusted to try to keep the economy on a track where we see continuing advance toward reach our destination of maximum employment and price stability.</t>
         </is>
       </c>
       <c r="B564" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="C564" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D564" t="n">
-        <v>142</v>
+        <v>11</v>
       </c>
       <c r="E564" t="n">
         <v>1</v>
@@ -13963,17 +13963,17 @@
     <row r="565">
       <c r="A565" t="inlineStr">
         <is>
-          <t>So we want to see that levelheaded process unfold as we decide what the true state of the economy is, and we think it will germinate in a way that will mean lower inflation.</t>
+          <t>Inflation has declined further below our yearner-feed objective, largely reflecting the lower energy prices I just mentioned.</t>
         </is>
       </c>
       <c r="B565" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="C565" t="n">
         <v>0</v>
       </c>
       <c r="D565" t="n">
-        <v>211</v>
+        <v>142</v>
       </c>
       <c r="E565" t="n">
         <v>1</v>
@@ -13987,17 +13987,17 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>An circumstantially sharp increase in wages or inflation could tell you that you’re reaching those points.</t>
+          <t>So we want to see that levelheaded process unfold as we decide what the true state of the economy is, and we think it will germinate in a way that will mean lower inflation.</t>
         </is>
       </c>
       <c r="B566" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="C566" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D566" t="n">
-        <v>7</v>
+        <v>211</v>
       </c>
       <c r="E566" t="n">
         <v>1</v>
@@ -14011,17 +14011,17 @@
     <row r="567">
       <c r="A567" t="inlineStr">
         <is>
-          <t>Now, we’ve long await, as most analysts have, to see some slowing in Formosan growth over time as they rebalance their economy.</t>
+          <t>An circumstantially sharp increase in wages or inflation could tell you that you’re reaching those points.</t>
         </is>
       </c>
       <c r="B567" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C567" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D567" t="n">
-        <v>171</v>
+        <v>7</v>
       </c>
       <c r="E567" t="n">
         <v>1</v>
@@ -14035,17 +14035,17 @@
     <row r="568">
       <c r="A568" t="inlineStr">
         <is>
-          <t>And I think, more broadly, monetary policy is also supporting household expenditure and home buying by keeping the labor commercialise strong, keeping worker’ incomes rising, and keeping consumer confidence at high levels, where it currently is.</t>
+          <t>Now, we’ve long await, as most analysts have, to see some slowing in Formosan growth over time as they rebalance their economy.</t>
         </is>
       </c>
       <c r="B568" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C568" t="n">
         <v>0</v>
       </c>
       <c r="D568" t="n">
-        <v>12</v>
+        <v>171</v>
       </c>
       <c r="E568" t="n">
         <v>1</v>
@@ -14059,17 +14059,17 @@
     <row r="569">
       <c r="A569" t="inlineStr">
         <is>
-          <t>But many other commodity prices have fallen further, and the reason I would collapse for that is that the emerging markets—China, the balance of Asia, and some other parts of the world—plus Europe, of course, are softer, and so globular commodity demand is weaker.</t>
+          <t>And I think, more broadly, monetary policy is also supporting household expenditure and home buying by keeping the labor commercialise strong, keeping worker’ incomes rising, and keeping consumer confidence at high levels, where it currently is.</t>
         </is>
       </c>
       <c r="B569" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C569" t="n">
         <v>0</v>
       </c>
       <c r="D569" t="n">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="E569" t="n">
         <v>1</v>
@@ -14083,17 +14083,17 @@
     <row r="570">
       <c r="A570" t="inlineStr">
         <is>
-          <t>If you look at the number of job orifice compared to the number of unemployed, it’s—we’re, we’re clearly on a path to a very strong labor market with high involvement, low unemployment, high employment, wages moving up across the spectrum.</t>
+          <t>But many other commodity prices have fallen further, and the reason I would collapse for that is that the emerging markets—China, the balance of Asia, and some other parts of the world—plus Europe, of course, are softer, and so globular commodity demand is weaker.</t>
         </is>
       </c>
       <c r="B570" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C570" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D570" t="n">
-        <v>129</v>
+        <v>81</v>
       </c>
       <c r="E570" t="n">
         <v>1</v>
@@ -14107,7 +14107,7 @@
     <row r="571">
       <c r="A571" t="inlineStr">
         <is>
-          <t>Our role, though, is also to, you know, to make sure that—that maximum employment happen in a context of price constancy and financial stability, which is why we’re gradually raising rates.</t>
+          <t>If you look at the number of job orifice compared to the number of unemployed, it’s—we’re, we’re clearly on a path to a very strong labor market with high involvement, low unemployment, high employment, wages moving up across the spectrum.</t>
         </is>
       </c>
       <c r="B571" t="n">
@@ -14117,7 +14117,7 @@
         <v>1</v>
       </c>
       <c r="D571" t="n">
-        <v>179</v>
+        <v>129</v>
       </c>
       <c r="E571" t="n">
         <v>1</v>
@@ -14131,17 +14131,17 @@
     <row r="572">
       <c r="A572" t="inlineStr">
         <is>
-          <t>And the room I would explain it is, is that inflation that’s too low will mean that interest rates are lower.</t>
+          <t>Our role, though, is also to, you know, to make sure that—that maximum employment happen in a context of price constancy and financial stability, which is why we’re gradually raising rates.</t>
         </is>
       </c>
       <c r="B572" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C572" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D572" t="n">
-        <v>38</v>
+        <v>179</v>
       </c>
       <c r="E572" t="n">
         <v>1</v>
@@ -14155,17 +14155,17 @@
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>So those who can get credit, unitedly with the low prices of houses, are at—able to buy much more house than they could have a few yr ago.</t>
+          <t>And the room I would explain it is, is that inflation that’s too low will mean that interest rates are lower.</t>
         </is>
       </c>
       <c r="B573" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C573" t="n">
         <v>0</v>
       </c>
       <c r="D573" t="n">
-        <v>207</v>
+        <v>38</v>
       </c>
       <c r="E573" t="n">
         <v>1</v>
@@ -14179,17 +14179,17 @@
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>Our authorization, sorry, is price inflation.</t>
+          <t>So those who can get credit, unitedly with the low prices of houses, are at—able to buy much more house than they could have a few yr ago.</t>
         </is>
       </c>
       <c r="B574" t="n">
         <v>2021</v>
       </c>
       <c r="C574" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D574" t="n">
-        <v>178</v>
+        <v>207</v>
       </c>
       <c r="E574" t="n">
         <v>1</v>
@@ -14203,17 +14203,17 @@
     <row r="575">
       <c r="A575" t="inlineStr">
         <is>
-          <t>And we’d like to find that in the form of a series of declining monthly inflation readings—that’s what we’re looking for.</t>
+          <t>Our authorization, sorry, is price inflation.</t>
         </is>
       </c>
       <c r="B575" t="n">
-        <v>2017</v>
+        <v>2021</v>
       </c>
       <c r="C575" t="n">
         <v>1</v>
       </c>
       <c r="D575" t="n">
-        <v>43</v>
+        <v>178</v>
       </c>
       <c r="E575" t="n">
         <v>1</v>
@@ -14227,17 +14227,17 @@
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t>So in—in—in U-6, the U-6 charge of unemployment has tripled from 7 percent to 21 percent.</t>
+          <t>And we’d like to find that in the form of a series of declining monthly inflation readings—that’s what we’re looking for.</t>
         </is>
       </c>
       <c r="B576" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="C576" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D576" t="n">
-        <v>192</v>
+        <v>43</v>
       </c>
       <c r="E576" t="n">
         <v>1</v>
@@ -14251,17 +14251,17 @@
     <row r="577">
       <c r="A577" t="inlineStr">
         <is>
-          <t>I mean, it really depends on how long it takes for wages and, more than that, prices to come polish for inflation to come down.</t>
+          <t>So in—in—in U-6, the U-6 charge of unemployment has tripled from 7 percent to 21 percent.</t>
         </is>
       </c>
       <c r="B577" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C577" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D577" t="n">
-        <v>114</v>
+        <v>192</v>
       </c>
       <c r="E577" t="n">
         <v>1</v>
@@ -14275,17 +14275,17 @@
     <row r="578">
       <c r="A578" t="inlineStr">
         <is>
-          <t>Earlier in the year, as you will all recall, after careful study over a menses of years, actually, the Committee announced the decision to enforce monetary policy in an ample-reserves regime.</t>
+          <t>I mean, it really depends on how long it takes for wages and, more than that, prices to come polish for inflation to come down.</t>
         </is>
       </c>
       <c r="B578" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="C578" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D578" t="n">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="E578" t="n">
         <v>1</v>
@@ -14299,17 +14299,17 @@
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
-          <t>But, I would say, boilersuit, we’re trying to prolong the expansion and keep, you know, close to our statutory goals, which are maximum employment and stable prices.</t>
+          <t>Earlier in the year, as you will all recall, after careful study over a menses of years, actually, the Committee announced the decision to enforce monetary policy in an ample-reserves regime.</t>
         </is>
       </c>
       <c r="B579" t="n">
-        <v>2014</v>
+        <v>2017</v>
       </c>
       <c r="C579" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D579" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="E579" t="n">
         <v>1</v>
@@ -14323,17 +14323,17 @@
     <row r="580">
       <c r="A580" t="inlineStr">
         <is>
-          <t>The “extended period” language is conditioned on just those same points: “Extended period” is conditioned on imagination slack, on subdued inflation, and on stable inflation expectations.</t>
+          <t>But, I would say, boilersuit, we’re trying to prolong the expansion and keep, you know, close to our statutory goals, which are maximum employment and stable prices.</t>
         </is>
       </c>
       <c r="B580" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="C580" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D580" t="n">
-        <v>256</v>
+        <v>89</v>
       </c>
       <c r="E580" t="n">
         <v>1</v>
@@ -14347,17 +14347,17 @@
     <row r="581">
       <c r="A581" t="inlineStr">
         <is>
-          <t>That said, many of my colleagues and I would see a portion of the slump in the unemployment rate as perhaps not representing a diminution of slack in the labor marketplace.</t>
+          <t>The “extended period” language is conditioned on just those same points: “Extended period” is conditioned on imagination slack, on subdued inflation, and on stable inflation expectations.</t>
         </is>
       </c>
       <c r="B581" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="C581" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D581" t="n">
-        <v>227</v>
+        <v>256</v>
       </c>
       <c r="E581" t="n">
         <v>1</v>
@@ -14371,17 +14371,17 @@
     <row r="582">
       <c r="A582" t="inlineStr">
         <is>
-          <t>And we were actually rather concerned that growth was not sufficient to continue to bring the unemployment rate down.</t>
+          <t>That said, many of my colleagues and I would see a portion of the slump in the unemployment rate as perhaps not representing a diminution of slack in the labor marketplace.</t>
         </is>
       </c>
       <c r="B582" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="C582" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D582" t="n">
-        <v>42</v>
+        <v>227</v>
       </c>
       <c r="E582" t="n">
         <v>1</v>
@@ -14395,17 +14395,17 @@
     <row r="583">
       <c r="A583" t="inlineStr">
         <is>
-          <t>These measures, along with our strong guidance on interest rates and on our equalizer sheet, will ensure that monetary policy will continue to support the economy until the recovery is thoroughgoing.</t>
+          <t>And we were actually rather concerned that growth was not sufficient to continue to bring the unemployment rate down.</t>
         </is>
       </c>
       <c r="B583" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="C583" t="n">
         <v>0</v>
       </c>
       <c r="D583" t="n">
-        <v>263</v>
+        <v>42</v>
       </c>
       <c r="E583" t="n">
         <v>1</v>
@@ -14419,17 +14419,17 @@
     <row r="584">
       <c r="A584" t="inlineStr">
         <is>
-          <t>Inflation pressures stay muted, and indicators of longer-term inflation expectations are at the lower end of their historical ranges.</t>
+          <t>These measures, along with our strong guidance on interest rates and on our equalizer sheet, will ensure that monetary policy will continue to support the economy until the recovery is thoroughgoing.</t>
         </is>
       </c>
       <c r="B584" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="C584" t="n">
         <v>0</v>
       </c>
       <c r="D584" t="n">
-        <v>145</v>
+        <v>263</v>
       </c>
       <c r="E584" t="n">
         <v>1</v>
@@ -14443,17 +14443,17 @@
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>And, as I think all of us—having that expectation and that if the saving extend to progress along the lines that we expected and we continued to escort the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate increases this year.</t>
+          <t>Inflation pressures stay muted, and indicators of longer-term inflation expectations are at the lower end of their historical ranges.</t>
         </is>
       </c>
       <c r="B585" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="C585" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D585" t="n">
-        <v>53</v>
+        <v>145</v>
       </c>
       <c r="E585" t="n">
         <v>1</v>
@@ -14467,17 +14467,17 @@
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>As always, our actions are guided by our congressional mandate to promote maximum employment and price stableness.</t>
+          <t>And, as I think all of us—having that expectation and that if the saving extend to progress along the lines that we expected and we continued to escort the risks as balanced—do regard it as appropriate to gradually remove accommodation that’s in place by having several interest rate increases this year.</t>
         </is>
       </c>
       <c r="B586" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="C586" t="n">
         <v>1</v>
       </c>
       <c r="D586" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="E586" t="n">
         <v>1</v>
@@ -14491,17 +14491,17 @@
     <row r="587">
       <c r="A587" t="inlineStr">
         <is>
-          <t>But I think that that’s a prudent move, to move in a gradual way to transfer Chair Yellen’s Crush Conference FINAL accommodation, with unemployment now—and not only, I should allege, the unemployment rate, but I think any indicator of labor market performance and tightness that you could look at, whether it’s household perceptions of the availableness of jobs, difficulty that firms describe in hiring workers, the rate at which workers are quitting their line, the rate of job openings, all of these indicators do signal a tight labor market.</t>
+          <t>As always, our actions are guided by our congressional mandate to promote maximum employment and price stableness.</t>
         </is>
       </c>
       <c r="B587" t="n">
-        <v>2011</v>
+        <v>2018</v>
       </c>
       <c r="C587" t="n">
         <v>1</v>
       </c>
       <c r="D587" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E587" t="n">
         <v>1</v>
@@ -14515,17 +14515,17 @@
     <row r="588">
       <c r="A588" t="inlineStr">
         <is>
-          <t>So unemployment has tended to go up much fast for minorities and for others who are—tend to be at the low end of the income spectrum.</t>
+          <t>But I think that that’s a prudent move, to move in a gradual way to transfer Chair Yellen’s Crush Conference FINAL accommodation, with unemployment now—and not only, I should allege, the unemployment rate, but I think any indicator of labor market performance and tightness that you could look at, whether it’s household perceptions of the availableness of jobs, difficulty that firms describe in hiring workers, the rate at which workers are quitting their line, the rate of job openings, all of these indicators do signal a tight labor market.</t>
         </is>
       </c>
       <c r="B588" t="n">
-        <v>2021</v>
+        <v>2011</v>
       </c>
       <c r="C588" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D588" t="n">
-        <v>208</v>
+        <v>72</v>
       </c>
       <c r="E588" t="n">
         <v>1</v>
@@ -14539,17 +14539,17 @@
     <row r="589">
       <c r="A589" t="inlineStr">
         <is>
-          <t>And you know, we haven’t yet—we just rival 2 percent core inflation, to selection one measure—just touched it for a few months, and then we’ve fallen back.</t>
+          <t>So unemployment has tended to go up much fast for minorities and for others who are—tend to be at the low end of the income spectrum.</t>
         </is>
       </c>
       <c r="B589" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C589" t="n">
         <v>0</v>
       </c>
       <c r="D589" t="n">
-        <v>49</v>
+        <v>208</v>
       </c>
       <c r="E589" t="n">
         <v>1</v>
@@ -14563,17 +14563,17 @@
     <row r="590">
       <c r="A590" t="inlineStr">
         <is>
-          <t>In any case, we, our task is to deliver price stability, and I think—you can think of price stability as an asset that just delivers large benefits to society over a long period of sentence.</t>
+          <t>And you know, we haven’t yet—we just rival 2 percent core inflation, to selection one measure—just touched it for a few months, and then we’ve fallen back.</t>
         </is>
       </c>
       <c r="B590" t="n">
         <v>2022</v>
       </c>
       <c r="C590" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D590" t="n">
-        <v>132</v>
+        <v>49</v>
       </c>
       <c r="E590" t="n">
         <v>1</v>
@@ -14587,17 +14587,17 @@
     <row r="591">
       <c r="A591" t="inlineStr">
         <is>
-          <t>That’s not going to happen without, without restoring price constancy.</t>
+          <t>In any case, we, our task is to deliver price stability, and I think—you can think of price stability as an asset that just delivers large benefits to society over a long period of sentence.</t>
         </is>
       </c>
       <c r="B591" t="n">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="C591" t="n">
         <v>1</v>
       </c>
       <c r="D591" t="n">
-        <v>230</v>
+        <v>132</v>
       </c>
       <c r="E591" t="n">
         <v>1</v>
@@ -14611,17 +14611,17 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>But in many country around the Chairperson Yellen’s Press Conference FINAL world that are important good exporters, the decline we’ve seen in oil prices has had a depressing effect on their growth, their trade with us and other trade partners, and caused problems that have had spillovers to the global thriftiness as well.</t>
+          <t>That’s not going to happen without, without restoring price constancy.</t>
         </is>
       </c>
       <c r="B592" t="n">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="C592" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D592" t="n">
-        <v>77</v>
+        <v>230</v>
       </c>
       <c r="E592" t="n">
         <v>1</v>
@@ -14635,17 +14635,17 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>More broadly, still, weaker demand, specially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run documentary.</t>
+          <t>But in many country around the Chairperson Yellen’s Press Conference FINAL world that are important good exporters, the decline we’ve seen in oil prices has had a depressing effect on their growth, their trade with us and other trade partners, and caused problems that have had spillovers to the global thriftiness as well.</t>
         </is>
       </c>
       <c r="B593" t="n">
-        <v>2014</v>
+        <v>2018</v>
       </c>
       <c r="C593" t="n">
         <v>0</v>
       </c>
       <c r="D593" t="n">
-        <v>167</v>
+        <v>77</v>
       </c>
       <c r="E593" t="n">
         <v>1</v>
@@ -14659,17 +14659,17 @@
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t>The American economy is very strong and well set to handle tighter monetary policy.</t>
+          <t>More broadly, still, weaker demand, specially in sectors that have been most affected by the pandemic, has held down consumer prices, and overall, inflation is running well below our 2 percent longer-run documentary.</t>
         </is>
       </c>
       <c r="B594" t="n">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="C594" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D594" t="n">
-        <v>232</v>
+        <v>167</v>
       </c>
       <c r="E594" t="n">
         <v>1</v>
@@ -14683,17 +14683,17 @@
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>The central tendency of the unemployment rate project is slightly lower than in the March projections and nowadays stands at 6.0 to 6.1 percent at the end of this year.</t>
+          <t>The American economy is very strong and well set to handle tighter monetary policy.</t>
         </is>
       </c>
       <c r="B595" t="n">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="C595" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D595" t="n">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="E595" t="n">
         <v>1</v>
@@ -14707,17 +14707,17 @@
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
-          <t>If we think that the potency growth rate of the economy is somewhere between, somewhere round 1.75 percent, 2.8 percent is strong economic growth.</t>
+          <t>The central tendency of the unemployment rate project is slightly lower than in the March projections and nowadays stands at 6.0 to 6.1 percent at the end of this year.</t>
         </is>
       </c>
       <c r="B596" t="n">
-        <v>2021</v>
+        <v>2012</v>
       </c>
       <c r="C596" t="n">
         <v>0</v>
       </c>
       <c r="D596" t="n">
-        <v>125</v>
+        <v>241</v>
       </c>
       <c r="E596" t="n">
         <v>1</v>
@@ -14731,17 +14731,17 @@
     <row r="597">
       <c r="A597" t="inlineStr">
         <is>
-          <t>Inflation has continued to run below our longer-run accusative, in part reflecting lower energy prices.</t>
+          <t>If we think that the potency growth rate of the economy is somewhere between, somewhere round 1.75 percent, 2.8 percent is strong economic growth.</t>
         </is>
       </c>
       <c r="B597" t="n">
-        <v>2012</v>
+        <v>2021</v>
       </c>
       <c r="C597" t="n">
         <v>0</v>
       </c>
       <c r="D597" t="n">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="E597" t="n">
         <v>1</v>
@@ -14755,17 +14755,17 @@
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>And, and that’s why we have adopted the flexible mediocre inflation-targeting framework.</t>
+          <t>Inflation has continued to run below our longer-run accusative, in part reflecting lower energy prices.</t>
         </is>
       </c>
       <c r="B598" t="n">
-        <v>2015</v>
+        <v>2012</v>
       </c>
       <c r="C598" t="n">
         <v>0</v>
       </c>
       <c r="D598" t="n">
-        <v>51</v>
+        <v>141</v>
       </c>
       <c r="E598" t="n">
         <v>1</v>
@@ -14779,17 +14779,17 @@
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>As I observe, monetary policy operates with lags, so, the policies we have in place, we suppose, will gradually—only gradually—move inflation back to 2 percent.</t>
+          <t>And, and that’s why we have adopted the flexible mediocre inflation-targeting framework.</t>
         </is>
       </c>
       <c r="B599" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="C599" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D599" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E599" t="n">
         <v>1</v>
@@ -14803,17 +14803,17 @@
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>As the factors restraining economical growth are projected to fade foster over time, the median rate rises to 3 percent by the end of 2018, close to its longer-run normal level.</t>
+          <t>As I observe, monetary policy operates with lags, so, the policies we have in place, we suppose, will gradually—only gradually—move inflation back to 2 percent.</t>
         </is>
       </c>
       <c r="B600" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="C600" t="n">
         <v>1</v>
       </c>
       <c r="D600" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E600" t="n">
         <v>1</v>
@@ -14827,17 +14827,17 @@
     <row r="601">
       <c r="A601" t="inlineStr">
         <is>
-          <t>And inflation is well above point.</t>
+          <t>As the factors restraining economical growth are projected to fade foster over time, the median rate rises to 3 percent by the end of 2018, close to its longer-run normal level.</t>
         </is>
       </c>
       <c r="B601" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C601" t="n">
         <v>1</v>
       </c>
       <c r="D601" t="n">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="E601" t="n">
         <v>1</v>
@@ -14851,17 +14851,17 @@
     <row r="602">
       <c r="A602" t="inlineStr">
         <is>
-          <t>I would say, in the orbit of commercial material estate, while valuations are high, we are seeing some tightening of lending standards and less debt growth associated with that rise in commercial real estate prices.</t>
+          <t>And inflation is well above point.</t>
         </is>
       </c>
       <c r="B602" t="n">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="C602" t="n">
         <v>1</v>
       </c>
       <c r="D602" t="n">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="E602" t="n">
         <v>1</v>
@@ -14875,17 +14875,17 @@
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>So, there has been impact through lower stake rates, but I think more broadly is the indirect effects.</t>
+          <t>I would say, in the orbit of commercial material estate, while valuations are high, we are seeing some tightening of lending standards and less debt growth associated with that rise in commercial real estate prices.</t>
         </is>
       </c>
       <c r="B603" t="n">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="C603" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D603" t="n">
-        <v>220</v>
+        <v>122</v>
       </c>
       <c r="E603" t="n">
         <v>1</v>
@@ -14899,17 +14899,17 @@
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>But, first, on inflation expectations, it is true that the breakevens from the inflation-adjusted—inflation-index bonds have come down.</t>
+          <t>So, there has been impact through lower stake rates, but I think more broadly is the indirect effects.</t>
         </is>
       </c>
       <c r="B604" t="n">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="C604" t="n">
         <v>0</v>
       </c>
       <c r="D604" t="n">
-        <v>91</v>
+        <v>220</v>
       </c>
       <c r="E604" t="n">
         <v>1</v>
@@ -14923,17 +14923,17 @@
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>In spite of having such slow growth, disappointing productivity growth, we have a labor market that last year return an mediocre of about 230,000 jobs a month and so far this class has been generating about 180,000 jobs a month.</t>
+          <t>But, first, on inflation expectations, it is true that the breakevens from the inflation-adjusted—inflation-index bonds have come down.</t>
         </is>
       </c>
       <c r="B605" t="n">
-        <v>2013</v>
+        <v>2022</v>
       </c>
       <c r="C605" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D605" t="n">
-        <v>138</v>
+        <v>91</v>
       </c>
       <c r="E605" t="n">
         <v>1</v>
@@ -14947,17 +14947,17 @@
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>By the direction, we’re also not at maximum employment, as I mentioned.</t>
+          <t>In spite of having such slow growth, disappointing productivity growth, we have a labor market that last year return an mediocre of about 230,000 jobs a month and so far this class has been generating about 180,000 jobs a month.</t>
         </is>
       </c>
       <c r="B606" t="n">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="C606" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D606" t="n">
-        <v>96</v>
+        <v>138</v>
       </c>
       <c r="E606" t="n">
         <v>1</v>
@@ -14971,17 +14971,17 @@
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>And if the stock theory of the portfolio is correct, which we believe it is, holding all of those securities murder of the market and reinvesting and still hold the, you know, rolling-over age securities, will still continue to put downward pressure on interest rates.</t>
+          <t>By the direction, we’re also not at maximum employment, as I mentioned.</t>
         </is>
       </c>
       <c r="B607" t="n">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="C607" t="n">
         <v>0</v>
       </c>
       <c r="D607" t="n">
-        <v>17</v>
+        <v>96</v>
       </c>
       <c r="E607" t="n">
         <v>1</v>
@@ -14995,17 +14995,17 @@
     <row r="608">
       <c r="A608" t="inlineStr">
         <is>
-          <t>And, you know, we do want inflation to extend moderately above 2 percent.</t>
+          <t>And if the stock theory of the portfolio is correct, which we believe it is, holding all of those securities murder of the market and reinvesting and still hold the, you know, rolling-over age securities, will still continue to put downward pressure on interest rates.</t>
         </is>
       </c>
       <c r="B608" t="n">
-        <v>2011</v>
+        <v>2013</v>
       </c>
       <c r="C608" t="n">
         <v>0</v>
       </c>
       <c r="D608" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="E608" t="n">
         <v>1</v>
@@ -15019,17 +15019,17 @@
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>For example, the unemployment rate has risen by 0.3 percentage points since March, and new arrogate for unemployment insurance have propel somewhat higher.</t>
+          <t>And, you know, we do want inflation to extend moderately above 2 percent.</t>
         </is>
       </c>
       <c r="B609" t="n">
-        <v>2021</v>
+        <v>2011</v>
       </c>
       <c r="C609" t="n">
         <v>0</v>
       </c>
       <c r="D609" t="n">
-        <v>103</v>
+        <v>57</v>
       </c>
       <c r="E609" t="n">
         <v>1</v>
@@ -15043,17 +15043,17 @@
     <row r="610">
       <c r="A610" t="inlineStr">
         <is>
-          <t>We’re not regard evidence in labor markets of very substantial upward pressure on labor that could signify extreme shortages of labor that could propel inflation higher in a very rapid way, and inflation is still operating below our objective.</t>
+          <t>For example, the unemployment rate has risen by 0.3 percentage points since March, and new arrogate for unemployment insurance have propel somewhat higher.</t>
         </is>
       </c>
       <c r="B610" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C610" t="n">
         <v>0</v>
       </c>
       <c r="D610" t="n">
-        <v>299</v>
+        <v>103</v>
       </c>
       <c r="E610" t="n">
         <v>1</v>
@@ -15067,17 +15067,17 @@
     <row r="611">
       <c r="A611" t="inlineStr">
         <is>
-          <t>And our plan as we do that is, as those purchases get to that level, we believe we can gradually reduce them, and we believe we can also gradually reduce repo as—as we range an plenteous level, as we’re satisfying demand now more from rudimentary reserves from peak purchases rather than from repo.</t>
+          <t>We’re not regard evidence in labor markets of very substantial upward pressure on labor that could signify extreme shortages of labor that could propel inflation higher in a very rapid way, and inflation is still operating below our objective.</t>
         </is>
       </c>
       <c r="B611" t="n">
-        <v>2011</v>
+        <v>2022</v>
       </c>
       <c r="C611" t="n">
         <v>0</v>
       </c>
       <c r="D611" t="n">
-        <v>28</v>
+        <v>299</v>
       </c>
       <c r="E611" t="n">
         <v>1</v>
@@ -15091,17 +15091,17 @@
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>The second point that I made was that when short-term interest rates hit zero, the tools of a central bank are no farsighted—are not exhausted, there are still other things that the exchange bank can do to create additional adjustment.</t>
+          <t>And our plan as we do that is, as those purchases get to that level, we believe we can gradually reduce them, and we believe we can also gradually reduce repo as—as we range an plenteous level, as we’re satisfying demand now more from rudimentary reserves from peak purchases rather than from repo.</t>
         </is>
       </c>
       <c r="B612" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C612" t="n">
         <v>0</v>
       </c>
       <c r="D612" t="n">
-        <v>252</v>
+        <v>28</v>
       </c>
       <c r="E612" t="n">
         <v>1</v>
@@ -15115,17 +15115,17 @@
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>And—but inflation outlook did not move strongly down here in the United States.</t>
+          <t>The second point that I made was that when short-term interest rates hit zero, the tools of a central bank are no farsighted—are not exhausted, there are still other things that the exchange bank can do to create additional adjustment.</t>
         </is>
       </c>
       <c r="B613" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C613" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D613" t="n">
-        <v>59</v>
+        <v>252</v>
       </c>
       <c r="E613" t="n">
         <v>1</v>
@@ -15139,17 +15139,17 @@
     <row r="614">
       <c r="A614" t="inlineStr">
         <is>
-          <t>And it is not—it’s not exactly the same as see global growth, where you see growth weakening, you see primal banks and governments responding with fiscal policy, and you see growth strengthening, and you see a business cycle.</t>
+          <t>And—but inflation outlook did not move strongly down here in the United States.</t>
         </is>
       </c>
       <c r="B614" t="n">
-        <v>2020</v>
+        <v>2011</v>
       </c>
       <c r="C614" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D614" t="n">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="E614" t="n">
         <v>1</v>
@@ -15163,17 +15163,17 @@
     <row r="615">
       <c r="A615" t="inlineStr">
         <is>
-          <t>The recent lower readings on inflation have been driven significantly by what appear to be one-murder simplification in certain categories of prices, such as wireless telephone services and prescription drugs.</t>
+          <t>And it is not—it’s not exactly the same as see global growth, where you see growth weakening, you see primal banks and governments responding with fiscal policy, and you see growth strengthening, and you see a business cycle.</t>
         </is>
       </c>
       <c r="B615" t="n">
-        <v>2012</v>
+        <v>2020</v>
       </c>
       <c r="C615" t="n">
         <v>0</v>
       </c>
       <c r="D615" t="n">
-        <v>251</v>
+        <v>22</v>
       </c>
       <c r="E615" t="n">
         <v>1</v>
@@ -15187,17 +15187,17 @@
     <row r="616">
       <c r="A616" t="inlineStr">
         <is>
-          <t>So you’re expire to have different perspectives from Committee player about how fast growth will be, how fast the labor market will heal, or how fast—sorry, inflation will move up.</t>
+          <t>The recent lower readings on inflation have been driven significantly by what appear to be one-murder simplification in certain categories of prices, such as wireless telephone services and prescription drugs.</t>
         </is>
       </c>
       <c r="B616" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="C616" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D616" t="n">
-        <v>213</v>
+        <v>251</v>
       </c>
       <c r="E616" t="n">
         <v>1</v>
@@ -15211,17 +15211,17 @@
     <row r="617">
       <c r="A617" t="inlineStr">
         <is>
-          <t>Against this backdrop, today the Federal Open Market Committee raised its policy pastime rate by ¾ percentage point and anticipate that ongoing increases in that rate will be appropriate.</t>
+          <t>So you’re expire to have different perspectives from Committee player about how fast growth will be, how fast the labor market will heal, or how fast—sorry, inflation will move up.</t>
         </is>
       </c>
       <c r="B617" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="C617" t="n">
         <v>1</v>
       </c>
       <c r="D617" t="n">
-        <v>5</v>
+        <v>213</v>
       </c>
       <c r="E617" t="n">
         <v>1</v>
@@ -15235,17 +15235,17 @@
     <row r="618">
       <c r="A618" t="inlineStr">
         <is>
-          <t>We have a 2 percentage symmetric inflation objective, and, for a number of years now, inflation has been running under 2 percent.</t>
+          <t>Against this backdrop, today the Federal Open Market Committee raised its policy pastime rate by ¾ percentage point and anticipate that ongoing increases in that rate will be appropriate.</t>
         </is>
       </c>
       <c r="B618" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="C618" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D618" t="n">
-        <v>278</v>
+        <v>5</v>
       </c>
       <c r="E618" t="n">
         <v>1</v>
@@ -15259,17 +15259,17 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>In addition, the median approximation of the longer-run normal unemployment rate moved down a tenth to 4.6 pct.</t>
+          <t>We have a 2 percentage symmetric inflation objective, and, for a number of years now, inflation has been running under 2 percent.</t>
         </is>
       </c>
       <c r="B619" t="n">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="C619" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D619" t="n">
-        <v>131</v>
+        <v>278</v>
       </c>
       <c r="E619" t="n">
         <v>1</v>
@@ -15283,17 +15283,17 @@
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>We deficiency to see lower unemployment.</t>
+          <t>In addition, the median approximation of the longer-run normal unemployment rate moved down a tenth to 4.6 pct.</t>
         </is>
       </c>
       <c r="B620" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="C620" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D620" t="n">
-        <v>288</v>
+        <v>131</v>
       </c>
       <c r="E620" t="n">
         <v>1</v>
@@ -15307,17 +15307,17 @@
     <row r="621">
       <c r="A621" t="inlineStr">
         <is>
-          <t>At the time of our FOMC meeting in Jan, scene for continued economic growth remained favorable, and we judged that monetary policy was well positioned to support that outlook.</t>
+          <t>We deficiency to see lower unemployment.</t>
         </is>
       </c>
       <c r="B621" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="C621" t="n">
         <v>0</v>
       </c>
       <c r="D621" t="n">
-        <v>69</v>
+        <v>288</v>
       </c>
       <c r="E621" t="n">
         <v>1</v>
@@ -15331,17 +15331,17 @@
     <row r="622">
       <c r="A622" t="inlineStr">
         <is>
-          <t>By contrast, raising rates too lento would raise the risk that monetary policy would need to tighten abruptly down the road, which could jeopardize the economic expansion.</t>
+          <t>At the time of our FOMC meeting in Jan, scene for continued economic growth remained favorable, and we judged that monetary policy was well positioned to support that outlook.</t>
         </is>
       </c>
       <c r="B622" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="C622" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D622" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="E622" t="n">
         <v>1</v>
@@ -15355,17 +15355,17 @@
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
-          <t>We, candidly, didn’t even get inflation back up to target—without seeing wages take out of touch with—with where they should be, so that’s the—that’s the biggest thing we can do.</t>
+          <t>By contrast, raising rates too lento would raise the risk that monetary policy would need to tighten abruptly down the road, which could jeopardize the economic expansion.</t>
         </is>
       </c>
       <c r="B623" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C623" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D623" t="n">
-        <v>290</v>
+        <v>94</v>
       </c>
       <c r="E623" t="n">
         <v>1</v>
@@ -15379,7 +15379,7 @@
     <row r="624">
       <c r="A624" t="inlineStr">
         <is>
-          <t>We have not focused on whether we meet the liftoff examination, because we assume’t meet the liftoff test now because we’re not at maximum employment.</t>
+          <t>We, candidly, didn’t even get inflation back up to target—without seeing wages take out of touch with—with where they should be, so that’s the—that’s the biggest thing we can do.</t>
         </is>
       </c>
       <c r="B624" t="n">
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="D624" t="n">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="E624" t="n">
         <v>1</v>
@@ -15403,17 +15403,17 @@
     <row r="625">
       <c r="A625" t="inlineStr">
         <is>
-          <t>The Federal Reserve is fully committed to both sides of its mandatory—to price stability as well as to uttermost employment—and it has both the tools and the will to act at the appropriate time to avoid any emerging threat to price stability.</t>
+          <t>We have not focused on whether we meet the liftoff examination, because we assume’t meet the liftoff test now because we’re not at maximum employment.</t>
         </is>
       </c>
       <c r="B625" t="n">
         <v>2020</v>
       </c>
       <c r="C625" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D625" t="n">
-        <v>235</v>
+        <v>283</v>
       </c>
       <c r="E625" t="n">
         <v>1</v>
@@ -15427,17 +15427,17 @@
     <row r="626">
       <c r="A626" t="inlineStr">
         <is>
-          <t>Well, you’re certainly right that we have been over-optimistic about taboo-year growth.</t>
+          <t>The Federal Reserve is fully committed to both sides of its mandatory—to price stability as well as to uttermost employment—and it has both the tools and the will to act at the appropriate time to avoid any emerging threat to price stability.</t>
         </is>
       </c>
       <c r="B626" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C626" t="n">
         <v>1</v>
       </c>
       <c r="D626" t="n">
-        <v>296</v>
+        <v>235</v>
       </c>
       <c r="E626" t="n">
         <v>1</v>
@@ -15451,17 +15451,17 @@
     <row r="627">
       <c r="A627" t="inlineStr">
         <is>
-          <t>We think that the economy will need highly accommodative monetary policy and the enjoyment of our tools for an extended period.</t>
+          <t>Well, you’re certainly right that we have been over-optimistic about taboo-year growth.</t>
         </is>
       </c>
       <c r="B627" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="C627" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D627" t="n">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="E627" t="n">
         <v>1</v>
@@ -15475,17 +15475,17 @@
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>And productiveness’s been very low.</t>
+          <t>We think that the economy will need highly accommodative monetary policy and the enjoyment of our tools for an extended period.</t>
         </is>
       </c>
       <c r="B628" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C628" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D628" t="n">
-        <v>30</v>
+        <v>286</v>
       </c>
       <c r="E628" t="n">
         <v>1</v>
@@ -15499,17 +15499,17 @@
     <row r="629">
       <c r="A629" t="inlineStr">
         <is>
-          <t>The persistence of that into, into inflation over clip is just not there.</t>
+          <t>And productiveness’s been very low.</t>
         </is>
       </c>
       <c r="B629" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C629" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D629" t="n">
-        <v>249</v>
+        <v>30</v>
       </c>
       <c r="E629" t="n">
         <v>1</v>
@@ -15523,17 +15523,17 @@
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
-          <t>So, if we maintain a highly accommodative monetary policy for a very long metre from here and the economy performs as we expect—namely, it’s strong and the risks that are kayoed there don’t materialize—my concern will be that we will have much more tightening in labor markets than you view in these projections.</t>
+          <t>The persistence of that into, into inflation over clip is just not there.</t>
         </is>
       </c>
       <c r="B630" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C630" t="n">
         <v>0</v>
       </c>
       <c r="D630" t="n">
-        <v>219</v>
+        <v>249</v>
       </c>
       <c r="E630" t="n">
         <v>1</v>
@@ -15547,17 +15547,17 @@
     <row r="631">
       <c r="A631" t="inlineStr">
         <is>
-          <t>We had a 10 percentage unemployment rate, and our congressional mandate is maximum employment and price stability.</t>
+          <t>So, if we maintain a highly accommodative monetary policy for a very long metre from here and the economy performs as we expect—namely, it’s strong and the risks that are kayoed there don’t materialize—my concern will be that we will have much more tightening in labor markets than you view in these projections.</t>
         </is>
       </c>
       <c r="B631" t="n">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="C631" t="n">
         <v>0</v>
       </c>
       <c r="D631" t="n">
-        <v>276</v>
+        <v>219</v>
       </c>
       <c r="E631" t="n">
         <v>1</v>
@@ -15571,17 +15571,17 @@
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>You recognise, what you hear out there is that demand—you talk to banks, and they’ll allege demand for loans is very, very low right now.</t>
+          <t>We had a 10 percentage unemployment rate, and our congressional mandate is maximum employment and price stability.</t>
         </is>
       </c>
       <c r="B632" t="n">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="C632" t="n">
         <v>0</v>
       </c>
       <c r="D632" t="n">
-        <v>313</v>
+        <v>276</v>
       </c>
       <c r="E632" t="n">
         <v>1</v>
@@ -15595,7 +15595,7 @@
     <row r="633">
       <c r="A633" t="inlineStr">
         <is>
-          <t>So, with this coronavirus arriving, we judged that the—the net effects of this will be to—to have inflation move down even a piddling turn more.</t>
+          <t>You recognise, what you hear out there is that demand—you talk to banks, and they’ll allege demand for loans is very, very low right now.</t>
         </is>
       </c>
       <c r="B633" t="n">
@@ -15605,7 +15605,7 @@
         <v>0</v>
       </c>
       <c r="D633" t="n">
-        <v>222</v>
+        <v>313</v>
       </c>
       <c r="E633" t="n">
         <v>1</v>
@@ -15619,17 +15619,17 @@
     <row r="634">
       <c r="A634" t="inlineStr">
         <is>
-          <t>These headwinds—which admit developments abroad, subdued household organization, and meager productivity growth—could persist for some time.</t>
+          <t>So, with this coronavirus arriving, we judged that the—the net effects of this will be to—to have inflation move down even a piddling turn more.</t>
         </is>
       </c>
       <c r="B634" t="n">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="C634" t="n">
         <v>0</v>
       </c>
       <c r="D634" t="n">
-        <v>262</v>
+        <v>222</v>
       </c>
       <c r="E634" t="n">
         <v>1</v>
@@ -15643,17 +15643,17 @@
     <row r="635">
       <c r="A635" t="inlineStr">
         <is>
-          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can raise interest rates at the reserve time, even if the balance sheet remains large for an extended menstruum.</t>
+          <t>These headwinds—which admit developments abroad, subdued household organization, and meager productivity growth—could persist for some time.</t>
         </is>
       </c>
       <c r="B635" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C635" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D635" t="n">
-        <v>188</v>
+        <v>262</v>
       </c>
       <c r="E635" t="n">
         <v>1</v>
@@ -15667,17 +15667,17 @@
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
-          <t>And no, we’re not—we, we have not at all changed our scene, and I harbor’t changed my view that inflation running above 2 percent, moderately above 2 percent, is a desirable thing.</t>
+          <t>So I, you know, I’m—I feel quite comfortable that we can—in particular, that we can raise interest rates at the reserve time, even if the balance sheet remains large for an extended menstruum.</t>
         </is>
       </c>
       <c r="B636" t="n">
-        <v>2011</v>
+        <v>2020</v>
       </c>
       <c r="C636" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D636" t="n">
-        <v>25</v>
+        <v>188</v>
       </c>
       <c r="E636" t="n">
         <v>1</v>
@@ -15691,17 +15691,17 @@
     <row r="637">
       <c r="A637" t="inlineStr">
         <is>
-          <t>Foresightful-term unemployment in the current economy is—is the worst—really the worst it’s been in the postwar period.</t>
+          <t>And no, we’re not—we, we have not at all changed our scene, and I harbor’t changed my view that inflation running above 2 percent, moderately above 2 percent, is a desirable thing.</t>
         </is>
       </c>
       <c r="B637" t="n">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C637" t="n">
         <v>0</v>
       </c>
       <c r="D637" t="n">
-        <v>162</v>
+        <v>25</v>
       </c>
       <c r="E637" t="n">
         <v>1</v>
@@ -15715,17 +15715,17 @@
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
-          <t>Well, if the economy worsens and inflation remains relatively low, then we wouldn’t begin to loss, and, therefore, we wouldn’t change the lyric.</t>
+          <t>Foresightful-term unemployment in the current economy is—is the worst—really the worst it’s been in the postwar period.</t>
         </is>
       </c>
       <c r="B638" t="n">
-        <v>2020</v>
+        <v>2012</v>
       </c>
       <c r="C638" t="n">
         <v>0</v>
       </c>
       <c r="D638" t="n">
-        <v>291</v>
+        <v>162</v>
       </c>
       <c r="E638" t="n">
         <v>1</v>
@@ -15739,17 +15739,17 @@
     <row r="639">
       <c r="A639" t="inlineStr">
         <is>
-          <t>Well, you know, if the economy were disappointing, we—you know, our action wouldn’t strictly be based on inflation, we would also take employment into account.</t>
+          <t>Well, if the economy worsens and inflation remains relatively low, then we wouldn’t begin to loss, and, therefore, we wouldn’t change the lyric.</t>
         </is>
       </c>
       <c r="B639" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C639" t="n">
         <v>0</v>
       </c>
       <c r="D639" t="n">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="E639" t="n">
         <v>1</v>
@@ -15763,17 +15763,17 @@
     <row r="640">
       <c r="A640" t="inlineStr">
         <is>
-          <t>The Federal Reserve’s response is guided by our mandate to advance maximum employment and stalls prices for the American people, along with our responsibilities to promote the stability of the financial system.</t>
+          <t>Well, you know, if the economy were disappointing, we—you know, our action wouldn’t strictly be based on inflation, we would also take employment into account.</t>
         </is>
       </c>
       <c r="B640" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C640" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D640" t="n">
-        <v>237</v>
+        <v>295</v>
       </c>
       <c r="E640" t="n">
         <v>1</v>
@@ -15787,41 +15787,41 @@
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>For [MASK], we have [MASK] some [MASK] our work to look [MASK] interest rate risk and [MASK] [MASK] [MASK] and, you know, found generally that banks can also sustain a significant increase in long-term interest [MASK] as well for [MASK] number of reasons, one of them being that higher interest rates increase their franchise value because it increases their net interest [MASK] over time.</t>
+          <t>The Federal Reserve’s response is guided by our mandate to advance maximum employment and stalls prices for the American people, along with our responsibilities to promote the stability of the financial system.</t>
         </is>
       </c>
       <c r="B641" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C641" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D641" t="n">
-        <v>104</v>
+        <v>237</v>
       </c>
       <c r="E641" t="n">
         <v>1</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>masking</t>
+          <t>synonym_replacement</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>[MASK]—and we do that with [MASK] that—that, you know, keep people in their homes; that—that support hiring; that support [MASK]; that avoid unnecessary, avoidable business [MASK].</t>
+          <t>For [MASK], we have [MASK] some [MASK] our work to look [MASK] interest rate risk and [MASK] [MASK] [MASK] and, you know, found generally that banks can also sustain a significant increase in long-term interest [MASK] as well for [MASK] number of reasons, one of them being that higher interest rates increase their franchise value because it increases their net interest [MASK] over time.</t>
         </is>
       </c>
       <c r="B642" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="C642" t="n">
         <v>2</v>
       </c>
       <c r="D642" t="n">
-        <v>58</v>
+        <v>104</v>
       </c>
       <c r="E642" t="n">
         <v>1</v>
@@ -15835,17 +15835,17 @@
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>For example, one—in the long-[MASK], the size of the balance sheet is going [MASK] [MASK] on the public’s demand for our liabilities, including currency [MASK] reserves.</t>
+          <t>[MASK]—and we do that with [MASK] that—that, you know, keep people in their homes; that—that support hiring; that support [MASK]; that avoid unnecessary, avoidable business [MASK].</t>
         </is>
       </c>
       <c r="B643" t="n">
-        <v>2021</v>
+        <v>2011</v>
       </c>
       <c r="C643" t="n">
         <v>2</v>
       </c>
       <c r="D643" t="n">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="E643" t="n">
         <v>1</v>
@@ -15859,17 +15859,17 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Now, [MASK] inflation below 2 percent, I think it’s appropriate that [MASK] labor market [MASK] that tight.</t>
+          <t>For example, one—in the long-[MASK], the size of the balance sheet is going [MASK] [MASK] on the public’s demand for our liabilities, including currency [MASK] reserves.</t>
         </is>
       </c>
       <c r="B644" t="n">
         <v>2021</v>
       </c>
       <c r="C644" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D644" t="n">
-        <v>172</v>
+        <v>102</v>
       </c>
       <c r="E644" t="n">
         <v>1</v>
@@ -15883,17 +15883,17 @@
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>The jobs picture continues to be [MASK], with the unemployment rate near historic lows [MASK] with stronger wage [MASK].</t>
+          <t>Now, [MASK] inflation below 2 percent, I think it’s appropriate that [MASK] labor market [MASK] that tight.</t>
         </is>
       </c>
       <c r="B645" t="n">
         <v>2021</v>
       </c>
       <c r="C645" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D645" t="n">
-        <v>247</v>
+        <v>172</v>
       </c>
       <c r="E645" t="n">
         <v>1</v>
@@ -15907,7 +15907,7 @@
     <row r="646">
       <c r="A646" t="inlineStr">
         <is>
-          <t>Our role, though, is also to, [MASK] know, to make [MASK] [MASK]—that maximum employment happens in a context of [MASK] stability and financial stability, which is why we’re [MASK] raising rates.</t>
+          <t>The jobs picture continues to be [MASK], with the unemployment rate near historic lows [MASK] with stronger wage [MASK].</t>
         </is>
       </c>
       <c r="B646" t="n">
@@ -15917,7 +15917,7 @@
         <v>1</v>
       </c>
       <c r="D646" t="n">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="E646" t="n">
         <v>1</v>
@@ -15931,17 +15931,17 @@
     <row r="647">
       <c r="A647" t="inlineStr">
         <is>
-          <t>In addition, [MASK] median estimate of the longer-run normal [MASK] rate moved down [MASK] tenth to 4.6 percent.</t>
+          <t>Our role, though, is also to, [MASK] know, to make [MASK] [MASK]—that maximum employment happens in a context of [MASK] stability and financial stability, which is why we’re [MASK] raising rates.</t>
         </is>
       </c>
       <c r="B647" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C647" t="n">
         <v>1</v>
       </c>
       <c r="D647" t="n">
-        <v>131</v>
+        <v>179</v>
       </c>
       <c r="E647" t="n">
         <v>1</v>
@@ -15955,17 +15955,17 @@
     <row r="648">
       <c r="A648" t="inlineStr">
         <is>
-          <t>That transition [MASK] could help bring inflation down, because, presumably, people would spend a little less on [MASK] while they start spending [MASK] on travel and all [MASK] of travel services [MASK] things like that.</t>
+          <t>In addition, [MASK] median estimate of the longer-run normal [MASK] rate moved down [MASK] tenth to 4.6 percent.</t>
         </is>
       </c>
       <c r="B648" t="n">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="C648" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D648" t="n">
-        <v>229</v>
+        <v>131</v>
       </c>
       <c r="E648" t="n">
         <v>1</v>
@@ -15979,17 +15979,17 @@
     <row r="649">
       <c r="A649" t="inlineStr">
         <is>
-          <t>[MASK] [MASK] has not—what, what [MASK] is that [MASK] wages move up because unemployment is low, companies have been absorbing that increase into their margins rather than raising prices.</t>
+          <t>That transition [MASK] could help bring inflation down, because, presumably, people would spend a little less on [MASK] while they start spending [MASK] on travel and all [MASK] of travel services [MASK] things like that.</t>
         </is>
       </c>
       <c r="B649" t="n">
-        <v>2020</v>
+        <v>2016</v>
       </c>
       <c r="C649" t="n">
         <v>2</v>
       </c>
       <c r="D649" t="n">
-        <v>84</v>
+        <v>229</v>
       </c>
       <c r="E649" t="n">
         <v>1</v>
@@ -16003,17 +16003,17 @@
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t>So you’[MASK] talking about the inflation target, basically.</t>
+          <t>[MASK] [MASK] has not—what, what [MASK] is that [MASK] wages move up because unemployment is low, companies have been absorbing that increase into their margins rather than raising prices.</t>
         </is>
       </c>
       <c r="B650" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C650" t="n">
         <v>2</v>
       </c>
       <c r="D650" t="n">
-        <v>215</v>
+        <v>84</v>
       </c>
       <c r="E650" t="n">
         <v>1</v>
@@ -16027,17 +16027,17 @@
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>[MASK], and those [MASK]—that’s again—that goes to [MASK] this episode as short [MASK] it can be and avoiding unnecessary business bankruptcies, unnecessary household bankruptcies, [MASK] unnecessary long-term stays of unemployment or supporting [MASK] through them so [MASK] they [MASK] maintain their financial footing and their lives [MASK] be able to go back to work in a productive way.</t>
+          <t>So you’[MASK] talking about the inflation target, basically.</t>
         </is>
       </c>
       <c r="B651" t="n">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="C651" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D651" t="n">
-        <v>52</v>
+        <v>215</v>
       </c>
       <c r="E651" t="n">
         <v>1</v>
@@ -16051,17 +16051,17 @@
     <row r="652">
       <c r="A652" t="inlineStr">
         <is>
-          <t>By the way, we’re also not at [MASK] employment, [MASK] I mentioned.</t>
+          <t>[MASK], and those [MASK]—that’s again—that goes to [MASK] this episode as short [MASK] it can be and avoiding unnecessary business bankruptcies, unnecessary household bankruptcies, [MASK] unnecessary long-term stays of unemployment or supporting [MASK] through them so [MASK] they [MASK] maintain their financial footing and their lives [MASK] be able to go back to work in a productive way.</t>
         </is>
       </c>
       <c r="B652" t="n">
-        <v>2017</v>
+        <v>2015</v>
       </c>
       <c r="C652" t="n">
         <v>0</v>
       </c>
       <c r="D652" t="n">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="E652" t="n">
         <v>1</v>
@@ -16075,17 +16075,17 @@
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>But now, let’s go to [MASK]—the part of your question about [MASK].</t>
+          <t>By the way, we’re also not at [MASK] employment, [MASK] I mentioned.</t>
         </is>
       </c>
       <c r="B653" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C653" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D653" t="n">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="E653" t="n">
         <v>1</v>
@@ -16099,17 +16099,17 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>So that means a more [MASK] shortfall of inflation.</t>
+          <t>But now, let’s go to [MASK]—the part of your question about [MASK].</t>
         </is>
       </c>
       <c r="B654" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C654" t="n">
         <v>2</v>
       </c>
       <c r="D654" t="n">
-        <v>199</v>
+        <v>83</v>
       </c>
       <c r="E654" t="n">
         <v>1</v>
@@ -16123,17 +16123,17 @@
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>[MASK]’s a lot more demand for risk [MASK], for liquidity services, and so on.</t>
+          <t>So that means a more [MASK] shortfall of inflation.</t>
         </is>
       </c>
       <c r="B655" t="n">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="C655" t="n">
         <v>2</v>
       </c>
       <c r="D655" t="n">
-        <v>259</v>
+        <v>199</v>
       </c>
       <c r="E655" t="n">
         <v>1</v>
@@ -16147,17 +16147,17 @@
     <row r="656">
       <c r="A656" t="inlineStr">
         <is>
-          <t>And [MASK]’s been very low.</t>
+          <t>[MASK]’s a lot more demand for risk [MASK], for liquidity services, and so on.</t>
         </is>
       </c>
       <c r="B656" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="C656" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D656" t="n">
-        <v>30</v>
+        <v>259</v>
       </c>
       <c r="E656" t="n">
         <v>1</v>
@@ -16171,17 +16171,17 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>As I mentioned, once [MASK]—once you’re, broadly speaking, in the range of neutral, I [MASK] it’[MASK] appropriate to be putting [MASK] individual estimates of that [MASK] be looking at what the incoming data are [MASK] you [MASK] the outlook, updating your estimates of what neutral might be, of what the natural [MASK] [MASK] unemployment might be, of the state of the economy, [MASK]—and letting that lead you to adjust your [MASK] and, therefore, your appropriate [MASK] for policy.</t>
+          <t>And [MASK]’s been very low.</t>
         </is>
       </c>
       <c r="B657" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="C657" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D657" t="n">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="E657" t="n">
         <v>1</v>
@@ -16195,17 +16195,17 @@
     <row r="658">
       <c r="A658" t="inlineStr">
         <is>
-          <t>So it’[MASK] a serious economic problem [MASK] the United [MASK], but it’s—it’s got underlying causes that [MASK] not [MASK] to monetary policy or to our response to the pandemic.</t>
+          <t>As I mentioned, once [MASK]—once you’re, broadly speaking, in the range of neutral, I [MASK] it’[MASK] appropriate to be putting [MASK] individual estimates of that [MASK] be looking at what the incoming data are [MASK] you [MASK] the outlook, updating your estimates of what neutral might be, of what the natural [MASK] [MASK] unemployment might be, of the state of the economy, [MASK]—and letting that lead you to adjust your [MASK] and, therefore, your appropriate [MASK] for policy.</t>
         </is>
       </c>
       <c r="B658" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="C658" t="n">
         <v>2</v>
       </c>
       <c r="D658" t="n">
-        <v>194</v>
+        <v>61</v>
       </c>
       <c r="E658" t="n">
         <v>1</v>
@@ -16219,17 +16219,17 @@
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
-          <t>So, you [MASK], as I [MASK], the Committee acutely feels its [MASK] to move to make sure that [MASK] restore price stability [MASK] is determined to use its tools to do so.</t>
+          <t>So it’[MASK] a serious economic problem [MASK] the United [MASK], but it’s—it’s got underlying causes that [MASK] not [MASK] to monetary policy or to our response to the pandemic.</t>
         </is>
       </c>
       <c r="B659" t="n">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="C659" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D659" t="n">
-        <v>224</v>
+        <v>194</v>
       </c>
       <c r="E659" t="n">
         <v>1</v>
@@ -16243,17 +16243,17 @@
     <row r="660">
       <c r="A660" t="inlineStr">
         <is>
-          <t>And so when asset prices [MASK] back up, probably there’ll [MASK] a swing around there, a positive [MASK].</t>
+          <t>So, you [MASK], as I [MASK], the Committee acutely feels its [MASK] to move to make sure that [MASK] restore price stability [MASK] is determined to use its tools to do so.</t>
         </is>
       </c>
       <c r="B660" t="n">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="C660" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D660" t="n">
-        <v>32</v>
+        <v>224</v>
       </c>
       <c r="E660" t="n">
         <v>1</v>
@@ -16267,7 +16267,7 @@
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>We also don’t conduct monetary [MASK] [MASK] order to prove our independence.</t>
+          <t>And so when asset prices [MASK] back up, probably there’ll [MASK] a swing around there, a positive [MASK].</t>
         </is>
       </c>
       <c r="B661" t="n">
@@ -16277,7 +16277,7 @@
         <v>2</v>
       </c>
       <c r="D661" t="n">
-        <v>270</v>
+        <v>32</v>
       </c>
       <c r="E661" t="n">
         <v>1</v>
@@ -16291,17 +16291,17 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>Inflation pressures [MASK] muted, and indicators of [MASK]-[MASK] inflation expectations are at the lower end of their historic ranges.</t>
+          <t>We also don’t conduct monetary [MASK] [MASK] order to prove our independence.</t>
         </is>
       </c>
       <c r="B662" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="C662" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D662" t="n">
-        <v>145</v>
+        <v>270</v>
       </c>
       <c r="E662" t="n">
         <v>1</v>
@@ -16315,17 +16315,17 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>And, and some [MASK] [MASK] answer to that may be price.</t>
+          <t>Inflation pressures [MASK] muted, and indicators of [MASK]-[MASK] inflation expectations are at the lower end of their historic ranges.</t>
         </is>
       </c>
       <c r="B663" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="C663" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D663" t="n">
-        <v>50</v>
+        <v>145</v>
       </c>
       <c r="E663" t="n">
         <v>1</v>
@@ -16339,17 +16339,17 @@
     <row r="664">
       <c r="A664" t="inlineStr">
         <is>
-          <t>[MASK] you’re right, you’re seeing—I, I can’t remember the number, but [MASK] might be [MASK] [MASK] 3s—3, 3½ percent growth for next year.</t>
+          <t>And, and some [MASK] [MASK] answer to that may be price.</t>
         </is>
       </c>
       <c r="B664" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="C664" t="n">
         <v>2</v>
       </c>
       <c r="D664" t="n">
-        <v>214</v>
+        <v>50</v>
       </c>
       <c r="E664" t="n">
         <v>1</v>
@@ -16363,17 +16363,17 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>We have not focused on whether we meet [MASK] liftoff test, because we don’t [MASK] the liftoff [MASK] now [MASK] we’re not at maximum employment.</t>
+          <t>[MASK] you’re right, you’re seeing—I, I can’t remember the number, but [MASK] might be [MASK] [MASK] 3s—3, 3½ percent growth for next year.</t>
         </is>
       </c>
       <c r="B665" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C665" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D665" t="n">
-        <v>283</v>
+        <v>214</v>
       </c>
       <c r="E665" t="n">
         <v>1</v>
@@ -16387,7 +16387,7 @@
     <row r="666">
       <c r="A666" t="inlineStr">
         <is>
-          <t>And it is not—it’s not exactly the same as watching global [MASK], where [MASK] see growth weakening, [MASK] [MASK] central banks and governments responding with fiscal policy, and you see growth [MASK], and [MASK] see a business cycle.</t>
+          <t>We have not focused on whether we meet [MASK] liftoff test, because we don’t [MASK] the liftoff [MASK] now [MASK] we’re not at maximum employment.</t>
         </is>
       </c>
       <c r="B666" t="n">
@@ -16397,7 +16397,7 @@
         <v>0</v>
       </c>
       <c r="D666" t="n">
-        <v>22</v>
+        <v>283</v>
       </c>
       <c r="E666" t="n">
         <v>1</v>
@@ -16411,17 +16411,17 @@
     <row r="667">
       <c r="A667" t="inlineStr">
         <is>
-          <t>It isn’t really just targeting the [MASK] numbers, but [MASK]’s about taking [MASK] of those things into [MASK] in your thinking about what constitutes maximum employment.</t>
+          <t>And it is not—it’s not exactly the same as watching global [MASK], where [MASK] see growth weakening, [MASK] [MASK] central banks and governments responding with fiscal policy, and you see growth [MASK], and [MASK] see a business cycle.</t>
         </is>
       </c>
       <c r="B667" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C667" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D667" t="n">
-        <v>150</v>
+        <v>22</v>
       </c>
       <c r="E667" t="n">
         <v>1</v>
@@ -16435,17 +16435,17 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>[MASK] tools work on demand.</t>
+          <t>It isn’t really just targeting the [MASK] numbers, but [MASK]’s about taking [MASK] of those things into [MASK] in your thinking about what constitutes maximum employment.</t>
         </is>
       </c>
       <c r="B668" t="n">
-        <v>2012</v>
+        <v>2021</v>
       </c>
       <c r="C668" t="n">
         <v>2</v>
       </c>
       <c r="D668" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E668" t="n">
         <v>1</v>
@@ -16459,17 +16459,17 @@
     <row r="669">
       <c r="A669" t="inlineStr">
         <is>
-          <t>I would say, in the area of commercial real [MASK], [MASK] valuations [MASK] [MASK], we are seeing some tightening of lending standards [MASK] less debt growth associated with that rise in commercial real estate prices.</t>
+          <t>[MASK] tools work on demand.</t>
         </is>
       </c>
       <c r="B669" t="n">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="C669" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D669" t="n">
-        <v>122</v>
+        <v>180</v>
       </c>
       <c r="E669" t="n">
         <v>1</v>
@@ -16483,17 +16483,17 @@
     <row r="670">
       <c r="A670" t="inlineStr">
         <is>
-          <t>If inflation remains higher during the course [MASK] 2022, [MASK] we may already [MASK] met that test by the time we reach liftoff.</t>
+          <t>I would say, in the area of commercial real [MASK], [MASK] valuations [MASK] [MASK], we are seeing some tightening of lending standards [MASK] less debt growth associated with that rise in commercial real estate prices.</t>
         </is>
       </c>
       <c r="B670" t="n">
         <v>2016</v>
       </c>
       <c r="C670" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D670" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E670" t="n">
         <v>1</v>
@@ -16507,17 +16507,17 @@
     <row r="671">
       <c r="A671" t="inlineStr">
         <is>
-          <t>You know, we’re, [MASK]’re—inflation measures are always going to be a [MASK] volatile.</t>
+          <t>If inflation remains higher during the course [MASK] 2022, [MASK] we may already [MASK] met that test by the time we reach liftoff.</t>
         </is>
       </c>
       <c r="B671" t="n">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="C671" t="n">
         <v>2</v>
       </c>
       <c r="D671" t="n">
-        <v>312</v>
+        <v>123</v>
       </c>
       <c r="E671" t="n">
         <v>1</v>
@@ -16531,17 +16531,17 @@
     <row r="672">
       <c r="A672" t="inlineStr">
         <is>
-          <t>We're [MASK] at wages and we're looking [MASK] ultimately inflation.</t>
+          <t>You know, we’re, [MASK]’re—inflation measures are always going to be a [MASK] volatile.</t>
         </is>
       </c>
       <c r="B672" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="C672" t="n">
         <v>2</v>
       </c>
       <c r="D672" t="n">
-        <v>289</v>
+        <v>312</v>
       </c>
       <c r="E672" t="n">
         <v>1</v>
@@ -16555,17 +16555,17 @@
     <row r="673">
       <c r="A673" t="inlineStr">
         <is>
-          <t>So you’re [MASK] to have different perspectives from Committee participants about how fast growth will be, how [MASK] [MASK] labor market will [MASK], or how fast—sorry, inflation [MASK] move up.</t>
+          <t>We're [MASK] at wages and we're looking [MASK] ultimately inflation.</t>
         </is>
       </c>
       <c r="B673" t="n">
         <v>2019</v>
       </c>
       <c r="C673" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D673" t="n">
-        <v>213</v>
+        <v>289</v>
       </c>
       <c r="E673" t="n">
         <v>1</v>
@@ -16579,17 +16579,17 @@
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>And that’[MASK] because of this misalignment [MASK] supply and demand.</t>
+          <t>So you’re [MASK] to have different perspectives from Committee participants about how fast growth will be, how [MASK] [MASK] labor market will [MASK], or how fast—sorry, inflation [MASK] move up.</t>
         </is>
       </c>
       <c r="B674" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C674" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D674" t="n">
-        <v>36</v>
+        <v>213</v>
       </c>
       <c r="E674" t="n">
         <v>1</v>
@@ -16603,7 +16603,7 @@
     <row r="675">
       <c r="A675" t="inlineStr">
         <is>
-          <t>But, certainly, we’ve had a lot of [MASK] in which interest rates [MASK] been low.</t>
+          <t>And that’[MASK] because of this misalignment [MASK] supply and demand.</t>
         </is>
       </c>
       <c r="B675" t="n">
@@ -16613,7 +16613,7 @@
         <v>2</v>
       </c>
       <c r="D675" t="n">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="E675" t="n">
         <v>1</v>
@@ -16627,17 +16627,17 @@
     <row r="676">
       <c r="A676" t="inlineStr">
         <is>
-          <t>So, as you know, the ultimate focus that we have is [MASK] [MASK] real economy: maximum employment [MASK] price stability.</t>
+          <t>But, certainly, we’ve had a lot of [MASK] in which interest rates [MASK] been low.</t>
         </is>
       </c>
       <c r="B676" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="C676" t="n">
         <v>2</v>
       </c>
       <c r="D676" t="n">
-        <v>218</v>
+        <v>90</v>
       </c>
       <c r="E676" t="n">
         <v>1</v>
@@ -16651,17 +16651,17 @@
     <row r="677">
       <c r="A677" t="inlineStr">
         <is>
-          <t>And the maximum level of [MASK] that’s consistent with price [MASK] evolves over time within a—within [MASK] business [MASK] and over a longer [MASK], in part reflecting [the] evolution [MASK] the factors that affect labor supply, [MASK] those related to the pandemic.</t>
+          <t>So, as you know, the ultimate focus that we have is [MASK] [MASK] real economy: maximum employment [MASK] price stability.</t>
         </is>
       </c>
       <c r="B677" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C677" t="n">
         <v>2</v>
       </c>
       <c r="D677" t="n">
-        <v>37</v>
+        <v>218</v>
       </c>
       <c r="E677" t="n">
         <v>1</v>
@@ -16675,17 +16675,17 @@
     <row r="678">
       <c r="A678" t="inlineStr">
         <is>
-          <t>So [MASK] Committee estimates that the longer-run normal level [MASK] the unemployment rate is 5.0 to 5.2.</t>
+          <t>And the maximum level of [MASK] that’s consistent with price [MASK] evolves over time within a—within [MASK] business [MASK] and over a longer [MASK], in part reflecting [the] evolution [MASK] the factors that affect labor supply, [MASK] those related to the pandemic.</t>
         </is>
       </c>
       <c r="B678" t="n">
-        <v>2013</v>
+        <v>2022</v>
       </c>
       <c r="C678" t="n">
         <v>2</v>
       </c>
       <c r="D678" t="n">
-        <v>202</v>
+        <v>37</v>
       </c>
       <c r="E678" t="n">
         <v>1</v>
@@ -16699,17 +16699,17 @@
     <row r="679">
       <c r="A679" t="inlineStr">
         <is>
-          <t>Last year, we [MASK] 1.9 percent productivity, which is much [MASK].</t>
+          <t>So [MASK] Committee estimates that the longer-run normal level [MASK] the unemployment rate is 5.0 to 5.2.</t>
         </is>
       </c>
       <c r="B679" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="C679" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D679" t="n">
-        <v>161</v>
+        <v>202</v>
       </c>
       <c r="E679" t="n">
         <v>1</v>
@@ -16723,17 +16723,17 @@
     <row r="680">
       <c r="A680" t="inlineStr">
         <is>
-          <t>So, we are taking [MASK] of international developments, including prospects for [MASK] in our [MASK] partners, in making the forecast we have here.</t>
+          <t>Last year, we [MASK] 1.9 percent productivity, which is much [MASK].</t>
         </is>
       </c>
       <c r="B680" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="C680" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D680" t="n">
-        <v>221</v>
+        <v>161</v>
       </c>
       <c r="E680" t="n">
         <v>1</v>
@@ -16747,17 +16747,17 @@
     <row r="681">
       <c r="A681" t="inlineStr">
         <is>
-          <t>If we—if we analyze inflation data and conclude [MASK], [MASK], transitory influences are holding down inflation, I do [MASK] want to say that we would [MASK] to that.</t>
+          <t>So, we are taking [MASK] of international developments, including prospects for [MASK] in our [MASK] partners, in making the forecast we have here.</t>
         </is>
       </c>
       <c r="B681" t="n">
-        <v>2021</v>
+        <v>2014</v>
       </c>
       <c r="C681" t="n">
         <v>2</v>
       </c>
       <c r="D681" t="n">
-        <v>126</v>
+        <v>221</v>
       </c>
       <c r="E681" t="n">
         <v>1</v>
@@ -16771,17 +16771,17 @@
     <row r="682">
       <c r="A682" t="inlineStr">
         <is>
-          <t>If we think that the potential growth rate [MASK] the economy [MASK] somewhere between, somewhere around 1.75 [MASK], 2.8 percent is strong economic growth.</t>
+          <t>If we—if we analyze inflation data and conclude [MASK], [MASK], transitory influences are holding down inflation, I do [MASK] want to say that we would [MASK] to that.</t>
         </is>
       </c>
       <c r="B682" t="n">
         <v>2021</v>
       </c>
       <c r="C682" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D682" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E682" t="n">
         <v>1</v>
@@ -16795,17 +16795,17 @@
     <row r="683">
       <c r="A683" t="inlineStr">
         <is>
-          <t>So in—in—in U-6, the U-6 level [MASK] [MASK] has tripled from 7 percent to 21 percent.</t>
+          <t>If we think that the potential growth rate [MASK] the economy [MASK] somewhere between, somewhere around 1.75 [MASK], 2.8 percent is strong economic growth.</t>
         </is>
       </c>
       <c r="B683" t="n">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="C683" t="n">
         <v>0</v>
       </c>
       <c r="D683" t="n">
-        <v>192</v>
+        <v>125</v>
       </c>
       <c r="E683" t="n">
         <v>1</v>
@@ -16819,17 +16819,17 @@
     <row r="684">
       <c r="A684" t="inlineStr">
         <is>
-          <t>[MASK] I assure you that my [MASK] and [MASK] will continue to conduct monetary policy without regard to political considerations.</t>
+          <t>So in—in—in U-6, the U-6 level [MASK] [MASK] has tripled from 7 percent to 21 percent.</t>
         </is>
       </c>
       <c r="B684" t="n">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="C684" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D684" t="n">
-        <v>8</v>
+        <v>192</v>
       </c>
       <c r="E684" t="n">
         <v>1</v>
@@ -16843,17 +16843,17 @@
     <row r="685">
       <c r="A685" t="inlineStr">
         <is>
-          <t>There [MASK] a lot of pent-up demand.</t>
+          <t>[MASK] I assure you that my [MASK] and [MASK] will continue to conduct monetary policy without regard to political considerations.</t>
         </is>
       </c>
       <c r="B685" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="C685" t="n">
         <v>2</v>
       </c>
       <c r="D685" t="n">
-        <v>258</v>
+        <v>8</v>
       </c>
       <c r="E685" t="n">
         <v>1</v>
@@ -16867,17 +16867,17 @@
     <row r="686">
       <c r="A686" t="inlineStr">
         <is>
-          <t>You know, it’s interest rates, it’s risk spreads, it’s currency, it’s [MASK] [MASK] [MASK], it’s credit availability, it’s many, [MASK] factors.</t>
+          <t>There [MASK] a lot of pent-up demand.</t>
         </is>
       </c>
       <c r="B686" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="C686" t="n">
         <v>2</v>
       </c>
       <c r="D686" t="n">
-        <v>309</v>
+        <v>258</v>
       </c>
       <c r="E686" t="n">
         <v>1</v>
@@ -16891,17 +16891,17 @@
     <row r="687">
       <c r="A687" t="inlineStr">
         <is>
-          <t>More broadly, however, weaker demand, especially in [MASK] that have [MASK] most affected by the pandemic, has held down consumer [MASK], and overall, inflation is running well below [MASK] 2 [MASK] longer-run objective.</t>
+          <t>You know, it’s interest rates, it’s risk spreads, it’s currency, it’s [MASK] [MASK] [MASK], it’s credit availability, it’s many, [MASK] factors.</t>
         </is>
       </c>
       <c r="B687" t="n">
-        <v>2014</v>
+        <v>2019</v>
       </c>
       <c r="C687" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D687" t="n">
-        <v>167</v>
+        <v>309</v>
       </c>
       <c r="E687" t="n">
         <v>1</v>
@@ -16915,17 +16915,17 @@
     <row r="688">
       <c r="A688" t="inlineStr">
         <is>
-          <t>Our mandate, [MASK], is price inflation.</t>
+          <t>More broadly, however, weaker demand, especially in [MASK] that have [MASK] most affected by the pandemic, has held down consumer [MASK], and overall, inflation is running well below [MASK] 2 [MASK] longer-run objective.</t>
         </is>
       </c>
       <c r="B688" t="n">
-        <v>2021</v>
+        <v>2014</v>
       </c>
       <c r="C688" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D688" t="n">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="E688" t="n">
         <v>1</v>
@@ -16939,17 +16939,17 @@
     <row r="689">
       <c r="A689" t="inlineStr">
         <is>
-          <t>So on the first, the Committee’s forecasts and [MASK] of most outside forecasters do show growth running below its longer-[MASK] potential this year [MASK] next [MASK].</t>
+          <t>Our mandate, [MASK], is price inflation.</t>
         </is>
       </c>
       <c r="B689" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C689" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D689" t="n">
-        <v>198</v>
+        <v>178</v>
       </c>
       <c r="E689" t="n">
         <v>1</v>
@@ -16963,17 +16963,17 @@
     <row r="690">
       <c r="A690" t="inlineStr">
         <is>
-          <t>So the—the sooner [MASK] get the virus under control, the sooner [MASK] [MASK] regain that confidence and regain their economic activity.</t>
+          <t>So on the first, the Committee’s forecasts and [MASK] of most outside forecasters do show growth running below its longer-[MASK] potential this year [MASK] next [MASK].</t>
         </is>
       </c>
       <c r="B690" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="C690" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D690" t="n">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="E690" t="n">
         <v>1</v>
@@ -16987,17 +16987,17 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>[MASK] you have seen a shift this time in most participants’ [MASK] of the appropriate path for policy, and, as I tried to indicate, I [MASK] that [MASK] reflects a somewhat slower projected path [MASK] global growth—[MASK] [MASK] in the global economy outside the [MASK] States—and for some tightening in credit conditions in [MASK] form of an increase in spreads.</t>
+          <t>So the—the sooner [MASK] get the virus under control, the sooner [MASK] [MASK] regain that confidence and regain their economic activity.</t>
         </is>
       </c>
       <c r="B691" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C691" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D691" t="n">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="E691" t="n">
         <v>1</v>
@@ -17011,17 +17011,17 @@
     <row r="692">
       <c r="A692" t="inlineStr">
         <is>
-          <t>[MASK] we’d like to [MASK] that in the form of a [MASK] of declining monthly inflation readings—that’[MASK] what we’re looking for.</t>
+          <t>[MASK] you have seen a shift this time in most participants’ [MASK] of the appropriate path for policy, and, as I tried to indicate, I [MASK] that [MASK] reflects a somewhat slower projected path [MASK] global growth—[MASK] [MASK] in the global economy outside the [MASK] States—and for some tightening in credit conditions in [MASK] form of an increase in spreads.</t>
         </is>
       </c>
       <c r="B692" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="C692" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D692" t="n">
-        <v>43</v>
+        <v>212</v>
       </c>
       <c r="E692" t="n">
         <v>1</v>
@@ -17035,17 +17035,17 @@
     <row r="693">
       <c r="A693" t="inlineStr">
         <is>
-          <t>I don’t really think asset prices themselves [MASK] a significant threat to financial [MASK], and that’s because households [MASK] in good shape [MASK] than they have been.</t>
+          <t>[MASK] we’d like to [MASK] that in the form of a [MASK] of declining monthly inflation readings—that’[MASK] what we’re looking for.</t>
         </is>
       </c>
       <c r="B693" t="n">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="C693" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D693" t="n">
-        <v>109</v>
+        <v>43</v>
       </c>
       <c r="E693" t="n">
         <v>1</v>
@@ -17059,17 +17059,17 @@
     <row r="694">
       <c r="A694" t="inlineStr">
         <is>
-          <t>But also [MASK] want to see inflation move up back to our 2 percent objective over the medium term, and so [MASK] above-trend growth and continuing tightness—greater tightness in labor and product markets—[MASK] think that [MASK] help [MASK] achieve our objective as [MASK] with respect to [MASK].</t>
+          <t>I don’t really think asset prices themselves [MASK] a significant threat to financial [MASK], and that’s because households [MASK] in good shape [MASK] than they have been.</t>
         </is>
       </c>
       <c r="B694" t="n">
-        <v>2018</v>
+        <v>2013</v>
       </c>
       <c r="C694" t="n">
         <v>0</v>
       </c>
       <c r="D694" t="n">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="E694" t="n">
         <v>1</v>
@@ -17083,17 +17083,17 @@
     <row r="695">
       <c r="A695" t="inlineStr">
         <is>
-          <t>As a further [MASK] in enhancing the clarity of [MASK] communications, the Committee recently [MASK] to begin publishing information [MASK] participants’ assessments of appropriate monetary policy—that [MASK], the path of policy that each participant judges as most [MASK] to foster mandate-consistent outcomes for employment and inflation if [MASK] economy [MASK] as expected.</t>
+          <t>But also [MASK] want to see inflation move up back to our 2 percent objective over the medium term, and so [MASK] above-trend growth and continuing tightness—greater tightness in labor and product markets—[MASK] think that [MASK] help [MASK] achieve our objective as [MASK] with respect to [MASK].</t>
         </is>
       </c>
       <c r="B695" t="n">
         <v>2018</v>
       </c>
       <c r="C695" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D695" t="n">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="E695" t="n">
         <v>1</v>
@@ -17107,17 +17107,17 @@
     <row r="696">
       <c r="A696" t="inlineStr">
         <is>
-          <t>[MASK] we do say that risks to the financial system—we [MASK] in our longer-run statement [MASK] goals [MASK] monetary policy [MASK] that risks to the financial system that could prevent us from achieving [MASK] goals are something that we [MASK] take into consideration.</t>
+          <t>As a further [MASK] in enhancing the clarity of [MASK] communications, the Committee recently [MASK] to begin publishing information [MASK] participants’ assessments of appropriate monetary policy—that [MASK], the path of policy that each participant judges as most [MASK] to foster mandate-consistent outcomes for employment and inflation if [MASK] economy [MASK] as expected.</t>
         </is>
       </c>
       <c r="B696" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="C696" t="n">
         <v>2</v>
       </c>
       <c r="D696" t="n">
-        <v>209</v>
+        <v>62</v>
       </c>
       <c r="E696" t="n">
         <v>1</v>
@@ -17131,17 +17131,17 @@
     <row r="697">
       <c r="A697" t="inlineStr">
         <is>
-          <t>[MASK], while I do not shirk the responsibility of [MASK] Fed [MASK] to [MASK] what it can to meet its mandate, obviously, a broad range [MASK] policies can affect growth and [MASK], and I hope [MASK] there [MASK] be a range of actions that will complement and supplement the Federal Reserve’s efforts.</t>
+          <t>[MASK] we do say that risks to the financial system—we [MASK] in our longer-run statement [MASK] goals [MASK] monetary policy [MASK] that risks to the financial system that could prevent us from achieving [MASK] goals are something that we [MASK] take into consideration.</t>
         </is>
       </c>
       <c r="B697" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="C697" t="n">
         <v>2</v>
       </c>
       <c r="D697" t="n">
-        <v>4</v>
+        <v>209</v>
       </c>
       <c r="E697" t="n">
         <v>1</v>
@@ -17155,17 +17155,17 @@
     <row r="698">
       <c r="A698" t="inlineStr">
         <is>
-          <t>And inflation is well [MASK] target.</t>
+          <t>[MASK], while I do not shirk the responsibility of [MASK] Fed [MASK] to [MASK] what it can to meet its mandate, obviously, a broad range [MASK] policies can affect growth and [MASK], and I hope [MASK] there [MASK] be a range of actions that will complement and supplement the Federal Reserve’s efforts.</t>
         </is>
       </c>
       <c r="B698" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C698" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D698" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E698" t="n">
         <v>1</v>
@@ -17179,17 +17179,17 @@
     <row r="699">
       <c r="A699" t="inlineStr">
         <is>
-          <t>By contrast, raising rates too slowly would raise the risk that monetary policy would [MASK] to [MASK] abruptly down the road, which could jeopardize the [MASK] [MASK].</t>
+          <t>And inflation is well [MASK] target.</t>
         </is>
       </c>
       <c r="B699" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C699" t="n">
         <v>1</v>
       </c>
       <c r="D699" t="n">
-        <v>94</v>
+        <v>21</v>
       </c>
       <c r="E699" t="n">
         <v>1</v>
@@ -17203,17 +17203,17 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Inflation has moved up in [MASK] months, mainly reflecting higher [MASK] for some commodities [MASK] imported goods.</t>
+          <t>By contrast, raising rates too slowly would raise the risk that monetary policy would [MASK] to [MASK] abruptly down the road, which could jeopardize the [MASK] [MASK].</t>
         </is>
       </c>
       <c r="B700" t="n">
-        <v>2012</v>
+        <v>2022</v>
       </c>
       <c r="C700" t="n">
         <v>1</v>
       </c>
       <c r="D700" t="n">
-        <v>143</v>
+        <v>94</v>
       </c>
       <c r="E700" t="n">
         <v>1</v>
@@ -17227,17 +17227,17 @@
     <row r="701">
       <c r="A701" t="inlineStr">
         <is>
-          <t>Again, that’s not a forecast, [MASK]’ve made a hypothesis, which [MASK] imply [MASK] improvement in unemployment.</t>
+          <t>Inflation has moved up in [MASK] months, mainly reflecting higher [MASK] for some commodities [MASK] imported goods.</t>
         </is>
       </c>
       <c r="B701" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="C701" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D701" t="n">
-        <v>3</v>
+        <v>143</v>
       </c>
       <c r="E701" t="n">
         <v>1</v>
@@ -17251,17 +17251,17 @@
     <row r="702">
       <c r="A702" t="inlineStr">
         <is>
-          <t>So I think, through all [MASK] those channels, [MASK] policy works.</t>
+          <t>Again, that’s not a forecast, [MASK]’ve made a hypothesis, which [MASK] imply [MASK] improvement in unemployment.</t>
         </is>
       </c>
       <c r="B702" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C702" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D702" t="n">
-        <v>187</v>
+        <v>3</v>
       </c>
       <c r="E702" t="n">
         <v>1</v>
@@ -17275,17 +17275,17 @@
     <row r="703">
       <c r="A703" t="inlineStr">
         <is>
-          <t>But you do see [MASK] in services, so you—this [MASK] around the world [MASK] Chair Powell’s Press Conference FINAL weak manufacturing</t>
+          <t>So I think, through all [MASK] those channels, [MASK] policy works.</t>
         </is>
       </c>
       <c r="B703" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="C703" t="n">
         <v>2</v>
       </c>
       <c r="D703" t="n">
-        <v>88</v>
+        <v>187</v>
       </c>
       <c r="E703" t="n">
         <v>1</v>
@@ -17299,17 +17299,17 @@
     <row r="704">
       <c r="A704" t="inlineStr">
         <is>
-          <t>But many other commodity prices have fallen further, and the reason I [MASK] give for [MASK] [MASK] that the emerging markets—China, the [MASK] of Asia, [MASK] some [MASK] parts of the world—plus Europe, of course, are [MASK], and so global commodity demand is weaker.</t>
+          <t>But you do see [MASK] in services, so you—this [MASK] around the world [MASK] Chair Powell’s Press Conference FINAL weak manufacturing</t>
         </is>
       </c>
       <c r="B704" t="n">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="C704" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D704" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="E704" t="n">
         <v>1</v>
@@ -17323,17 +17323,17 @@
     <row r="705">
       <c r="A705" t="inlineStr">
         <is>
-          <t>Everyone, particularly people on fixed [MASK], [MASK] at the lower part of the income distribution are better off with [MASK] prices.</t>
+          <t>But many other commodity prices have fallen further, and the reason I [MASK] give for [MASK] [MASK] that the emerging markets—China, the [MASK] of Asia, [MASK] some [MASK] parts of the world—plus Europe, of course, are [MASK], and so global commodity demand is weaker.</t>
         </is>
       </c>
       <c r="B705" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C705" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D705" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E705" t="n">
         <v>1</v>
@@ -17347,17 +17347,17 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>The [MASK] of [MASK] into, into inflation over time is just not there.</t>
+          <t>Everyone, particularly people on fixed [MASK], [MASK] at the lower part of the income distribution are better off with [MASK] prices.</t>
         </is>
       </c>
       <c r="B706" t="n">
         <v>2021</v>
       </c>
       <c r="C706" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D706" t="n">
-        <v>249</v>
+        <v>100</v>
       </c>
       <c r="E706" t="n">
         <v>1</v>
@@ -17371,7 +17371,7 @@
     <row r="707">
       <c r="A707" t="inlineStr">
         <is>
-          <t>The housing sector [MASK] fully recovered from the downturn, supported in [MASK] by low [MASK] interest rates.</t>
+          <t>The [MASK] of [MASK] into, into inflation over time is just not there.</t>
         </is>
       </c>
       <c r="B707" t="n">
@@ -17381,7 +17381,7 @@
         <v>0</v>
       </c>
       <c r="D707" t="n">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E707" t="n">
         <v>1</v>
@@ -17395,7 +17395,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Now, we [MASK]—[MASK] know, we haven’t anticipated that slowdown in [MASK], and that’s one of the main reasons [MASK] we haven’t anticipated the relatively slow growth.</t>
+          <t>The housing sector [MASK] fully recovered from the downturn, supported in [MASK] by low [MASK] interest rates.</t>
         </is>
       </c>
       <c r="B708" t="n">
@@ -17405,7 +17405,7 @@
         <v>0</v>
       </c>
       <c r="D708" t="n">
-        <v>170</v>
+        <v>246</v>
       </c>
       <c r="E708" t="n">
         <v>1</v>
@@ -17419,17 +17419,17 @@
     <row r="709">
       <c r="A709" t="inlineStr">
         <is>
-          <t>And, you know, we do want [MASK] to run moderately above 2 [MASK].</t>
+          <t>Now, we [MASK]—[MASK] know, we haven’t anticipated that slowdown in [MASK], and that’s one of the main reasons [MASK] we haven’t anticipated the relatively slow growth.</t>
         </is>
       </c>
       <c r="B709" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="C709" t="n">
         <v>0</v>
       </c>
       <c r="D709" t="n">
-        <v>57</v>
+        <v>170</v>
       </c>
       <c r="E709" t="n">
         <v>1</v>
@@ -17443,17 +17443,17 @@
     <row r="710">
       <c r="A710" t="inlineStr">
         <is>
-          <t>And obviously [MASK] are benefits from a strong economy to every household in the economy, including savers, from having a better job [MASK] and [MASK] more [MASK] economy.</t>
+          <t>And, you know, we do want [MASK] to run moderately above 2 [MASK].</t>
         </is>
       </c>
       <c r="B710" t="n">
         <v>2011</v>
       </c>
       <c r="C710" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D710" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="E710" t="n">
         <v>1</v>
@@ -17467,17 +17467,17 @@
     <row r="711">
       <c r="A711" t="inlineStr">
         <is>
-          <t>I’m just saying, [MASK], that is what fiscal policy [MASK] do that, really, monetary [MASK] can’t [MASK]—is, is invest in [MASK] future productive capacity of the economy, raise potential growth.</t>
+          <t>And obviously [MASK] are benefits from a strong economy to every household in the economy, including savers, from having a better job [MASK] and [MASK] more [MASK] economy.</t>
         </is>
       </c>
       <c r="B711" t="n">
-        <v>2020</v>
+        <v>2011</v>
       </c>
       <c r="C711" t="n">
         <v>2</v>
       </c>
       <c r="D711" t="n">
-        <v>158</v>
+        <v>26</v>
       </c>
       <c r="E711" t="n">
         <v>1</v>
@@ -17491,17 +17491,17 @@
     <row r="712">
       <c r="A712" t="inlineStr">
         <is>
-          <t>Wage growth is not—there are many [MASK] that [MASK] it—it’[MASK] not definitive in any sense in determining our policy,</t>
+          <t>I’m just saying, [MASK], that is what fiscal policy [MASK] do that, really, monetary [MASK] can’t [MASK]—is, is invest in [MASK] future productive capacity of the economy, raise potential growth.</t>
         </is>
       </c>
       <c r="B712" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C712" t="n">
         <v>2</v>
       </c>
       <c r="D712" t="n">
-        <v>267</v>
+        <v>158</v>
       </c>
       <c r="E712" t="n">
         <v>1</v>
@@ -17515,17 +17515,17 @@
     <row r="713">
       <c r="A713" t="inlineStr">
         <is>
-          <t>We are quite aware that [MASK] low interest rates, particularly for a protracted period, [MASK] have costs for a lot [MASK] people.</t>
+          <t>Wage growth is not—there are many [MASK] that [MASK] it—it’[MASK] not definitive in any sense in determining our policy,</t>
         </is>
       </c>
       <c r="B713" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C713" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D713" t="n">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="E713" t="n">
         <v>1</v>
@@ -17539,17 +17539,17 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Well, we—[MASK] a [MASK], we do not desire inflation undershoots.</t>
+          <t>We are quite aware that [MASK] low interest rates, particularly for a protracted period, [MASK] have costs for a lot [MASK] people.</t>
         </is>
       </c>
       <c r="B714" t="n">
         <v>2020</v>
       </c>
       <c r="C714" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D714" t="n">
-        <v>294</v>
+        <v>273</v>
       </c>
       <c r="E714" t="n">
         <v>1</v>
@@ -17563,17 +17563,17 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>The Committee will continue to pay close [MASK] to the evolution [MASK] inflation and inflation expectations.</t>
+          <t>Well, we—[MASK] a [MASK], we do not desire inflation undershoots.</t>
         </is>
       </c>
       <c r="B715" t="n">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="C715" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D715" t="n">
-        <v>233</v>
+        <v>294</v>
       </c>
       <c r="E715" t="n">
         <v>1</v>
@@ -17587,17 +17587,17 @@
     <row r="716">
       <c r="A716" t="inlineStr">
         <is>
-          <t>But there’s also a role for monetary [MASK].</t>
+          <t>The Committee will continue to pay close [MASK] to the evolution [MASK] inflation and inflation expectations.</t>
         </is>
       </c>
       <c r="B716" t="n">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="C716" t="n">
         <v>2</v>
       </c>
       <c r="D716" t="n">
-        <v>85</v>
+        <v>233</v>
       </c>
       <c r="E716" t="n">
         <v>1</v>
@@ -17611,22 +17611,46 @@
     <row r="717">
       <c r="A717" t="inlineStr">
         <is>
+          <t>But there’s also a role for monetary [MASK].</t>
+        </is>
+      </c>
+      <c r="B717" t="n">
+        <v>2014</v>
+      </c>
+      <c r="C717" t="n">
+        <v>2</v>
+      </c>
+      <c r="D717" t="n">
+        <v>85</v>
+      </c>
+      <c r="E717" t="n">
+        <v>1</v>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>masking</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
           <t>And [MASK], what [MASK] statement emphasizes, and this is [MASK] same language we used in December and [MASK], we used the language [MASK] if inflation is running below our 2 percent objective.</t>
         </is>
       </c>
-      <c r="B717" t="n">
+      <c r="B718" t="n">
         <v>2017</v>
       </c>
-      <c r="C717" t="n">
-        <v>0</v>
-      </c>
-      <c r="D717" t="n">
+      <c r="C718" t="n">
+        <v>0</v>
+      </c>
+      <c r="D718" t="n">
         <v>40</v>
       </c>
-      <c r="E717" t="n">
-        <v>1</v>
-      </c>
-      <c r="F717" t="inlineStr">
+      <c r="E718" t="n">
+        <v>1</v>
+      </c>
+      <c r="F718" t="inlineStr">
         <is>
           <t>masking</t>
         </is>

</xml_diff>